<commit_message>
Revise annualized replacement cost accounts
</commit_message>
<xml_diff>
--- a/cost/Cost_Database.xlsx
+++ b/cost/Cost_Database.xlsx
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4617" uniqueCount="716">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4617" uniqueCount="717">
   <si>
     <t>Account</t>
   </si>
@@ -1305,10 +1305,10 @@
 Cost is scaled as a fraction of CAPEX unless specific parameters are added to indicate more/less frequent replacements (e.g. GCMR)</t>
   </si>
   <si>
-    <t>Annualized RPV Replacements</t>
-  </si>
-  <si>
-    <t>Annualized Core Barrel Replacements</t>
+    <t>Annualized Outer Vessel Structure Replacements</t>
+  </si>
+  <si>
+    <t>Annualized Inner Vessel Structure Replacements</t>
   </si>
   <si>
     <t>Annualized Moderator Replacements</t>
@@ -1317,10 +1317,10 @@
     <t>Annualized Reflector Replacements</t>
   </si>
   <si>
-    <t>Annualized Reactivity Control Replacements</t>
-  </si>
-  <si>
-    <t>Annualized Integrated Heat Transfer System Replacements</t>
+    <t>Annualized Reactor Control Devices Replacements</t>
+  </si>
+  <si>
+    <t>Annualized Main Heat Transport System Replacements</t>
   </si>
   <si>
     <t>Annualized Misc. Replacements</t>
@@ -2255,6 +2255,9 @@
   </si>
   <si>
     <t>Remotely Monitored</t>
+  </si>
+  <si>
+    <t>Annualized Moderator Booster Replacements</t>
   </si>
 </sst>
 </file>
@@ -19192,7 +19195,7 @@
       <c r="AF172" s="79"/>
       <c r="AG172" s="77"/>
     </row>
-    <row r="173" spans="1:33" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:33" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="37">
         <v>751</v>
       </c>
@@ -19205,7 +19208,7 @@
       </c>
       <c r="D173" s="39" t="str">
         <f t="shared" si="43"/>
-        <v xml:space="preserve">            Annualized RPV Replacements</v>
+        <v xml:space="preserve">            Annualized Outer Vessel Structure Replacements</v>
       </c>
       <c r="E173" s="39"/>
       <c r="F173" s="39"/>
@@ -19243,7 +19246,7 @@
       <c r="AF173" s="79"/>
       <c r="AG173" s="77"/>
     </row>
-    <row r="174" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:33" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="37">
         <v>752</v>
       </c>
@@ -19256,7 +19259,7 @@
       </c>
       <c r="D174" s="39" t="str">
         <f t="shared" si="43"/>
-        <v xml:space="preserve">            Annualized Core Barrel Replacements</v>
+        <v xml:space="preserve">            Annualized Inner Vessel Structure Replacements</v>
       </c>
       <c r="E174" s="39"/>
       <c r="F174" s="39"/>
@@ -19391,7 +19394,7 @@
       </c>
       <c r="D177" s="39" t="str">
         <f t="shared" si="43"/>
-        <v xml:space="preserve">            Annualized Reactivity Control Replacements</v>
+        <v xml:space="preserve">            Annualized Reactor Control Devices Replacements</v>
       </c>
       <c r="E177" s="39"/>
       <c r="F177" s="39"/>
@@ -19423,20 +19426,20 @@
       <c r="AF177" s="79"/>
       <c r="AG177" s="77"/>
     </row>
-    <row r="178" spans="1:33" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:33" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" s="37">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B178" s="38">
         <f t="shared" si="44"/>
         <v>2</v>
       </c>
       <c r="C178" s="56" t="s">
-        <v>405</v>
+        <v>716</v>
       </c>
       <c r="D178" s="39" t="str">
         <f t="shared" si="43"/>
-        <v xml:space="preserve">            Annualized Integrated Heat Transfer System Replacements</v>
+        <v xml:space="preserve">            Annualized Moderator Booster Replacements</v>
       </c>
       <c r="E178" s="39"/>
       <c r="F178" s="39"/>

</xml_diff>

<commit_message>
Break out annualized plant maintenance accounts
</commit_message>
<xml_diff>
--- a/cost/Cost_Database.xlsx
+++ b/cost/Cost_Database.xlsx
@@ -21,7 +21,7 @@
     <sheet name="Central Facility Database" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cost Database'!$A$1:$AB$184</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cost Database'!$A$1:$AB$192</definedName>
     <definedName name="CRF">#REF!</definedName>
     <definedName name="DiscountRate">#REF!</definedName>
     <definedName name="FacilityLifetime">#REF!</definedName>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4617" uniqueCount="717">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4625" uniqueCount="726">
   <si>
     <t>Account</t>
   </si>
@@ -2258,6 +2258,33 @@
   </si>
   <si>
     <t>Annualized Moderator Booster Replacements</t>
+  </si>
+  <si>
+    <t>Annualized Plant Maintenance (Misc.)</t>
+  </si>
+  <si>
+    <t>Annualized Building and Structural Maintenance (Accounts 212–215)</t>
+  </si>
+  <si>
+    <t>Annualized Main Heat Transport System Maintenance (Accounts 222.1–222.3 and 222.6)</t>
+  </si>
+  <si>
+    <t>Annualized Safety System Maintenance (Account 223)</t>
+  </si>
+  <si>
+    <t>Annualized Reactor Plant Equipment Maintenance (Accounts 221.11, 226, and 228)</t>
+  </si>
+  <si>
+    <t>Annualized Reactor I&amp;C Maintenance (Account 227)</t>
+  </si>
+  <si>
+    <t>Annualized Energy Conversion System Maintenance (Account 23)</t>
+  </si>
+  <si>
+    <t>Annualized Electrical Equipment Maintenance (Account 24)</t>
+  </si>
+  <si>
+    <t>Annualized Miscellaneous Equipment Maintenance (Account 26)</t>
   </si>
 </sst>
 </file>
@@ -5388,7 +5415,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AJ184"/>
+  <dimension ref="A1:AJ192"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.6640625" style="3" customWidth="1"/>
@@ -18572,7 +18599,7 @@
         <v>381</v>
       </c>
       <c r="D165" s="39" t="str">
-        <f t="shared" ref="D162:D181" si="43">REPT("   ", B165*2) &amp; C165</f>
+        <f t="shared" ref="D162:D189" si="43">REPT("   ", B165*2) &amp; C165</f>
         <v xml:space="preserve">            Operators </v>
       </c>
       <c r="E165" s="39" t="s">
@@ -19480,11 +19507,11 @@
         <v>2</v>
       </c>
       <c r="C179" s="56" t="s">
-        <v>406</v>
+        <v>717</v>
       </c>
       <c r="D179" s="39" t="str">
         <f t="shared" si="43"/>
-        <v xml:space="preserve">            Annualized Misc. Replacements</v>
+        <v xml:space="preserve">            Annualized Plant Maintenance (Misc.)</v>
       </c>
       <c r="E179" s="39"/>
       <c r="F179" s="39"/>
@@ -19516,27 +19543,20 @@
       <c r="AF179" s="79"/>
       <c r="AG179" s="77"/>
     </row>
-    <row r="180" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:33" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="37">
-        <v>78</v>
+        <v>759.1</v>
       </c>
       <c r="B180" s="38">
-        <f>IF(ISNUMBER(A180),
-    IF(AND(A180=INT(A180), MOD(A180, 10) = 0), 0,
-        IF(AND(A180=INT(A180), LEN(A180)=2), 1,
-            IF(AND(A180=INT(A180), LEN(A180)=3), 2,
-                LEN(A180) - FIND(".", A180) + 2)
-        )
-    ),
-"")</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(A180),IF(AND(A180=INT(A180),MOD(A180,10)=0),0,IF(AND(A180=INT(A180),LEN(A180)=2),1,IF(AND(A180=INT(A180),LEN(A180)=3),2,LEN(A180)-FIND(".",A180)+2))),"")</f>
+        <v>3</v>
       </c>
       <c r="C180" s="56" t="s">
-        <v>407</v>
+        <v>718</v>
       </c>
       <c r="D180" s="39" t="str">
-        <f t="shared" si="43"/>
-        <v xml:space="preserve">      Annualized Decommissioning Cost</v>
+        <f>REPT("   ",B180*2)&amp;C180</f>
+        <v>                  Annualized Building and Structural Maintenance (Accounts 212–215)</v>
       </c>
       <c r="E180" s="39"/>
       <c r="F180" s="39"/>
@@ -19544,20 +19564,18 @@
       <c r="H180" s="39"/>
       <c r="I180" s="39"/>
       <c r="J180" s="43"/>
-      <c r="K180" s="72"/>
+      <c r="K180" s="61"/>
       <c r="L180" s="49"/>
-      <c r="M180" s="45"/>
+      <c r="M180" s="59"/>
       <c r="N180" s="49"/>
       <c r="O180" s="49"/>
       <c r="P180" s="49"/>
       <c r="Q180" s="66"/>
-      <c r="R180" s="73"/>
-      <c r="S180" s="59"/>
-      <c r="T180" s="59"/>
+      <c r="R180" s="49"/>
+      <c r="S180" s="143"/>
+      <c r="T180" s="143"/>
       <c r="U180" s="49"/>
-      <c r="V180" s="59" t="s">
-        <v>408</v>
-      </c>
+      <c r="V180" s="143"/>
       <c r="W180" s="77"/>
       <c r="X180" s="80"/>
       <c r="Y180" s="80"/>
@@ -19570,46 +19588,39 @@
       <c r="AF180" s="79"/>
       <c r="AG180" s="77"/>
     </row>
-    <row r="181" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:33" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="37">
-        <v>80</v>
+        <v>759.2</v>
       </c>
       <c r="B181" s="38">
-        <f>IF(ISNUMBER(A181),
-IF(AND(A181=INT(A181), MOD(A181, 10) = 0), 0,
-IF(AND(A181=INT(A181), LEN(A181)=2), 1,
-IF(AND(A181=INT(A181), LEN(A181)=3), 2,
-LEN(A181) - FIND(".", A181) + 2)
-)
-),
-"")</f>
-        <v>0</v>
-      </c>
-      <c r="C181" s="71" t="s">
-        <v>409</v>
+        <f>IF(ISNUMBER(A181),IF(AND(A181=INT(A181),MOD(A181,10)=0),0,IF(AND(A181=INT(A181),LEN(A181)=2),1,IF(AND(A181=INT(A181),LEN(A181)=3),2,LEN(A181)-FIND(".",A181)+2))),"")</f>
+        <v>3</v>
+      </c>
+      <c r="C181" s="56" t="s">
+        <v>719</v>
       </c>
       <c r="D181" s="39" t="str">
-        <f t="shared" si="43"/>
-        <v>Annualized Fuel Cost</v>
+        <f>REPT("   ",B181*2)&amp;C181</f>
+        <v>                  Annualized Main Heat Transport System Maintenance (Accounts 222.1–222.3 and 222.6)</v>
       </c>
       <c r="E181" s="39"/>
       <c r="F181" s="39"/>
       <c r="G181" s="39"/>
       <c r="H181" s="39"/>
       <c r="I181" s="39"/>
-      <c r="J181" s="40"/>
-      <c r="K181" s="40"/>
-      <c r="L181" s="38"/>
-      <c r="M181" s="41"/>
-      <c r="N181" s="38"/>
-      <c r="O181" s="38"/>
-      <c r="P181" s="38"/>
-      <c r="Q181" s="40"/>
-      <c r="R181" s="38"/>
-      <c r="S181" s="41"/>
-      <c r="T181" s="38"/>
-      <c r="U181" s="38"/>
-      <c r="V181" s="38"/>
+      <c r="J181" s="43"/>
+      <c r="K181" s="61"/>
+      <c r="L181" s="49"/>
+      <c r="M181" s="59"/>
+      <c r="N181" s="49"/>
+      <c r="O181" s="49"/>
+      <c r="P181" s="49"/>
+      <c r="Q181" s="66"/>
+      <c r="R181" s="49"/>
+      <c r="S181" s="143"/>
+      <c r="T181" s="143"/>
+      <c r="U181" s="49"/>
+      <c r="V181" s="143"/>
       <c r="W181" s="77"/>
       <c r="X181" s="80"/>
       <c r="Y181" s="80"/>
@@ -19622,121 +19633,65 @@
       <c r="AF181" s="79"/>
       <c r="AG181" s="77"/>
     </row>
-    <row r="182" spans="1:33" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:33" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="37">
-        <v>81</v>
+        <v>759.3</v>
       </c>
       <c r="B182" s="38">
-        <f>IF(ISNUMBER(A182),
-IF(AND(A182=INT(A182), MOD(A182, 10) = 0), 0,
-IF(AND(A182=INT(A182), LEN(A182)=2), 1,
-IF(AND(A182=INT(A182), LEN(A182)=3), 2,
-LEN(A182) - FIND(".", A182) + 2)
-)
-),
-"")</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(A182),IF(AND(A182=INT(A182),MOD(A182,10)=0),0,IF(AND(A182=INT(A182),LEN(A182)=2),1,IF(AND(A182=INT(A182),LEN(A182)=3),2,LEN(A182)-FIND(".",A182)+2))),"")</f>
+        <v>3</v>
       </c>
       <c r="C182" s="56" t="s">
-        <v>410</v>
+        <v>720</v>
       </c>
       <c r="D182" s="39" t="str">
-        <f t="shared" si="43"/>
-        <v xml:space="preserve">      Refueling Operations</v>
-      </c>
-      <c r="E182" s="39" t="s">
-        <v>264</v>
-      </c>
+        <f>REPT("   ",B182*2)&amp;C182</f>
+        <v>                  Annualized Safety System Maintenance (Account 223)</v>
+      </c>
+      <c r="E182" s="39"/>
       <c r="F182" s="39"/>
       <c r="G182" s="39"/>
       <c r="H182" s="39"/>
       <c r="I182" s="39"/>
       <c r="J182" s="43"/>
-      <c r="K182" s="61">
-        <v>178500</v>
-      </c>
-      <c r="L182" s="49" t="s">
-        <v>382</v>
-      </c>
-      <c r="M182" s="59" t="s">
-        <v>383</v>
-      </c>
+      <c r="K182" s="61"/>
+      <c r="L182" s="49"/>
+      <c r="M182" s="59"/>
       <c r="N182" s="49"/>
       <c r="O182" s="49"/>
-      <c r="P182" s="49">
-        <v>1</v>
-      </c>
-      <c r="Q182" s="66">
-        <v>2024</v>
-      </c>
-      <c r="R182" s="73" t="s">
-        <v>53</v>
-      </c>
-      <c r="S182" s="59"/>
-      <c r="T182" s="59" t="s">
-        <v>384</v>
-      </c>
+      <c r="P182" s="49"/>
+      <c r="Q182" s="66"/>
+      <c r="R182" s="49"/>
+      <c r="S182" s="143"/>
+      <c r="T182" s="143"/>
       <c r="U182" s="49"/>
-      <c r="V182" s="49"/>
-      <c r="W182" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="X182" s="80">
-        <f>0.9*$J182</f>
-        <v>0</v>
-      </c>
-      <c r="Y182" s="80">
-        <f>1.5*J182</f>
-        <v>0</v>
-      </c>
-      <c r="Z182" s="77" t="s">
-        <v>44</v>
-      </c>
-      <c r="AA182" s="79">
-        <f>0.9*K182</f>
-        <v>160650</v>
-      </c>
-      <c r="AB182" s="79">
-        <f>1.3*K182</f>
-        <v>232050</v>
-      </c>
-      <c r="AC182" s="77" t="s">
-        <v>44</v>
-      </c>
-      <c r="AD182" s="79" t="s">
-        <v>45</v>
-      </c>
-      <c r="AE182" s="79" t="s">
-        <v>46</v>
-      </c>
-      <c r="AF182" s="79" t="s">
-        <v>47</v>
-      </c>
-      <c r="AG182" s="77" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="183" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V182" s="143"/>
+      <c r="W182" s="77"/>
+      <c r="X182" s="80"/>
+      <c r="Y182" s="80"/>
+      <c r="Z182" s="77"/>
+      <c r="AA182" s="79"/>
+      <c r="AB182" s="79"/>
+      <c r="AC182" s="77"/>
+      <c r="AD182" s="79"/>
+      <c r="AE182" s="79"/>
+      <c r="AF182" s="79"/>
+      <c r="AG182" s="77"/>
+    </row>
+    <row r="183" spans="1:33" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" s="37">
-        <v>82</v>
+        <v>759.4</v>
       </c>
       <c r="B183" s="38">
-        <f>IF(ISNUMBER(A183),
-IF(AND(A183=INT(A183), MOD(A183, 10) = 0), 0,
-IF(AND(A183=INT(A183), LEN(A183)=2), 1,
-IF(AND(A183=INT(A183), LEN(A183)=3), 2,
-LEN(A183) - FIND(".", A183) + 2)
-)
-),
-"")</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(A183),IF(AND(A183=INT(A183),MOD(A183,10)=0),0,IF(AND(A183=INT(A183),LEN(A183)=2),1,IF(AND(A183=INT(A183),LEN(A183)=3),2,LEN(A183)-FIND(".",A183)+2))),"")</f>
+        <v>3</v>
       </c>
       <c r="C183" s="56" t="s">
-        <v>411</v>
+        <v>721</v>
       </c>
       <c r="D183" s="39" t="str">
-        <f t="shared" si="43"/>
-        <v xml:space="preserve">      Additional Nuclear Fuel</v>
+        <f>REPT("   ",B183*2)&amp;C183</f>
+        <v>                  Annualized Reactor Plant Equipment Maintenance (Accounts 221.11, 226, and 228)</v>
       </c>
       <c r="E183" s="39"/>
       <c r="F183" s="39"/>
@@ -19752,10 +19707,10 @@
       <c r="P183" s="49"/>
       <c r="Q183" s="66"/>
       <c r="R183" s="49"/>
-      <c r="S183" s="59"/>
-      <c r="T183" s="49"/>
+      <c r="S183" s="143"/>
+      <c r="T183" s="143"/>
       <c r="U183" s="49"/>
-      <c r="V183" s="49"/>
+      <c r="V183" s="143"/>
       <c r="W183" s="77"/>
       <c r="X183" s="80"/>
       <c r="Y183" s="80"/>
@@ -19768,105 +19723,537 @@
       <c r="AF183" s="79"/>
       <c r="AG183" s="77"/>
     </row>
-    <row r="184" spans="1:33" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:33" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" s="37">
-        <v>83</v>
+        <v>759.5</v>
       </c>
       <c r="B184" s="38">
-        <f>IF(ISNUMBER(A184),
-IF(AND(A184=INT(A184), MOD(A184, 10) = 0), 0,
-IF(AND(A184=INT(A184), LEN(A184)=2), 1,
-IF(AND(A184=INT(A184), LEN(A184)=3), 2,
-LEN(A184) - FIND(".", A184) + 2)
-)
-),
-"")</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(A184),IF(AND(A184=INT(A184),MOD(A184,10)=0),0,IF(AND(A184=INT(A184),LEN(A184)=2),1,IF(AND(A184=INT(A184),LEN(A184)=3),2,LEN(A184)-FIND(".",A184)+2))),"")</f>
+        <v>3</v>
       </c>
       <c r="C184" s="56" t="s">
-        <v>412</v>
+        <v>722</v>
       </c>
       <c r="D184" s="39" t="str">
-        <f t="shared" si="43"/>
-        <v xml:space="preserve">      Spent Fuel Management</v>
-      </c>
-      <c r="E184" s="39" t="s">
-        <v>35</v>
-      </c>
+        <f>REPT("   ",B184*2)&amp;C184</f>
+        <v>                  Annualized Reactor I&amp;C Maintenance (Account 227)</v>
+      </c>
+      <c r="E184" s="39"/>
       <c r="F184" s="39"/>
       <c r="G184" s="39"/>
       <c r="H184" s="39"/>
       <c r="I184" s="39"/>
       <c r="J184" s="43"/>
-      <c r="K184" s="61">
-        <v>1</v>
-      </c>
-      <c r="L184" s="49" t="s">
-        <v>413</v>
-      </c>
-      <c r="M184" s="59" t="s">
-        <v>414</v>
-      </c>
+      <c r="K184" s="61"/>
+      <c r="L184" s="49"/>
+      <c r="M184" s="59"/>
       <c r="N184" s="49"/>
       <c r="O184" s="49"/>
-      <c r="P184" s="49">
+      <c r="P184" s="49"/>
+      <c r="Q184" s="66"/>
+      <c r="R184" s="49"/>
+      <c r="S184" s="143"/>
+      <c r="T184" s="143"/>
+      <c r="U184" s="49"/>
+      <c r="V184" s="143"/>
+      <c r="W184" s="77"/>
+      <c r="X184" s="80"/>
+      <c r="Y184" s="80"/>
+      <c r="Z184" s="77"/>
+      <c r="AA184" s="79"/>
+      <c r="AB184" s="79"/>
+      <c r="AC184" s="77"/>
+      <c r="AD184" s="79"/>
+      <c r="AE184" s="79"/>
+      <c r="AF184" s="79"/>
+      <c r="AG184" s="77"/>
+    </row>
+    <row r="185" spans="1:33" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A185" s="37">
+        <v>759.6</v>
+      </c>
+      <c r="B185" s="38">
+        <f>IF(ISNUMBER(A185),IF(AND(A185=INT(A185),MOD(A185,10)=0),0,IF(AND(A185=INT(A185),LEN(A185)=2),1,IF(AND(A185=INT(A185),LEN(A185)=3),2,LEN(A185)-FIND(".",A185)+2))),"")</f>
+        <v>3</v>
+      </c>
+      <c r="C185" s="56" t="s">
+        <v>723</v>
+      </c>
+      <c r="D185" s="39" t="str">
+        <f>REPT("   ",B185*2)&amp;C185</f>
+        <v>                  Annualized Energy Conversion System Maintenance (Account 23)</v>
+      </c>
+      <c r="E185" s="39"/>
+      <c r="F185" s="39"/>
+      <c r="G185" s="39"/>
+      <c r="H185" s="39"/>
+      <c r="I185" s="39"/>
+      <c r="J185" s="43"/>
+      <c r="K185" s="61"/>
+      <c r="L185" s="49"/>
+      <c r="M185" s="59"/>
+      <c r="N185" s="49"/>
+      <c r="O185" s="49"/>
+      <c r="P185" s="49"/>
+      <c r="Q185" s="66"/>
+      <c r="R185" s="49"/>
+      <c r="S185" s="143"/>
+      <c r="T185" s="143"/>
+      <c r="U185" s="49"/>
+      <c r="V185" s="143"/>
+      <c r="W185" s="77"/>
+      <c r="X185" s="80"/>
+      <c r="Y185" s="80"/>
+      <c r="Z185" s="77"/>
+      <c r="AA185" s="79"/>
+      <c r="AB185" s="79"/>
+      <c r="AC185" s="77"/>
+      <c r="AD185" s="79"/>
+      <c r="AE185" s="79"/>
+      <c r="AF185" s="79"/>
+      <c r="AG185" s="77"/>
+    </row>
+    <row r="186" spans="1:33" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A186" s="37">
+        <v>759.7</v>
+      </c>
+      <c r="B186" s="38">
+        <f>IF(ISNUMBER(A186),IF(AND(A186=INT(A186),MOD(A186,10)=0),0,IF(AND(A186=INT(A186),LEN(A186)=2),1,IF(AND(A186=INT(A186),LEN(A186)=3),2,LEN(A186)-FIND(".",A186)+2))),"")</f>
+        <v>3</v>
+      </c>
+      <c r="C186" s="56" t="s">
+        <v>724</v>
+      </c>
+      <c r="D186" s="39" t="str">
+        <f>REPT("   ",B186*2)&amp;C186</f>
+        <v>                  Annualized Electrical Equipment Maintenance (Account 24)</v>
+      </c>
+      <c r="E186" s="39"/>
+      <c r="F186" s="39"/>
+      <c r="G186" s="39"/>
+      <c r="H186" s="39"/>
+      <c r="I186" s="39"/>
+      <c r="J186" s="43"/>
+      <c r="K186" s="61"/>
+      <c r="L186" s="49"/>
+      <c r="M186" s="59"/>
+      <c r="N186" s="49"/>
+      <c r="O186" s="49"/>
+      <c r="P186" s="49"/>
+      <c r="Q186" s="66"/>
+      <c r="R186" s="49"/>
+      <c r="S186" s="143"/>
+      <c r="T186" s="143"/>
+      <c r="U186" s="49"/>
+      <c r="V186" s="143"/>
+      <c r="W186" s="77"/>
+      <c r="X186" s="80"/>
+      <c r="Y186" s="80"/>
+      <c r="Z186" s="77"/>
+      <c r="AA186" s="79"/>
+      <c r="AB186" s="79"/>
+      <c r="AC186" s="77"/>
+      <c r="AD186" s="79"/>
+      <c r="AE186" s="79"/>
+      <c r="AF186" s="79"/>
+      <c r="AG186" s="77"/>
+    </row>
+    <row r="187" spans="1:33" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A187" s="37">
+        <v>759.8</v>
+      </c>
+      <c r="B187" s="38">
+        <f>IF(ISNUMBER(A187),IF(AND(A187=INT(A187),MOD(A187,10)=0),0,IF(AND(A187=INT(A187),LEN(A187)=2),1,IF(AND(A187=INT(A187),LEN(A187)=3),2,LEN(A187)-FIND(".",A187)+2))),"")</f>
+        <v>3</v>
+      </c>
+      <c r="C187" s="56" t="s">
+        <v>725</v>
+      </c>
+      <c r="D187" s="39" t="str">
+        <f>REPT("   ",B187*2)&amp;C187</f>
+        <v>                  Annualized Miscellaneous Equipment Maintenance (Account 26)</v>
+      </c>
+      <c r="E187" s="39"/>
+      <c r="F187" s="39"/>
+      <c r="G187" s="39"/>
+      <c r="H187" s="39"/>
+      <c r="I187" s="39"/>
+      <c r="J187" s="43"/>
+      <c r="K187" s="61"/>
+      <c r="L187" s="49"/>
+      <c r="M187" s="59"/>
+      <c r="N187" s="49"/>
+      <c r="O187" s="49"/>
+      <c r="P187" s="49"/>
+      <c r="Q187" s="66"/>
+      <c r="R187" s="49"/>
+      <c r="S187" s="143"/>
+      <c r="T187" s="143"/>
+      <c r="U187" s="49"/>
+      <c r="V187" s="143"/>
+      <c r="W187" s="77"/>
+      <c r="X187" s="80"/>
+      <c r="Y187" s="80"/>
+      <c r="Z187" s="77"/>
+      <c r="AA187" s="79"/>
+      <c r="AB187" s="79"/>
+      <c r="AC187" s="77"/>
+      <c r="AD187" s="79"/>
+      <c r="AE187" s="79"/>
+      <c r="AF187" s="79"/>
+      <c r="AG187" s="77"/>
+    </row>
+    <row r="188" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A188" s="37">
+        <v>78</v>
+      </c>
+      <c r="B188" s="38">
+        <f>IF(ISNUMBER(A188),
+    IF(AND(A188=INT(A188), MOD(A188, 10) = 0), 0,
+        IF(AND(A188=INT(A188), LEN(A188)=2), 1,
+            IF(AND(A188=INT(A188), LEN(A188)=3), 2,
+                LEN(A188) - FIND(".", A188) + 2)
+        )
+    ),
+"")</f>
         <v>1</v>
       </c>
-      <c r="Q184" s="66">
+      <c r="C188" s="56" t="s">
+        <v>407</v>
+      </c>
+      <c r="D188" s="39" t="str">
+        <f t="shared" si="43"/>
+        <v xml:space="preserve">      Annualized Decommissioning Cost</v>
+      </c>
+      <c r="E188" s="39"/>
+      <c r="F188" s="39"/>
+      <c r="G188" s="39"/>
+      <c r="H188" s="39"/>
+      <c r="I188" s="39"/>
+      <c r="J188" s="43"/>
+      <c r="K188" s="72"/>
+      <c r="L188" s="49"/>
+      <c r="M188" s="45"/>
+      <c r="N188" s="49"/>
+      <c r="O188" s="49"/>
+      <c r="P188" s="49"/>
+      <c r="Q188" s="66"/>
+      <c r="R188" s="73"/>
+      <c r="S188" s="59"/>
+      <c r="T188" s="59"/>
+      <c r="U188" s="49"/>
+      <c r="V188" s="59" t="s">
+        <v>408</v>
+      </c>
+      <c r="W188" s="77"/>
+      <c r="X188" s="80"/>
+      <c r="Y188" s="80"/>
+      <c r="Z188" s="77"/>
+      <c r="AA188" s="79"/>
+      <c r="AB188" s="79"/>
+      <c r="AC188" s="77"/>
+      <c r="AD188" s="79"/>
+      <c r="AE188" s="79"/>
+      <c r="AF188" s="79"/>
+      <c r="AG188" s="77"/>
+    </row>
+    <row r="189" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A189" s="37">
+        <v>80</v>
+      </c>
+      <c r="B189" s="38">
+        <f>IF(ISNUMBER(A189),
+IF(AND(A189=INT(A189), MOD(A189, 10) = 0), 0,
+IF(AND(A189=INT(A189), LEN(A189)=2), 1,
+IF(AND(A189=INT(A189), LEN(A189)=3), 2,
+LEN(A189) - FIND(".", A189) + 2)
+)
+),
+"")</f>
+        <v>0</v>
+      </c>
+      <c r="C189" s="71" t="s">
+        <v>409</v>
+      </c>
+      <c r="D189" s="39" t="str">
+        <f t="shared" si="43"/>
+        <v>Annualized Fuel Cost</v>
+      </c>
+      <c r="E189" s="39"/>
+      <c r="F189" s="39"/>
+      <c r="G189" s="39"/>
+      <c r="H189" s="39"/>
+      <c r="I189" s="39"/>
+      <c r="J189" s="40"/>
+      <c r="K189" s="40"/>
+      <c r="L189" s="38"/>
+      <c r="M189" s="41"/>
+      <c r="N189" s="38"/>
+      <c r="O189" s="38"/>
+      <c r="P189" s="38"/>
+      <c r="Q189" s="40"/>
+      <c r="R189" s="38"/>
+      <c r="S189" s="41"/>
+      <c r="T189" s="38"/>
+      <c r="U189" s="38"/>
+      <c r="V189" s="38"/>
+      <c r="W189" s="77"/>
+      <c r="X189" s="80"/>
+      <c r="Y189" s="80"/>
+      <c r="Z189" s="77"/>
+      <c r="AA189" s="79"/>
+      <c r="AB189" s="79"/>
+      <c r="AC189" s="77"/>
+      <c r="AD189" s="79"/>
+      <c r="AE189" s="79"/>
+      <c r="AF189" s="79"/>
+      <c r="AG189" s="77"/>
+    </row>
+    <row r="190" spans="1:33" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A190" s="37">
+        <v>81</v>
+      </c>
+      <c r="B190" s="38">
+        <f>IF(ISNUMBER(A190),
+IF(AND(A190=INT(A190), MOD(A190, 10) = 0), 0,
+IF(AND(A190=INT(A190), LEN(A190)=2), 1,
+IF(AND(A190=INT(A190), LEN(A190)=3), 2,
+LEN(A190) - FIND(".", A190) + 2)
+)
+),
+"")</f>
+        <v>1</v>
+      </c>
+      <c r="C190" s="56" t="s">
+        <v>410</v>
+      </c>
+      <c r="D190" s="39" t="str">
+        <f t="shared" si="43"/>
+        <v xml:space="preserve">      Refueling Operations</v>
+      </c>
+      <c r="E190" s="39" t="s">
+        <v>264</v>
+      </c>
+      <c r="F190" s="39"/>
+      <c r="G190" s="39"/>
+      <c r="H190" s="39"/>
+      <c r="I190" s="39"/>
+      <c r="J190" s="43"/>
+      <c r="K190" s="61">
+        <v>178500</v>
+      </c>
+      <c r="L190" s="49" t="s">
+        <v>382</v>
+      </c>
+      <c r="M190" s="59" t="s">
+        <v>383</v>
+      </c>
+      <c r="N190" s="49"/>
+      <c r="O190" s="49"/>
+      <c r="P190" s="49">
+        <v>1</v>
+      </c>
+      <c r="Q190" s="66">
         <v>2024</v>
       </c>
-      <c r="R184" s="49" t="s">
+      <c r="R190" s="73" t="s">
+        <v>53</v>
+      </c>
+      <c r="S190" s="59"/>
+      <c r="T190" s="59" t="s">
+        <v>384</v>
+      </c>
+      <c r="U190" s="49"/>
+      <c r="V190" s="49"/>
+      <c r="W190" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="X190" s="80">
+        <f>0.9*$J190</f>
+        <v>0</v>
+      </c>
+      <c r="Y190" s="80">
+        <f>1.5*J190</f>
+        <v>0</v>
+      </c>
+      <c r="Z190" s="77" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA190" s="79">
+        <f>0.9*K190</f>
+        <v>160650</v>
+      </c>
+      <c r="AB190" s="79">
+        <f>1.3*K190</f>
+        <v>232050</v>
+      </c>
+      <c r="AC190" s="77" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD190" s="79" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE190" s="79" t="s">
+        <v>46</v>
+      </c>
+      <c r="AF190" s="79" t="s">
+        <v>47</v>
+      </c>
+      <c r="AG190" s="77" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="191" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A191" s="37">
+        <v>82</v>
+      </c>
+      <c r="B191" s="38">
+        <f>IF(ISNUMBER(A191),
+IF(AND(A191=INT(A191), MOD(A191, 10) = 0), 0,
+IF(AND(A191=INT(A191), LEN(A191)=2), 1,
+IF(AND(A191=INT(A191), LEN(A191)=3), 2,
+LEN(A191) - FIND(".", A191) + 2)
+)
+),
+"")</f>
+        <v>1</v>
+      </c>
+      <c r="C191" s="56" t="s">
+        <v>411</v>
+      </c>
+      <c r="D191" s="39" t="str">
+        <f t="shared" si="43"/>
+        <v xml:space="preserve">      Additional Nuclear Fuel</v>
+      </c>
+      <c r="E191" s="39"/>
+      <c r="F191" s="39"/>
+      <c r="G191" s="39"/>
+      <c r="H191" s="39"/>
+      <c r="I191" s="39"/>
+      <c r="J191" s="43"/>
+      <c r="K191" s="61"/>
+      <c r="L191" s="49"/>
+      <c r="M191" s="59"/>
+      <c r="N191" s="49"/>
+      <c r="O191" s="49"/>
+      <c r="P191" s="49"/>
+      <c r="Q191" s="66"/>
+      <c r="R191" s="49"/>
+      <c r="S191" s="59"/>
+      <c r="T191" s="49"/>
+      <c r="U191" s="49"/>
+      <c r="V191" s="49"/>
+      <c r="W191" s="77"/>
+      <c r="X191" s="80"/>
+      <c r="Y191" s="80"/>
+      <c r="Z191" s="77"/>
+      <c r="AA191" s="79"/>
+      <c r="AB191" s="79"/>
+      <c r="AC191" s="77"/>
+      <c r="AD191" s="79"/>
+      <c r="AE191" s="79"/>
+      <c r="AF191" s="79"/>
+      <c r="AG191" s="77"/>
+    </row>
+    <row r="192" spans="1:33" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A192" s="37">
+        <v>83</v>
+      </c>
+      <c r="B192" s="38">
+        <f>IF(ISNUMBER(A192),
+IF(AND(A192=INT(A192), MOD(A192, 10) = 0), 0,
+IF(AND(A192=INT(A192), LEN(A192)=2), 1,
+IF(AND(A192=INT(A192), LEN(A192)=3), 2,
+LEN(A192) - FIND(".", A192) + 2)
+)
+),
+"")</f>
+        <v>1</v>
+      </c>
+      <c r="C192" s="56" t="s">
+        <v>412</v>
+      </c>
+      <c r="D192" s="39" t="str">
+        <f t="shared" si="43"/>
+        <v xml:space="preserve">      Spent Fuel Management</v>
+      </c>
+      <c r="E192" s="39" t="s">
+        <v>35</v>
+      </c>
+      <c r="F192" s="39"/>
+      <c r="G192" s="39"/>
+      <c r="H192" s="39"/>
+      <c r="I192" s="39"/>
+      <c r="J192" s="43"/>
+      <c r="K192" s="61">
+        <v>1</v>
+      </c>
+      <c r="L192" s="49" t="s">
+        <v>413</v>
+      </c>
+      <c r="M192" s="59" t="s">
+        <v>414</v>
+      </c>
+      <c r="N192" s="49"/>
+      <c r="O192" s="49"/>
+      <c r="P192" s="49">
+        <v>1</v>
+      </c>
+      <c r="Q192" s="66">
+        <v>2024</v>
+      </c>
+      <c r="R192" s="49" t="s">
         <v>86</v>
       </c>
-      <c r="S184" s="59"/>
-      <c r="T184" s="49"/>
-      <c r="U184" s="49"/>
-      <c r="V184" s="49"/>
-      <c r="W184" s="77" t="s">
+      <c r="S192" s="59"/>
+      <c r="T192" s="49"/>
+      <c r="U192" s="49"/>
+      <c r="V192" s="49"/>
+      <c r="W192" s="77" t="s">
         <v>43</v>
       </c>
-      <c r="X184" s="80">
-        <f>0.9*$J184</f>
-        <v>0</v>
-      </c>
-      <c r="Y184" s="80">
-        <f>1.5*J184</f>
-        <v>0</v>
-      </c>
-      <c r="Z184" s="77" t="s">
-        <v>44</v>
-      </c>
-      <c r="AA184" s="79">
-        <f>0.9*K184</f>
+      <c r="X192" s="80">
+        <f>0.9*$J192</f>
+        <v>0</v>
+      </c>
+      <c r="Y192" s="80">
+        <f>1.5*J192</f>
+        <v>0</v>
+      </c>
+      <c r="Z192" s="77" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA192" s="79">
+        <f>0.9*K192</f>
         <v>0.9</v>
       </c>
-      <c r="AB184" s="79">
-        <f>1.3*K184</f>
+      <c r="AB192" s="79">
+        <f>1.3*K192</f>
         <v>1.3</v>
       </c>
-      <c r="AC184" s="77" t="s">
-        <v>44</v>
-      </c>
-      <c r="AD184" s="79" t="s">
+      <c r="AC192" s="77" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD192" s="79" t="s">
         <v>45</v>
       </c>
-      <c r="AE184" s="79" t="s">
+      <c r="AE192" s="79" t="s">
         <v>46</v>
       </c>
-      <c r="AF184" s="79" t="s">
+      <c r="AF192" s="79" t="s">
         <v>47</v>
       </c>
-      <c r="AG184" s="77" t="s">
+      <c r="AG192" s="77" t="s">
         <v>48</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB184" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:AB192" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="53">
     <mergeCell ref="T138:T143"/>
     <mergeCell ref="U30:U32"/>
     <mergeCell ref="S52:S54"/>
-    <mergeCell ref="T173:T179"/>
+    <mergeCell ref="T173:T187"/>
     <mergeCell ref="U15:U17"/>
     <mergeCell ref="U46:U48"/>
     <mergeCell ref="S145:S150"/>
@@ -19874,7 +20261,7 @@
     <mergeCell ref="S61:S63"/>
     <mergeCell ref="U61:U63"/>
     <mergeCell ref="U57:U59"/>
-    <mergeCell ref="S173:S179"/>
+    <mergeCell ref="S173:S187"/>
     <mergeCell ref="U76:U80"/>
     <mergeCell ref="S57:S59"/>
     <mergeCell ref="S37:S39"/>
@@ -19897,7 +20284,7 @@
     <mergeCell ref="T109:T110"/>
     <mergeCell ref="S138:S143"/>
     <mergeCell ref="T11:T13"/>
-    <mergeCell ref="V173:V179"/>
+    <mergeCell ref="V173:V187"/>
     <mergeCell ref="S30:S32"/>
     <mergeCell ref="S15:S17"/>
     <mergeCell ref="T37:T39"/>
@@ -19976,7 +20363,7 @@
       <formula>$B108=3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A74:V99 A107:V107 A173:R179">
+  <conditionalFormatting sqref="A74:V99 A107:V107 A173:R187">
     <cfRule type="expression" dxfId="286" priority="487">
       <formula>$B74=2</formula>
     </cfRule>
@@ -20031,18 +20418,18 @@
       <formula>$B152=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A181:V184">
+  <conditionalFormatting sqref="A189:V192">
     <cfRule type="expression" dxfId="273" priority="649">
-      <formula>$B181=3</formula>
+      <formula>$B189=3</formula>
     </cfRule>
     <cfRule type="expression" dxfId="272" priority="650">
-      <formula>$B181=2</formula>
+      <formula>$B189=2</formula>
     </cfRule>
     <cfRule type="expression" dxfId="271" priority="651">
-      <formula>$B181&lt;2</formula>
+      <formula>$B189&lt;2</formula>
     </cfRule>
     <cfRule type="expression" dxfId="270" priority="652">
-      <formula>$B181=0</formula>
+      <formula>$B189=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:AG4 A5:S6 U5:AG6 A109:F111 A112:V114 U116:V122 U123:U124 A127:S128 U127:V128 A138:B143 U138:V143 A144:V144 N145:V145 N146:R146 U146:V151 K147:R147 A151:T151 T155:V160 A161:V164 A165:J166 A167:L171 U169:V171">
@@ -20053,7 +20440,7 @@
       <formula>$B1=2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:AG4 A5:S6 U5:AG6 A7:AG51 A173:R179">
+  <conditionalFormatting sqref="A1:AG4 A5:S6 U5:AG6 A7:AG51 A173:R187">
     <cfRule type="expression" dxfId="267" priority="489">
       <formula>$B1=0</formula>
     </cfRule>
@@ -20069,12 +20456,12 @@
       <formula>$B7&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A49:AG51 F52:AG52 A52:E54 F53:U54 W53:AG54 A55:AG75 A76:V82 A83:AG87 A100:B106 A112:AG123 A124:U124 W124:AG124 A125:AG134 A135:V135 A136:Y136 A137:AG137 S173:AG173 U174:U179 W174:AG179 A180:AG184 A97:AG97">
+  <conditionalFormatting sqref="A49:AG51 F52:AG52 A52:E54 F53:U54 W53:AG54 A55:AG75 A76:V82 A83:AG87 A100:B106 A112:AG123 A124:U124 W124:AG124 A125:AG134 A135:V135 A136:Y136 A137:AG137 S173:AG173 U174:U187 W174:AG187 A188:AG192 A97:AG97">
     <cfRule type="expression" dxfId="263" priority="750">
       <formula>$B49=2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A49:AG51 F52:AG52 A52:E54 F53:U54 W53:AG54 A55:AG75 A76:V82 A83:AG87 A97:AG97 A100:B106 A112:AG123 A124:U124 W124:AG124 A125:AG134 A135:V135 A136:Y136 A137:AG137 S173:AG173 U174:U179 W174:AG179 A180:AG184">
+  <conditionalFormatting sqref="A49:AG51 F52:AG52 A52:E54 F53:U54 W53:AG54 A55:AG75 A76:V82 A83:AG87 A97:AG97 A100:B106 A112:AG123 A124:U124 W124:AG124 A125:AG134 A135:V135 A136:Y136 A137:AG137 S173:AG173 U174:U187 W174:AG187 A188:AG192">
     <cfRule type="expression" dxfId="262" priority="751">
       <formula>$B49&lt;2</formula>
     </cfRule>
@@ -20132,7 +20519,7 @@
       <formula>$B144=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A180:AG184 A55:AG75 A83:AG87 A125:AG134 A135:V135 A136:Y136 A137:AG137 A112:AG123 A76:V82 A100:B106 A49:AG51 F52:AG52 F53:U54 A52:E54 W53:AG54 A124:U124 W124:AG124 S173:AG173 U174:U179 W174:AG179">
+  <conditionalFormatting sqref="A188:AG192 A55:AG75 A83:AG87 A125:AG134 A135:V135 A136:Y136 A137:AG137 A112:AG123 A76:V82 A100:B106 A49:AG51 F52:AG52 F53:U54 A52:E54 W53:AG54 A124:U124 W124:AG124 S173:AG173 U174:U187 W174:AG187">
     <cfRule type="expression" dxfId="248" priority="749">
       <formula>$B49=3</formula>
     </cfRule>
@@ -20206,7 +20593,7 @@
       <formula>$B138=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D80 D82 D87:D137 D144:D184">
+  <conditionalFormatting sqref="D2:D80 D82 D87:D137 D144:D192">
     <cfRule type="colorScale" priority="1037">
       <colorScale>
         <cfvo type="min"/>
@@ -20398,7 +20785,7 @@
       <formula>$B106=3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F53:U54 W53:AG54 A55:AG75 A107:AG108 A109:V112 A112:AG123 A124:U124 W124:AG124 A125:AG134 A129:V144 S173:AG173 U174:U179 W174:AG179 A180:AG184">
+  <conditionalFormatting sqref="F53:U54 W53:AG54 A55:AG75 A107:AG108 A109:V112 A112:AG123 A124:U124 W124:AG124 A125:AG134 A129:V144 S173:AG173 U174:U187 W174:AG187 A188:AG192">
     <cfRule type="expression" dxfId="188" priority="752">
       <formula>$B53=0</formula>
     </cfRule>
@@ -21102,31 +21489,31 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="15">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q152 Q154:Q184 Q185:R192" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q152 Q154:Q192 Q185:R192" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>1950</formula1>
       <formula2>2025</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J130 J133:J134 J137:J144 J148:J184 K2:K9 K11:K48 K52:K54 K57:K59 K61:K63 K67:K79 K87 K97:K107 K109:K150 K152:K184 N1:N67 N71:N83 N88:N106 N105:N1048576" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J130 J133:J134 J137:J144 J148:J192 K2:K9 K11:K48 K52:K54 K57:K59 K61:K63 K67:K79 K87 K97:K107 K109:K150 K152:K192 N1:N67 N71:N83 N88:N106 N105:N1048576" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M359:M369" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Land Area, Power MWe, Excavation Volume,  Reactor Building Slab Roof Volume,	Reactor Building  Basement Volume, Reactor Building  Exterior Walls Volume,		Turbine Building Slab Roof Volume,	Turbine Building  Basement Volume,	Turbine Building  Exterior Wall"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1 L182:L1048576" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1 L190:L1048576" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"$/acres, $/MWe, $/m^3, $/MWt"</formula1>
     </dataValidation>
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P185:P338" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>0</formula1>
       <formula2>2</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P80 P82:P137 P144:P184" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P80 P82:P137 P144:P192" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>0</formula1>
       <formula2>2</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O80 O82:O134 O137 O144:O184" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O80 O82:O134 O137 O144:O192" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"acres, MWe, m^3, MWt, Kg, Drums, kW, $, m^2, kg/s"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L80 L82:L113 L115:L137 L144:L184" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L80 L82:L113 L115:L137 L144:L192" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"$/m^2,$/MWeHour,$/FTE, $/acres, $/MWe, $/m^3, $/MWt, $/Kg, $/Drum, $/(kg.sec), $/SWU, unitless, $/kWe"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O135:O136" xr:uid="{00000000-0002-0000-0000-000008000000}">
@@ -21142,10 +21529,10 @@
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E184" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E192" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"standard, nonstandard"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R2:R184" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R2:R192" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"NA, General, Labor, Material, Equipment,Lab and Mat and Equip, 'Lab and Equip"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L114" xr:uid="{00000000-0002-0000-0000-00000E000000}">

</xml_diff>

<commit_message>
Clarify on-site operator parameter
</commit_message>
<xml_diff>
--- a/cost/Cost_Database.xlsx
+++ b/cost/Cost_Database.xlsx
@@ -1876,7 +1876,7 @@
     <t>$/FTE</t>
   </si>
   <si>
-    <t>Number of Operators</t>
+    <t>Number of On-Site Operators per Shift</t>
   </si>
   <si>
     <t>de Candido, I., A. Al Rashdan, A. Abou-Jaoude, and J. Buongiorno. 2024. “Assessment of Technoeconomic Opportunities in Automation for Nuclear Microreactors.” Nuclear Science and Engineering, 1–20. https://doi.org/10.1080/00295639.2024.2372511.</t>
@@ -2694,7 +2694,7 @@
     <t>Operators (Testing Only)</t>
   </si>
   <si>
-    <t>MFG Testing Number of Operators</t>
+    <t>MFG Testing Number of On-Site Operators per Shift</t>
   </si>
   <si>
     <t>Warehouse Staff</t>
@@ -3015,7 +3015,7 @@
     <t>Shift To Headcount</t>
   </si>
   <si>
-    <t>SER Number of Operators Per Shift</t>
+    <t>SER Number of On-Site Operators per Shift Per Shift</t>
   </si>
   <si>
     <t>SER Security Staff Per Shift</t>

</xml_diff>

<commit_message>
Fix manufacturing operator parameter lookup
</commit_message>
<xml_diff>
--- a/cost/Cost_Database.xlsx
+++ b/cost/Cost_Database.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Database" sheetId="1" r:id="Rd09f38df92c548d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MARVEL_Cost" sheetId="2" r:id="R6ecdd67b153c4627"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Variables" sheetId="3" r:id="Rb5533a590ac94c81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inflation Adjustment" sheetId="4" r:id="Re92964ed09ba40fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economics Parameters" sheetId="5" r:id="R97da12fc1c7a4202"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturing Campus Database" sheetId="7" r:id="Rda28546308ae4396"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servicing Campus Database" sheetId="8" r:id="R8147a9e33a154705"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Database" sheetId="1" r:id="Raee221fb551f4d08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MARVEL_Cost" sheetId="2" r:id="Ra299e229cc5c4b48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Variables" sheetId="3" r:id="R1136f3a8c77840bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inflation Adjustment" sheetId="4" r:id="R0212ed239f5e42b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economics Parameters" sheetId="5" r:id="R6434e323901e4bda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturing Campus Database" sheetId="7" r:id="R9ee7b8ca55e84603"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servicing Campus Database" sheetId="8" r:id="Rb07cc31647744dd1"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="CRF">#REF!</x:definedName>
@@ -2898,9 +2898,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Operators (Testing Only)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">MFG Testing Number of On-Site Operators per Shift</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Warehouse Staff</x:t>
@@ -23915,19 +23912,19 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="Rb6a757536a1e48b8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U5" r:id="Rb22de9407a7a4819"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="Raab305e837174012"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="Rb61430fcc4a24a97"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U33" r:id="Rb92345b2f55d443a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U49" r:id="Rc169c2b43ada43e9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U109" r:id="Re832671e46cd41d8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U120" r:id="Rc193e8d6960548f2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U130" r:id="Rd271ce1e6d804b70"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U131" r:id="Rbf16ca840e6b4b6c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U135" r:id="Redb2433ebaf34e6b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U136" r:id="R06ceb00dfb4546b6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U169" r:id="R1ce9ec4ce48942c6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="Rbd0c5c3805ef4e05"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U5" r:id="Rc7e9d4e2578d49ef"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="R34b91720f5c04dba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="R385e030e8c444c8f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U33" r:id="R8c6725ede10446b6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U49" r:id="Re933932b96c44a93"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U109" r:id="R638f7fcf1223489d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U120" r:id="R33d13cad100f41f0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U130" r:id="R105ba6ec51324274"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U131" r:id="R9bfe1e2cd16644b2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U135" r:id="R3e4024a1c8064ba8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U136" r:id="R63a66a6acd284df3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U169" r:id="R46a3c2895cc349e7"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -26772,8 +26769,8 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3074a36633e4412a"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e6e4ec42ff14067"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bf8797f5b7e46bc"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb11a00de6a8420b"/>
 </x:worksheet>
 </file>
 
@@ -30629,8 +30626,8 @@
       <x:c r="L48" s="103" t="s">
         <x:v>386</x:v>
       </x:c>
-      <x:c r="M48" s="110" t="s">
-        <x:v>672</x:v>
+      <x:c r="M48" s="110" t="str">
+        <x:v>MFG Testing Number of Operators</x:v>
       </x:c>
       <x:c r="N48" s="103"/>
       <x:c r="O48" s="103"/>
@@ -30696,7 +30693,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C49" s="109" t="s">
-        <x:v>673</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="D49" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -30717,7 +30714,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M49" s="58" t="s">
-        <x:v>674</x:v>
+        <x:v>673</x:v>
       </x:c>
       <x:c r="N49" s="103"/>
       <x:c r="O49" s="103"/>
@@ -30731,10 +30728,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="S49" s="58" t="s">
+        <x:v>674</x:v>
+      </x:c>
+      <x:c r="T49" s="58" t="s">
         <x:v>675</x:v>
-      </x:c>
-      <x:c r="T49" s="58" t="s">
-        <x:v>676</x:v>
       </x:c>
       <x:c r="U49" s="103"/>
       <x:c r="V49" s="103"/>
@@ -30806,7 +30803,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M50" s="58" t="s">
-        <x:v>677</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="N50" s="103"/>
       <x:c r="O50" s="103"/>
@@ -30872,7 +30869,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C51" s="109" t="s">
-        <x:v>678</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="D51" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -30893,7 +30890,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M51" s="58" t="s">
-        <x:v>679</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="N51" s="103"/>
       <x:c r="O51" s="103"/>
@@ -30959,7 +30956,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C52" s="109" t="s">
-        <x:v>680</x:v>
+        <x:v>679</x:v>
       </x:c>
       <x:c r="D52" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -30980,7 +30977,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M52" s="183" t="s">
-        <x:v>681</x:v>
+        <x:v>680</x:v>
       </x:c>
       <x:c r="N52" s="103"/>
       <x:c r="O52" s="103"/>
@@ -31042,7 +31039,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C53" s="109" t="s">
-        <x:v>682</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="D53" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -31115,7 +31112,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C54" s="109" t="s">
-        <x:v>683</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="D54" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -31188,7 +31185,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C55" s="109" t="s">
-        <x:v>684</x:v>
+        <x:v>683</x:v>
       </x:c>
       <x:c r="D55" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -31277,7 +31274,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C56" s="109" t="s">
-        <x:v>685</x:v>
+        <x:v>684</x:v>
       </x:c>
       <x:c r="D56" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -31366,7 +31363,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C57" s="109" t="s">
-        <x:v>686</x:v>
+        <x:v>685</x:v>
       </x:c>
       <x:c r="D57" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -31411,7 +31408,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C58" s="109" t="s">
-        <x:v>687</x:v>
+        <x:v>686</x:v>
       </x:c>
       <x:c r="D58" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -31482,7 +31479,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C59" s="109" t="s">
-        <x:v>688</x:v>
+        <x:v>687</x:v>
       </x:c>
       <x:c r="D59" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -31553,7 +31550,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C60" s="109" t="s">
-        <x:v>689</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="D60" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -31624,7 +31621,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C61" s="109" t="s">
-        <x:v>690</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="D61" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -31713,7 +31710,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C62" s="109" t="s">
-        <x:v>691</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="D62" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -31802,7 +31799,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C63" s="109" t="s">
-        <x:v>692</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="D63" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -31891,7 +31888,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C64" s="109" t="s">
-        <x:v>693</x:v>
+        <x:v>692</x:v>
       </x:c>
       <x:c r="D64" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -31962,7 +31959,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C65" s="109" t="s">
-        <x:v>694</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="D65" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -32031,7 +32028,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C66" s="109" t="s">
-        <x:v>695</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="D66" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -32056,7 +32053,7 @@
         <x:v>186</x:v>
       </x:c>
       <x:c r="M66" s="183" t="s">
-        <x:v>696</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="N66" s="103"/>
       <x:c r="O66" s="103" t="s">
@@ -32126,7 +32123,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C67" s="109" t="s">
-        <x:v>697</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="D67" s="93" t="str">
         <x:f t="shared" si="25"/>
@@ -32533,13 +32530,13 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R728af51f0c224e1d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U27" r:id="R321f3d02a8984c75"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U66" r:id="R7671ba8ce6054bb2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R41634fb1c3ba42d4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U27" r:id="Rb9ef6038711449fe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U66" r:id="Re89ec1ce24494120"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8672e896a47a4873"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3962e203a664540"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47ea54c41ff7458f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec0e2daf42104d54"/>
 </x:worksheet>
 </file>
 
@@ -32771,7 +32768,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="M3" s="100" t="s">
-        <x:v>698</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="N3" s="121"/>
       <x:c r="O3" s="100" t="s">
@@ -32867,7 +32864,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="M4" s="100" t="s">
-        <x:v>699</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="N4" s="121"/>
       <x:c r="O4" s="100" t="s">
@@ -33370,7 +33367,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="M11" s="100" t="s">
-        <x:v>700</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="N11" s="121"/>
       <x:c r="O11" s="100" t="s">
@@ -33473,7 +33470,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="M12" s="100" t="s">
-        <x:v>700</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="N12" s="121"/>
       <x:c r="O12" s="100" t="s">
@@ -33563,7 +33560,7 @@
         <x:v>614</x:v>
       </x:c>
       <x:c r="M13" s="125" t="s">
-        <x:v>701</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="N13" s="126">
         <x:v>1</x:v>
@@ -33702,7 +33699,7 @@
         <x:v>619</x:v>
       </x:c>
       <x:c r="M15" s="100" t="s">
-        <x:v>702</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="N15" s="121"/>
       <x:c r="O15" s="100"/>
@@ -33766,7 +33763,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C16" s="98" t="s">
-        <x:v>703</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="D16" s="93" t="str">
         <x:f t="shared" si="1"/>
@@ -33792,7 +33789,7 @@
         <x:v>619</x:v>
       </x:c>
       <x:c r="M16" s="100" t="s">
-        <x:v>704</x:v>
+        <x:v>703</x:v>
       </x:c>
       <x:c r="N16" s="121"/>
       <x:c r="O16" s="100"/>
@@ -33882,7 +33879,7 @@
         <x:v>619</x:v>
       </x:c>
       <x:c r="M17" s="100" t="s">
-        <x:v>705</x:v>
+        <x:v>704</x:v>
       </x:c>
       <x:c r="N17" s="121"/>
       <x:c r="O17" s="100"/>
@@ -33991,7 +33988,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C19" s="98" t="s">
-        <x:v>706</x:v>
+        <x:v>705</x:v>
       </x:c>
       <x:c r="D19" s="93" t="str">
         <x:f t="shared" si="1"/>
@@ -34036,7 +34033,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C20" s="150" t="s">
-        <x:v>707</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="D20" s="151" t="str">
         <x:f t="shared" si="1"/>
@@ -34062,7 +34059,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M20" s="155" t="s">
-        <x:v>708</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="N20" s="142" t="n">
         <x:f>338988/(3.2808^2)</x:f>
@@ -34081,7 +34078,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S20" s="144" t="s">
-        <x:v>709</x:v>
+        <x:v>708</x:v>
       </x:c>
       <x:c r="T20" s="170"/>
       <x:c r="U20" s="171"/>
@@ -34133,7 +34130,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C21" s="98" t="s">
-        <x:v>710</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="D21" s="93"/>
       <x:c r="E21" s="93"/>
@@ -34175,7 +34172,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C22" s="150" t="s">
-        <x:v>711</x:v>
+        <x:v>710</x:v>
       </x:c>
       <x:c r="D22" s="151" t="str">
         <x:f t="shared" ref="D22" si="13">REPT("   ", B22*2) &amp; C22</x:f>
@@ -34201,7 +34198,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M22" s="155" t="s">
-        <x:v>712</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="N22" s="142">
         <x:v>1</x:v>
@@ -34219,7 +34216,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S22" s="144" t="s">
-        <x:v>713</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="T22" s="170"/>
       <x:c r="U22" s="171"/>
@@ -34322,7 +34319,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C24" s="98" t="s">
-        <x:v>714</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="D24" s="93" t="str">
         <x:f t="shared" ref="D24:D31" si="18">REPT("   ", B24*2) &amp; C24</x:f>
@@ -34348,7 +34345,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M24" s="98" t="s">
-        <x:v>715</x:v>
+        <x:v>714</x:v>
       </x:c>
       <x:c r="N24" s="142">
         <x:v>1</x:v>
@@ -34417,7 +34414,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C25" s="98" t="s">
-        <x:v>716</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="D25" s="93" t="str">
         <x:f t="shared" si="18"/>
@@ -34443,7 +34440,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M25" s="98" t="s">
-        <x:v>717</x:v>
+        <x:v>716</x:v>
       </x:c>
       <x:c r="N25" s="142">
         <x:v>1</x:v>
@@ -34520,7 +34517,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C26" s="98" t="s">
-        <x:v>718</x:v>
+        <x:v>717</x:v>
       </x:c>
       <x:c r="D26" s="93" t="str">
         <x:f t="shared" si="18"/>
@@ -34565,7 +34562,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C27" s="98" t="s">
-        <x:v>719</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="D27" s="93" t="str">
         <x:f t="shared" si="18"/>
@@ -34591,7 +34588,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M27" s="155" t="s">
-        <x:v>720</x:v>
+        <x:v>719</x:v>
       </x:c>
       <x:c r="N27" s="142">
         <x:v>1</x:v>
@@ -34609,7 +34606,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S27" s="144" t="s">
-        <x:v>713</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="T27" s="102"/>
       <x:c r="U27" s="122"/>
@@ -34661,7 +34658,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C28" s="98" t="s">
-        <x:v>721</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="D28" s="93" t="str">
         <x:f t="shared" si="18"/>
@@ -34683,7 +34680,7 @@
         <x:v>186</x:v>
       </x:c>
       <x:c r="M28" s="155" t="s">
-        <x:v>722</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="N28" s="121">
         <x:v>1</x:v>
@@ -34701,11 +34698,11 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S28" s="102" t="s">
-        <x:v>723</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="T28" s="102"/>
       <x:c r="U28" s="140" t="s">
-        <x:v>724</x:v>
+        <x:v>723</x:v>
       </x:c>
       <x:c r="V28" s="103"/>
       <x:c r="W28" s="145" t="s">
@@ -34755,7 +34752,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C29" s="98" t="s">
-        <x:v>725</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="D29" s="93" t="str">
         <x:f t="shared" si="18"/>
@@ -34777,7 +34774,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M29" s="155" t="s">
-        <x:v>726</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="N29" s="121">
         <x:v>1</x:v>
@@ -34795,7 +34792,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S29" s="144" t="s">
-        <x:v>713</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="T29" s="102"/>
       <x:c r="U29" s="122"/>
@@ -34847,7 +34844,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C30" s="98" t="s">
-        <x:v>727</x:v>
+        <x:v>726</x:v>
       </x:c>
       <x:c r="D30" s="93" t="str">
         <x:f t="shared" si="18"/>
@@ -34892,7 +34889,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C31" s="98" t="s">
-        <x:v>728</x:v>
+        <x:v>727</x:v>
       </x:c>
       <x:c r="D31" s="93" t="str">
         <x:f t="shared" si="18"/>
@@ -34921,7 +34918,7 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S31" s="144" t="s">
-        <x:v>729</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="T31" s="102"/>
       <x:c r="U31" s="122"/>
@@ -35017,7 +35014,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C33" s="150" t="s">
-        <x:v>730</x:v>
+        <x:v>729</x:v>
       </x:c>
       <x:c r="D33" s="151" t="str">
         <x:f>REPT("   ", B33*2) &amp; C33</x:f>
@@ -35037,7 +35034,7 @@
       </x:c>
       <x:c r="L33" s="142"/>
       <x:c r="M33" s="155" t="s">
-        <x:v>731</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="N33" s="142">
         <x:v>300</x:v>
@@ -35114,7 +35111,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C34" s="150" t="s">
-        <x:v>732</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="D34" s="151" t="str">
         <x:f>REPT("   ", B34*2) &amp; C34</x:f>
@@ -35134,7 +35131,7 @@
       </x:c>
       <x:c r="L34" s="142"/>
       <x:c r="M34" s="155" t="s">
-        <x:v>731</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="N34" s="142">
         <x:v>300</x:v>
@@ -35211,7 +35208,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C35" s="150" t="s">
-        <x:v>733</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="D35" s="151" t="str">
         <x:f>REPT("   ", B35*2) &amp; C35</x:f>
@@ -35232,7 +35229,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M35" s="155" t="s">
-        <x:v>734</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="N35" s="142">
         <x:v>1</x:v>
@@ -35329,7 +35326,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M36" s="155" t="s">
-        <x:v>735</x:v>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="N36" s="142">
         <x:v>1</x:v>
@@ -35443,7 +35440,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C38" s="98" t="s">
-        <x:v>736</x:v>
+        <x:v>735</x:v>
       </x:c>
       <x:c r="D38" s="93" t="str">
         <x:f>REPT("   ", B38*2) &amp; C38</x:f>
@@ -35453,7 +35450,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F38" s="93" t="s">
-        <x:v>737</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="G38" s="94">
         <x:v>1</x:v>
@@ -35527,7 +35524,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C39" s="150" t="s">
-        <x:v>738</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="D39" s="151" t="str">
         <x:f t="shared" ref="D39" si="35">REPT("   ", B39*2) &amp; C39</x:f>
@@ -35551,7 +35548,7 @@
       </x:c>
       <x:c r="L39" s="142"/>
       <x:c r="M39" s="155" t="s">
-        <x:v>739</x:v>
+        <x:v>738</x:v>
       </x:c>
       <x:c r="N39" s="198" t="n">
         <x:f>200/3600</x:f>
@@ -35570,10 +35567,10 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S39" s="144" t="s">
+        <x:v>739</x:v>
+      </x:c>
+      <x:c r="T39" s="170" t="s">
         <x:v>740</x:v>
-      </x:c>
-      <x:c r="T39" s="170" t="s">
-        <x:v>741</x:v>
       </x:c>
       <x:c r="U39" s="171" t="s">
         <x:v>306</x:v>
@@ -35625,7 +35622,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C40" s="98" t="s">
-        <x:v>742</x:v>
+        <x:v>741</x:v>
       </x:c>
       <x:c r="D40" s="93" t="str">
         <x:f>REPT("   ", B40*2) &amp; C40</x:f>
@@ -35635,7 +35632,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F40" s="93" t="s">
-        <x:v>743</x:v>
+        <x:v>742</x:v>
       </x:c>
       <x:c r="G40" s="94">
         <x:v>1</x:v>
@@ -35663,7 +35660,7 @@
       <x:c r="T40" s="102"/>
       <x:c r="U40" s="122"/>
       <x:c r="V40" s="103" t="s">
-        <x:v>744</x:v>
+        <x:v>743</x:v>
       </x:c>
       <x:c r="W40" s="96" t="s">
         <x:v>43</x:v>
@@ -35721,7 +35718,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F41" s="93" t="s">
-        <x:v>737</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="G41" s="94">
         <x:v>1</x:v>
@@ -35745,13 +35742,13 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S41" s="102" t="s">
+        <x:v>744</x:v>
+      </x:c>
+      <x:c r="T41" s="102" t="s">
         <x:v>745</x:v>
       </x:c>
-      <x:c r="T41" s="102" t="s">
+      <x:c r="U41" s="140" t="s">
         <x:v>746</x:v>
-      </x:c>
-      <x:c r="U41" s="140" t="s">
-        <x:v>747</x:v>
       </x:c>
       <x:c r="V41" s="103"/>
       <x:c r="W41" s="145" t="s">
@@ -35800,7 +35797,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C42" s="98" t="s">
-        <x:v>748</x:v>
+        <x:v>747</x:v>
       </x:c>
       <x:c r="D42" s="93" t="str">
         <x:f>REPT("   ", B42*2) &amp; C42</x:f>
@@ -35823,7 +35820,7 @@
       </x:c>
       <x:c r="L42" s="100"/>
       <x:c r="M42" s="93" t="s">
-        <x:v>749</x:v>
+        <x:v>748</x:v>
       </x:c>
       <x:c r="N42" s="121"/>
       <x:c r="O42" s="100"/>
@@ -35835,7 +35832,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S42" s="102" t="s">
-        <x:v>750</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="T42" s="102"/>
       <x:c r="U42" s="122"/>
@@ -35886,7 +35883,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C43" s="98" t="s">
-        <x:v>751</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="D43" s="93" t="str">
         <x:f>REPT("   ", B43*2) &amp; C43</x:f>
@@ -35909,7 +35906,7 @@
       <x:c r="K43" s="120"/>
       <x:c r="L43" s="100"/>
       <x:c r="M43" s="93" t="s">
-        <x:v>752</x:v>
+        <x:v>751</x:v>
       </x:c>
       <x:c r="N43" s="121"/>
       <x:c r="O43" s="100"/>
@@ -36054,7 +36051,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="M45" s="155" t="s">
-        <x:v>753</x:v>
+        <x:v>752</x:v>
       </x:c>
       <x:c r="N45" s="142">
         <x:v>1</x:v>
@@ -36131,7 +36128,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C46" s="150" t="s">
-        <x:v>754</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="D46" s="151" t="str">
         <x:f>REPT("   ", B46*2) &amp; C46</x:f>
@@ -36141,7 +36138,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F46" s="151" t="s">
-        <x:v>755</x:v>
+        <x:v>754</x:v>
       </x:c>
       <x:c r="G46" s="153">
         <x:v>1</x:v>
@@ -36164,7 +36161,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S46" s="144" t="s">
-        <x:v>713</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="T46" s="102"/>
       <x:c r="U46" s="122"/>
@@ -36233,7 +36230,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F47" s="151" t="s">
-        <x:v>756</x:v>
+        <x:v>755</x:v>
       </x:c>
       <x:c r="G47" s="153">
         <x:v>1</x:v>
@@ -36331,7 +36328,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M48" s="155" t="s">
-        <x:v>757</x:v>
+        <x:v>756</x:v>
       </x:c>
       <x:c r="N48" s="142">
         <x:v>1</x:v>
@@ -36430,7 +36427,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="M49" s="155" t="s">
-        <x:v>699</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="N49" s="142">
         <x:v>300</x:v>
@@ -36555,7 +36552,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F51" s="93" t="s">
-        <x:v>758</x:v>
+        <x:v>757</x:v>
       </x:c>
       <x:c r="G51" s="94">
         <x:v>1</x:v>
@@ -36642,7 +36639,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F52" s="93" t="s">
-        <x:v>759</x:v>
+        <x:v>758</x:v>
       </x:c>
       <x:c r="G52" s="94">
         <x:v>1</x:v>
@@ -36717,7 +36714,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C53" s="168" t="s">
-        <x:v>760</x:v>
+        <x:v>759</x:v>
       </x:c>
       <x:c r="D53" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -36762,7 +36759,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C54" s="168" t="s">
-        <x:v>761</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="D54" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -36772,7 +36769,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F54" s="93" t="s">
-        <x:v>762</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="G54" s="94">
         <x:v>1</x:v>
@@ -36847,7 +36844,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C55" s="168" t="s">
-        <x:v>763</x:v>
+        <x:v>762</x:v>
       </x:c>
       <x:c r="D55" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -36857,7 +36854,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F55" s="93" t="s">
-        <x:v>764</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="G55" s="94">
         <x:v>1</x:v>
@@ -36932,7 +36929,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C56" s="168" t="s">
-        <x:v>765</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="D56" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -36942,7 +36939,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F56" s="93" t="s">
-        <x:v>766</x:v>
+        <x:v>765</x:v>
       </x:c>
       <x:c r="G56" s="94">
         <x:v>1</x:v>
@@ -37017,7 +37014,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C57" s="168" t="s">
-        <x:v>767</x:v>
+        <x:v>766</x:v>
       </x:c>
       <x:c r="D57" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -37027,7 +37024,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F57" s="93" t="s">
-        <x:v>768</x:v>
+        <x:v>767</x:v>
       </x:c>
       <x:c r="G57" s="94">
         <x:v>1</x:v>
@@ -37102,7 +37099,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C58" s="168" t="s">
-        <x:v>769</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="D58" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -37147,7 +37144,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C59" s="168" t="s">
-        <x:v>770</x:v>
+        <x:v>769</x:v>
       </x:c>
       <x:c r="D59" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -37157,7 +37154,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F59" s="93" t="s">
-        <x:v>771</x:v>
+        <x:v>770</x:v>
       </x:c>
       <x:c r="G59" s="94">
         <x:v>1</x:v>
@@ -37180,7 +37177,7 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S59" s="110" t="s">
-        <x:v>729</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="T59" s="110"/>
       <x:c r="U59" s="200"/>
@@ -37232,7 +37229,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C60" s="168" t="s">
-        <x:v>772</x:v>
+        <x:v>771</x:v>
       </x:c>
       <x:c r="D60" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -37265,7 +37262,7 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S60" s="110" t="s">
-        <x:v>729</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="T60" s="110"/>
       <x:c r="U60" s="200"/>
@@ -37385,7 +37382,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="M62" s="178" t="s">
-        <x:v>700</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="N62" s="103">
         <x:v>1068</x:v>
@@ -37462,7 +37459,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F63" s="93" t="s">
-        <x:v>773</x:v>
+        <x:v>772</x:v>
       </x:c>
       <x:c r="G63" s="94">
         <x:v>1</x:v>
@@ -37546,7 +37543,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F64" s="93" t="s">
-        <x:v>774</x:v>
+        <x:v>773</x:v>
       </x:c>
       <x:c r="G64" s="94">
         <x:v>1</x:v>
@@ -37630,7 +37627,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F65" s="93" t="s">
-        <x:v>775</x:v>
+        <x:v>774</x:v>
       </x:c>
       <x:c r="G65" s="94">
         <x:v>1</x:v>
@@ -37704,7 +37701,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C66" s="168" t="s">
-        <x:v>776</x:v>
+        <x:v>775</x:v>
       </x:c>
       <x:c r="D66" s="93" t="str">
         <x:f>REPT("   ", B66*2) &amp; C66</x:f>
@@ -37714,7 +37711,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F66" s="93" t="s">
-        <x:v>777</x:v>
+        <x:v>776</x:v>
       </x:c>
       <x:c r="G66" s="94">
         <x:v>1</x:v>
@@ -38263,7 +38260,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M75" s="93" t="s">
-        <x:v>749</x:v>
+        <x:v>748</x:v>
       </x:c>
       <x:c r="N75" s="103"/>
       <x:c r="O75" s="103"/>
@@ -38339,7 +38336,7 @@
         <x:v>268</x:v>
       </x:c>
       <x:c r="F76" s="93" t="s">
-        <x:v>778</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="G76" s="94">
         <x:v>1</x:v>
@@ -38354,7 +38351,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M76" s="58" t="s">
-        <x:v>779</x:v>
+        <x:v>778</x:v>
       </x:c>
       <x:c r="N76" s="103"/>
       <x:c r="O76" s="103"/>
@@ -38420,7 +38417,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C77" s="109" t="s">
-        <x:v>678</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="D77" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -38430,7 +38427,7 @@
         <x:v>268</x:v>
       </x:c>
       <x:c r="F77" s="93" t="s">
-        <x:v>778</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="G77" s="94">
         <x:v>1</x:v>
@@ -38445,7 +38442,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M77" s="58" t="s">
-        <x:v>780</x:v>
+        <x:v>779</x:v>
       </x:c>
       <x:c r="N77" s="103"/>
       <x:c r="O77" s="103"/>
@@ -38511,7 +38508,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C78" s="109" t="s">
-        <x:v>781</x:v>
+        <x:v>780</x:v>
       </x:c>
       <x:c r="D78" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -38532,7 +38529,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M78" s="183" t="s">
-        <x:v>782</x:v>
+        <x:v>781</x:v>
       </x:c>
       <x:c r="N78" s="103"/>
       <x:c r="O78" s="103"/>
@@ -38594,7 +38591,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C79" s="109" t="s">
-        <x:v>682</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="D79" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -38655,7 +38652,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C80" s="109" t="s">
-        <x:v>683</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="D80" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -38716,7 +38713,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C81" s="109" t="s">
-        <x:v>686</x:v>
+        <x:v>685</x:v>
       </x:c>
       <x:c r="D81" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -38761,7 +38758,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C82" s="109" t="s">
-        <x:v>783</x:v>
+        <x:v>782</x:v>
       </x:c>
       <x:c r="D82" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -38820,7 +38817,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C83" s="109" t="s">
-        <x:v>784</x:v>
+        <x:v>783</x:v>
       </x:c>
       <x:c r="D83" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -38879,7 +38876,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C84" s="109" t="s">
-        <x:v>689</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="D84" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -38938,7 +38935,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C85" s="109" t="s">
-        <x:v>690</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="D85" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -38963,7 +38960,7 @@
         <x:v>426</x:v>
       </x:c>
       <x:c r="M85" s="93" t="s">
-        <x:v>785</x:v>
+        <x:v>784</x:v>
       </x:c>
       <x:c r="N85" s="103"/>
       <x:c r="O85" s="103"/>
@@ -39027,7 +39024,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C86" s="109" t="s">
-        <x:v>694</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="D86" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -39086,7 +39083,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C87" s="109" t="s">
-        <x:v>786</x:v>
+        <x:v>785</x:v>
       </x:c>
       <x:c r="D87" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -39131,7 +39128,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C88" s="109" t="s">
-        <x:v>787</x:v>
+        <x:v>786</x:v>
       </x:c>
       <x:c r="D88" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -39141,7 +39138,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F88" s="93" t="s">
-        <x:v>788</x:v>
+        <x:v>787</x:v>
       </x:c>
       <x:c r="G88" s="94">
         <x:v>1</x:v>
@@ -39164,12 +39161,12 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S88" s="110" t="s">
-        <x:v>789</x:v>
+        <x:v>788</x:v>
       </x:c>
       <x:c r="T88" s="111"/>
       <x:c r="U88" s="182"/>
       <x:c r="V88" s="103" t="s">
-        <x:v>790</x:v>
+        <x:v>789</x:v>
       </x:c>
       <x:c r="W88" s="96" t="s">
         <x:v>43</x:v>
@@ -39216,7 +39213,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C89" s="109" t="s">
-        <x:v>791</x:v>
+        <x:v>790</x:v>
       </x:c>
       <x:c r="D89" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -39226,7 +39223,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F89" s="93" t="s">
-        <x:v>792</x:v>
+        <x:v>791</x:v>
       </x:c>
       <x:c r="G89" s="94">
         <x:v>1</x:v>
@@ -39321,7 +39318,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C90" s="109" t="s">
-        <x:v>793</x:v>
+        <x:v>792</x:v>
       </x:c>
       <x:c r="D90" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -39331,7 +39328,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F90" s="93" t="s">
-        <x:v>794</x:v>
+        <x:v>793</x:v>
       </x:c>
       <x:c r="G90" s="94">
         <x:v>1</x:v>
@@ -39354,12 +39351,12 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S90" s="110" t="s">
-        <x:v>789</x:v>
+        <x:v>788</x:v>
       </x:c>
       <x:c r="T90" s="111"/>
       <x:c r="U90" s="182"/>
       <x:c r="V90" s="103" t="s">
-        <x:v>790</x:v>
+        <x:v>789</x:v>
       </x:c>
       <x:c r="W90" s="96" t="s">
         <x:v>43</x:v>
@@ -39406,7 +39403,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C91" s="109" t="s">
-        <x:v>695</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="D91" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -39431,7 +39428,7 @@
         <x:v>186</x:v>
       </x:c>
       <x:c r="M91" s="110" t="s">
-        <x:v>795</x:v>
+        <x:v>794</x:v>
       </x:c>
       <x:c r="N91" s="103"/>
       <x:c r="O91" s="103" t="s">
@@ -39501,7 +39498,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C92" s="109" t="s">
-        <x:v>697</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="D92" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -39546,7 +39543,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C93" s="109" t="s">
-        <x:v>796</x:v>
+        <x:v>795</x:v>
       </x:c>
       <x:c r="D93" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -39591,7 +39588,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C94" s="168" t="s">
-        <x:v>797</x:v>
+        <x:v>796</x:v>
       </x:c>
       <x:c r="D94" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -39601,7 +39598,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F94" s="93" t="s">
-        <x:v>762</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="G94" s="94">
         <x:v>1</x:v>
@@ -39675,7 +39672,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C95" s="168" t="s">
-        <x:v>798</x:v>
+        <x:v>797</x:v>
       </x:c>
       <x:c r="D95" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -39685,7 +39682,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F95" s="93" t="s">
-        <x:v>764</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="G95" s="94">
         <x:v>1</x:v>
@@ -39759,7 +39756,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C96" s="168" t="s">
-        <x:v>799</x:v>
+        <x:v>798</x:v>
       </x:c>
       <x:c r="D96" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -39769,7 +39766,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F96" s="93" t="s">
-        <x:v>766</x:v>
+        <x:v>765</x:v>
       </x:c>
       <x:c r="G96" s="94">
         <x:v>1</x:v>
@@ -39843,7 +39840,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C97" s="168" t="s">
-        <x:v>800</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="D97" s="93" t="str">
         <x:f t="shared" si="44"/>
@@ -39853,7 +39850,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F97" s="93" t="s">
-        <x:v>768</x:v>
+        <x:v>767</x:v>
       </x:c>
       <x:c r="G97" s="94">
         <x:v>1</x:v>
@@ -40267,14 +40264,14 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R2ad1b1489ade4d8f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U28" r:id="Rff2748059c9a4aea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U39" r:id="R86c49c6e4be44f11"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U41" r:id="Rf90db87564f247b2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U91" r:id="R453239ad03994f92"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R068b229e001347fe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U28" r:id="Rc2677a276c53417e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U39" r:id="Rdc4d9a12530b4af2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U41" r:id="Rb2482be7c8cc4fba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U91" r:id="R70fd82d2dd914985"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re973f8de94c44059"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f53923f849d4d4d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0408c5e59efc4cb8"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73b17a3281fd49a5"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
review the learning rate for the I&C
</commit_message>
<xml_diff>
--- a/cost/Cost_Database.xlsx
+++ b/cost/Cost_Database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hannbn/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{396B7A26-B56F-DE47-84C2-CDB0D8DE6E1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0F6E66C-7A4E-0649-AAD6-8993B7B57FBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7123,6 +7123,114 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>647700</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F2ABC046-3547-9390-8110-2C1ED17FE39B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>647700</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B3ED3600-9A72-7A2E-D279-FB6A7B8E306D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -7177,6 +7285,114 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>609600</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>584200</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="AutoShape 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0024F735-21E0-4121-B717-94EC49AD7E18}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>609600</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>584200</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="AutoShape 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C7ED2439-8D13-6B90-CF3C-7EE7333B5DCE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -7224,6 +7440,114 @@
             <a:srgbClr val="000000"/>
           </a:solidFill>
           <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>609600</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>431800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="AutoShape 33">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A8946A51-B997-79FA-8123-ABD74F135478}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>609600</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="AutoShape 33">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E33490CB-640B-7AEE-C7DE-535CA439729F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
           <a:headEnd/>
           <a:tailEnd/>
         </a:ln>
@@ -18438,8 +18762,8 @@
       <c r="V131" s="49" t="s">
         <v>331</v>
       </c>
-      <c r="W131" s="74" t="s">
-        <v>157</v>
+      <c r="W131" s="3" t="s">
+        <v>340</v>
       </c>
       <c r="X131" s="77">
         <f t="shared" si="28"/>
@@ -18796,7 +19120,7 @@
       </c>
       <c r="V136" s="49"/>
       <c r="W136" s="74" t="s">
-        <v>157</v>
+        <v>340</v>
       </c>
       <c r="X136" s="77">
         <f>0.9*$J136</f>
@@ -28479,7 +28803,7 @@
       <c r="AF18" s="97"/>
       <c r="AG18" s="96"/>
     </row>
-    <row r="19" spans="1:33" ht="57" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:33" ht="71" x14ac:dyDescent="0.2">
       <c r="A19" s="107">
         <v>214.31</v>
       </c>
@@ -28975,7 +29299,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="25" spans="1:33" ht="57" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:33" ht="71" x14ac:dyDescent="0.2">
       <c r="A25" s="148">
         <v>225</v>
       </c>
@@ -29334,7 +29658,7 @@
       <c r="AF29" s="97"/>
       <c r="AG29" s="96"/>
     </row>
-    <row r="30" spans="1:33" ht="57" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:33" ht="71" x14ac:dyDescent="0.2">
       <c r="A30" s="148">
         <v>283</v>
       </c>
@@ -29427,7 +29751,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="31" spans="1:33" ht="57" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:33" ht="71" x14ac:dyDescent="0.2">
       <c r="A31" s="148">
         <v>284</v>
       </c>
@@ -30573,7 +30897,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="49" spans="1:33" ht="57" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:33" ht="71" x14ac:dyDescent="0.2">
       <c r="A49" s="107">
         <v>712</v>
       </c>

</xml_diff>

<commit_message>
imporve the shielding estimation capability
</commit_message>
<xml_diff>
--- a/cost/Cost_Database.xlsx
+++ b/cost/Cost_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hannbn/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7FDA0AA-A281-F041-BB3D-1C90CC64D0A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9618D5C-A140-5F40-95A5-312EBA168CE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cost Database" sheetId="1" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4672" uniqueCount="743">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4676" uniqueCount="747">
   <si>
     <t>Account</t>
   </si>
@@ -2357,6 +2357,18 @@
   <si>
     <t>Primary Loop Purification</t>
   </si>
+  <si>
+    <t>UO2 Learning</t>
+  </si>
+  <si>
+    <t>TRISO Learning</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># UO2 learning rate = 0.02 per doubling. This is an inferred effective rate that gives a 12.6% reduction by unit 100, consistent with the approximately 8–15% fabrication-cost reduction associated with increased UO2 plant throughput in AFC-CBR Module D1-1, Section D1-1.10.2 and Figure D1-1.6. </t>
+  </si>
+  <si>
+    <t># TRISO learning rate = 0.13 per doubling. This is an inferred effective rate that gives a 60.4% reduction by unit 100, approximately representing the reduction from the report’s ~$25,000/kgU current-production estimate toward its ~$10,000/kgU automated-production target in AFC-CBR Module D1-3, Section D1-3.8 and Tables D1-3-8 through D1-3-10.</t>
+  </si>
 </sst>
 </file>
 
@@ -2371,7 +2383,7 @@
     <numFmt numFmtId="168" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="169" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;?_);_(@_)"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2496,6 +2508,12 @@
       <sz val="13"/>
       <color rgb="FF222222"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -2708,7 +2726,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="167">
+  <cellXfs count="169">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3077,21 +3095,21 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -3099,8 +3117,8 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="11" fillId="2" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3125,15 +3143,17 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Comma" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -5488,6 +5508,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>647700</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DF208E70-AB10-8224-E903-7971C5164110}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -5961,7 +6035,7 @@
       <c r="S3" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="T3" s="143" t="s">
+      <c r="T3" s="147" t="s">
         <v>41</v>
       </c>
       <c r="U3" s="150" t="s">
@@ -6586,13 +6660,13 @@
       <c r="R11" s="45" t="s">
         <v>73</v>
       </c>
-      <c r="S11" s="143" t="s">
+      <c r="S11" s="147" t="s">
         <v>74</v>
       </c>
-      <c r="T11" s="143" t="s">
+      <c r="T11" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="U11" s="148" t="s">
+      <c r="U11" s="146" t="s">
         <v>76</v>
       </c>
       <c r="V11" s="49"/>
@@ -6909,13 +6983,13 @@
       <c r="R15" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="S15" s="143" t="s">
+      <c r="S15" s="147" t="s">
         <v>74</v>
       </c>
-      <c r="T15" s="143" t="s">
+      <c r="T15" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="U15" s="148" t="s">
+      <c r="U15" s="146" t="s">
         <v>76</v>
       </c>
       <c r="V15" s="49"/>
@@ -7455,13 +7529,13 @@
       <c r="R22" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="S22" s="143" t="s">
+      <c r="S22" s="147" t="s">
         <v>105</v>
       </c>
-      <c r="T22" s="143" t="s">
+      <c r="T22" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="U22" s="148" t="s">
+      <c r="U22" s="146" t="s">
         <v>76</v>
       </c>
       <c r="V22" s="49"/>
@@ -7764,13 +7838,13 @@
       <c r="R26" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="S26" s="143" t="s">
+      <c r="S26" s="147" t="s">
         <v>105</v>
       </c>
-      <c r="T26" s="143" t="s">
+      <c r="T26" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="U26" s="148" t="s">
+      <c r="U26" s="146" t="s">
         <v>76</v>
       </c>
       <c r="V26" s="49"/>
@@ -8081,13 +8155,13 @@
       <c r="R30" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="S30" s="143" t="s">
+      <c r="S30" s="147" t="s">
         <v>105</v>
       </c>
-      <c r="T30" s="143" t="s">
+      <c r="T30" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="U30" s="148" t="s">
+      <c r="U30" s="146" t="s">
         <v>76</v>
       </c>
       <c r="V30" s="49"/>
@@ -8588,13 +8662,13 @@
       <c r="R37" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="S37" s="143" t="s">
+      <c r="S37" s="147" t="s">
         <v>74</v>
       </c>
-      <c r="T37" s="143" t="s">
+      <c r="T37" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="U37" s="148" t="s">
+      <c r="U37" s="146" t="s">
         <v>76</v>
       </c>
       <c r="V37" s="49"/>
@@ -8895,13 +8969,13 @@
       <c r="R41" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="S41" s="143" t="s">
+      <c r="S41" s="147" t="s">
         <v>74</v>
       </c>
-      <c r="T41" s="143" t="s">
+      <c r="T41" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="U41" s="148" t="s">
+      <c r="U41" s="146" t="s">
         <v>76</v>
       </c>
       <c r="V41" s="49"/>
@@ -9256,13 +9330,13 @@
       <c r="R46" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="S46" s="143" t="s">
+      <c r="S46" s="147" t="s">
         <v>105</v>
       </c>
-      <c r="T46" s="143" t="s">
+      <c r="T46" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="U46" s="148" t="s">
+      <c r="U46" s="146" t="s">
         <v>76</v>
       </c>
       <c r="V46" s="49"/>
@@ -9707,16 +9781,16 @@
       <c r="R52" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="S52" s="143" t="s">
+      <c r="S52" s="147" t="s">
         <v>105</v>
       </c>
-      <c r="T52" s="143" t="s">
+      <c r="T52" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="U52" s="148" t="s">
+      <c r="U52" s="146" t="s">
         <v>76</v>
       </c>
-      <c r="V52" s="149" t="s">
+      <c r="V52" s="152" t="s">
         <v>162</v>
       </c>
       <c r="W52" s="74" t="s">
@@ -10063,13 +10137,13 @@
       <c r="R57" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="S57" s="143" t="s">
+      <c r="S57" s="147" t="s">
         <v>105</v>
       </c>
-      <c r="T57" s="143" t="s">
+      <c r="T57" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="U57" s="148" t="s">
+      <c r="U57" s="146" t="s">
         <v>76</v>
       </c>
       <c r="V57" s="49"/>
@@ -10372,13 +10446,13 @@
       <c r="R61" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="S61" s="143" t="s">
+      <c r="S61" s="147" t="s">
         <v>74</v>
       </c>
-      <c r="T61" s="143" t="s">
+      <c r="T61" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="U61" s="148" t="s">
+      <c r="U61" s="146" t="s">
         <v>76</v>
       </c>
       <c r="V61" s="49"/>
@@ -10876,7 +10950,7 @@
       <c r="S68" s="58" t="s">
         <v>196</v>
       </c>
-      <c r="T68" s="146" t="s">
+      <c r="T68" s="148" t="s">
         <v>197</v>
       </c>
       <c r="U68" s="55"/>
@@ -11557,10 +11631,10 @@
       <c r="S76" s="58" t="s">
         <v>209</v>
       </c>
-      <c r="T76" s="146" t="s">
+      <c r="T76" s="148" t="s">
         <v>210</v>
       </c>
-      <c r="U76" s="152" t="s">
+      <c r="U76" s="149" t="s">
         <v>211</v>
       </c>
       <c r="V76" s="58" t="s">
@@ -12738,7 +12812,7 @@
       <c r="T89" s="58" t="s">
         <v>210</v>
       </c>
-      <c r="U89" s="152" t="s">
+      <c r="U89" s="149" t="s">
         <v>211</v>
       </c>
       <c r="V89" s="49"/>
@@ -14470,13 +14544,13 @@
       <c r="S109" s="58" t="s">
         <v>272</v>
       </c>
-      <c r="T109" s="146" t="s">
+      <c r="T109" s="148" t="s">
         <v>273</v>
       </c>
       <c r="U109" s="151" t="s">
         <v>274</v>
       </c>
-      <c r="V109" s="146"/>
+      <c r="V109" s="148"/>
       <c r="W109" s="74" t="s">
         <v>157</v>
       </c>
@@ -15761,7 +15835,7 @@
         <v>296</v>
       </c>
       <c r="U123" s="80"/>
-      <c r="V123" s="146" t="s">
+      <c r="V123" s="148" t="s">
         <v>311</v>
       </c>
       <c r="W123" s="74" t="s">
@@ -16885,10 +16959,10 @@
       <c r="R138" s="49" t="s">
         <v>86</v>
       </c>
-      <c r="S138" s="147" t="s">
+      <c r="S138" s="143" t="s">
         <v>344</v>
       </c>
-      <c r="T138" s="147" t="s">
+      <c r="T138" s="143" t="s">
         <v>345</v>
       </c>
       <c r="U138" s="49"/>
@@ -17414,7 +17488,7 @@
       <c r="AF144" s="76"/>
       <c r="AG144" s="74"/>
     </row>
-    <row r="145" spans="1:33" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:34" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="53">
         <v>251</v>
       </c>
@@ -17455,10 +17529,10 @@
       <c r="R145" s="49" t="s">
         <v>219</v>
       </c>
-      <c r="S145" s="146" t="s">
+      <c r="S145" s="148" t="s">
         <v>354</v>
       </c>
-      <c r="T145" s="146" t="s">
+      <c r="T145" s="148" t="s">
         <v>355</v>
       </c>
       <c r="U145" s="49"/>
@@ -17501,7 +17575,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="146" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="53">
         <v>252</v>
       </c>
@@ -17584,7 +17658,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="147" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="53">
         <v>253</v>
       </c>
@@ -17669,7 +17743,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="148" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="53">
         <v>254</v>
       </c>
@@ -17760,7 +17834,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="149" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="53">
         <v>254</v>
       </c>
@@ -17799,7 +17873,7 @@
       </c>
       <c r="J149" s="65"/>
       <c r="K149" s="65">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="L149" s="49" t="s">
         <v>186</v>
@@ -17811,7 +17885,7 @@
       <c r="O149" s="49"/>
       <c r="P149" s="49"/>
       <c r="Q149" s="65">
-        <v>2023</v>
+        <v>2017</v>
       </c>
       <c r="R149" s="49" t="s">
         <v>219</v>
@@ -17821,7 +17895,7 @@
       <c r="U149" s="49"/>
       <c r="V149" s="49"/>
       <c r="W149" s="74" t="s">
-        <v>157</v>
+        <v>743</v>
       </c>
       <c r="X149" s="77">
         <f t="shared" si="38"/>
@@ -17835,12 +17909,10 @@
         <v>44</v>
       </c>
       <c r="AA149" s="76">
-        <f t="shared" si="40"/>
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="AB149" s="76">
-        <f t="shared" si="41"/>
-        <v>325</v>
+        <v>575</v>
       </c>
       <c r="AC149" s="74" t="s">
         <v>44</v>
@@ -17857,8 +17929,11 @@
       <c r="AG149" s="74" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="150" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AH149" s="167" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="150" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="53">
         <v>254</v>
       </c>
@@ -17893,7 +17968,7 @@
       <c r="I150" s="45"/>
       <c r="J150" s="65"/>
       <c r="K150" s="65">
-        <v>10000</v>
+        <v>10900</v>
       </c>
       <c r="L150" s="49" t="s">
         <v>186</v>
@@ -17905,7 +17980,7 @@
       <c r="O150" s="49"/>
       <c r="P150" s="49"/>
       <c r="Q150" s="65">
-        <v>2009</v>
+        <v>2017</v>
       </c>
       <c r="R150" s="49" t="s">
         <v>219</v>
@@ -17915,7 +17990,7 @@
       <c r="U150" s="49"/>
       <c r="V150" s="49"/>
       <c r="W150" s="74" t="s">
-        <v>157</v>
+        <v>744</v>
       </c>
       <c r="X150" s="77">
         <f t="shared" si="38"/>
@@ -17929,12 +18004,12 @@
         <v>44</v>
       </c>
       <c r="AA150" s="76">
-        <f t="shared" si="40"/>
-        <v>9000</v>
+        <f>0.5*K150</f>
+        <v>5450</v>
       </c>
       <c r="AB150" s="76">
-        <f t="shared" si="41"/>
-        <v>13000</v>
+        <f>3*K150</f>
+        <v>32700</v>
       </c>
       <c r="AC150" s="74" t="s">
         <v>44</v>
@@ -17951,8 +18026,11 @@
       <c r="AG150" s="74" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="151" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AH150" s="168" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="151" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="37">
         <v>26</v>
       </c>
@@ -18042,7 +18120,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="152" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="37">
         <v>27</v>
       </c>
@@ -18109,7 +18187,7 @@
       <c r="AF152" s="76"/>
       <c r="AG152" s="74"/>
     </row>
-    <row r="153" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="50">
         <v>30</v>
       </c>
@@ -18161,7 +18239,7 @@
       <c r="AF153" s="76"/>
       <c r="AG153" s="74"/>
     </row>
-    <row r="154" spans="1:33" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:34" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="50">
         <v>31</v>
       </c>
@@ -18205,7 +18283,7 @@
       <c r="AF154" s="76"/>
       <c r="AG154" s="74"/>
     </row>
-    <row r="155" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="50">
         <v>32</v>
       </c>
@@ -18249,7 +18327,7 @@
       <c r="AF155" s="76"/>
       <c r="AG155" s="74"/>
     </row>
-    <row r="156" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="37">
         <v>33</v>
       </c>
@@ -18294,7 +18372,7 @@
       <c r="R156" s="46" t="s">
         <v>73</v>
       </c>
-      <c r="S156" s="143" t="s">
+      <c r="S156" s="147" t="s">
         <v>320</v>
       </c>
       <c r="T156" s="46"/>
@@ -18338,7 +18416,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="157" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="37">
         <v>34</v>
       </c>
@@ -18418,7 +18496,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="158" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="37">
         <v>35</v>
       </c>
@@ -18498,7 +18576,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="159" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="37">
         <v>36</v>
       </c>
@@ -18578,7 +18656,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="160" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="37">
         <v>40</v>
       </c>
@@ -19550,14 +19628,14 @@
       <c r="P174" s="49"/>
       <c r="Q174" s="65"/>
       <c r="R174" s="49"/>
-      <c r="S174" s="146" t="s">
+      <c r="S174" s="148" t="s">
         <v>403</v>
       </c>
-      <c r="T174" s="146" t="s">
+      <c r="T174" s="148" t="s">
         <v>403</v>
       </c>
       <c r="U174" s="49"/>
-      <c r="V174" s="146" t="s">
+      <c r="V174" s="148" t="s">
         <v>404</v>
       </c>
       <c r="W174" s="74"/>
@@ -20548,6 +20626,43 @@
     </row>
   </sheetData>
   <mergeCells count="53">
+    <mergeCell ref="T26:T28"/>
+    <mergeCell ref="T41:T43"/>
+    <mergeCell ref="V109:V110"/>
+    <mergeCell ref="T61:T63"/>
+    <mergeCell ref="T76:T80"/>
+    <mergeCell ref="S138:S143"/>
+    <mergeCell ref="T11:T13"/>
+    <mergeCell ref="V174:V188"/>
+    <mergeCell ref="S30:S32"/>
+    <mergeCell ref="S15:S17"/>
+    <mergeCell ref="T37:T39"/>
+    <mergeCell ref="T46:T48"/>
+    <mergeCell ref="T22:T24"/>
+    <mergeCell ref="U52:U54"/>
+    <mergeCell ref="S26:S28"/>
+    <mergeCell ref="U26:U28"/>
+    <mergeCell ref="T52:T54"/>
+    <mergeCell ref="V123:V124"/>
+    <mergeCell ref="S156:S159"/>
+    <mergeCell ref="T145:T150"/>
+    <mergeCell ref="V52:V54"/>
+    <mergeCell ref="U3:U4"/>
+    <mergeCell ref="T57:T59"/>
+    <mergeCell ref="T15:T17"/>
+    <mergeCell ref="S41:S43"/>
+    <mergeCell ref="U109:U110"/>
+    <mergeCell ref="T68:T73"/>
+    <mergeCell ref="S46:S48"/>
+    <mergeCell ref="S22:S24"/>
+    <mergeCell ref="U22:U24"/>
+    <mergeCell ref="T30:T32"/>
+    <mergeCell ref="U5:U6"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="S11:S13"/>
+    <mergeCell ref="U11:U13"/>
+    <mergeCell ref="U37:U39"/>
+    <mergeCell ref="T109:T110"/>
     <mergeCell ref="T138:T143"/>
     <mergeCell ref="U30:U32"/>
     <mergeCell ref="S52:S54"/>
@@ -20564,43 +20679,6 @@
     <mergeCell ref="S57:S59"/>
     <mergeCell ref="S37:S39"/>
     <mergeCell ref="U89:U99"/>
-    <mergeCell ref="U3:U4"/>
-    <mergeCell ref="T57:T59"/>
-    <mergeCell ref="T15:T17"/>
-    <mergeCell ref="S41:S43"/>
-    <mergeCell ref="U109:U110"/>
-    <mergeCell ref="T68:T73"/>
-    <mergeCell ref="S46:S48"/>
-    <mergeCell ref="S22:S24"/>
-    <mergeCell ref="U22:U24"/>
-    <mergeCell ref="T30:T32"/>
-    <mergeCell ref="U5:U6"/>
-    <mergeCell ref="T3:T4"/>
-    <mergeCell ref="S11:S13"/>
-    <mergeCell ref="U11:U13"/>
-    <mergeCell ref="U37:U39"/>
-    <mergeCell ref="T109:T110"/>
-    <mergeCell ref="S138:S143"/>
-    <mergeCell ref="T11:T13"/>
-    <mergeCell ref="V174:V188"/>
-    <mergeCell ref="S30:S32"/>
-    <mergeCell ref="S15:S17"/>
-    <mergeCell ref="T37:T39"/>
-    <mergeCell ref="T46:T48"/>
-    <mergeCell ref="T22:T24"/>
-    <mergeCell ref="U52:U54"/>
-    <mergeCell ref="S26:S28"/>
-    <mergeCell ref="U26:U28"/>
-    <mergeCell ref="T52:T54"/>
-    <mergeCell ref="V123:V124"/>
-    <mergeCell ref="S156:S159"/>
-    <mergeCell ref="T145:T150"/>
-    <mergeCell ref="V52:V54"/>
-    <mergeCell ref="T26:T28"/>
-    <mergeCell ref="T41:T43"/>
-    <mergeCell ref="V109:V110"/>
-    <mergeCell ref="T61:T63"/>
-    <mergeCell ref="T76:T80"/>
   </mergeCells>
   <conditionalFormatting sqref="A100:B106">
     <cfRule type="expression" dxfId="312" priority="586">
@@ -20677,17 +20755,17 @@
       <formula>$B76=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A98:V99 D100:D106 A125:V126 A129:B130 D129:V130 A131:V143 A144:AG147 A148:G149 I148:AG149 A150:AG151 A152:V152 A153:AG173">
+  <conditionalFormatting sqref="A98:V99 D100:D106 A125:V126 A129:B130 D129:V130 A131:V143 A144:AG147 A148:G149 I148:AG149 A150:AG151 A152:V152 A153:AG173 W145:W150">
     <cfRule type="expression" dxfId="293" priority="633">
       <formula>$B98&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A112:V114 U116:V122 U123:U124 A127:S128 U127:V128 A144:AG147 A148:G149 I148:AG149 A150:AG151 A153:AG173 A138:B143 U138:V143 U146:V152 A5:S6 A109:F111 X152:AG152 A1:AG4 U5:AG6">
+  <conditionalFormatting sqref="A112:V114 U116:V122 U123:U124 A127:S128 U127:V128 A144:AG147 A148:G149 I148:AG149 A150:AG151 A153:AG173 A138:B143 U138:V143 U146:V152 A5:S6 A109:F111 X152:AG152 A1:AG4 U5:AG6 W145:W150">
     <cfRule type="expression" dxfId="292" priority="797">
       <formula>$B1=3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A125:V126 A129:B130 D129:V130 A131:V143 A98:V99 D100:D106 A152:V152 A144:AG147 A148:G149 I148:AG149 A150:AG151 A153:AG173">
+  <conditionalFormatting sqref="A125:V126 A129:B130 D129:V130 A131:V143 A98:V99 D100:D106 A152:V152 A144:AG147 A148:G149 I148:AG149 A150:AG151 A153:AG173 W145:W150">
     <cfRule type="expression" dxfId="291" priority="632">
       <formula>$B98=2</formula>
     </cfRule>
@@ -20811,7 +20889,7 @@
       <formula>$B136=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A144:AG147 A148:G149 I148:AG149 A150:AG151 A152:V153 A153:AG173">
+  <conditionalFormatting sqref="A144:AG147 A148:G149 I148:AG149 A150:AG151 A152:V153 A153:AG173 W145:W150">
     <cfRule type="expression" dxfId="261" priority="566">
       <formula>$B144=0</formula>
     </cfRule>
@@ -24747,7 +24825,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.5" customWidth="1"/>
@@ -24936,6 +25014,22 @@
         <v>575</v>
       </c>
     </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>743</v>
+      </c>
+      <c r="B18">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>744</v>
+      </c>
+      <c r="B19">
+        <v>0.13</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="C9:C17"/>
@@ -24943,6 +25037,7 @@
     <mergeCell ref="D9:D16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -25195,7 +25290,7 @@
       <c r="T3" s="162" t="s">
         <v>41</v>
       </c>
-      <c r="U3" s="165" t="s">
+      <c r="U3" s="166" t="s">
         <v>42</v>
       </c>
       <c r="V3" s="105"/>
@@ -25391,7 +25486,7 @@
       <c r="T5" s="162" t="s">
         <v>63</v>
       </c>
-      <c r="U5" s="165" t="s">
+      <c r="U5" s="166" t="s">
         <v>58</v>
       </c>
       <c r="V5" s="105"/>
@@ -25841,7 +25936,7 @@
       <c r="T11" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U11" s="164" t="s">
+      <c r="U11" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V11" s="105"/>
@@ -26394,7 +26489,7 @@
       <c r="T18" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U18" s="164" t="s">
+      <c r="U18" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V18" s="105"/>
@@ -26805,7 +26900,7 @@
       <c r="T23" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U23" s="164" t="s">
+      <c r="U23" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V23" s="105"/>
@@ -27216,7 +27311,7 @@
       <c r="T28" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U28" s="164" t="s">
+      <c r="U28" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V28" s="105"/>
@@ -27627,7 +27722,7 @@
       <c r="T33" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U33" s="164" t="s">
+      <c r="U33" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V33" s="105"/>
@@ -28038,7 +28133,7 @@
       <c r="T38" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U38" s="164" t="s">
+      <c r="U38" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V38" s="105"/>
@@ -28588,7 +28683,7 @@
       <c r="T45" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U45" s="164" t="s">
+      <c r="U45" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V45" s="105"/>
@@ -29146,7 +29241,7 @@
       <c r="T52" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U52" s="164" t="s">
+      <c r="U52" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V52" s="105"/>
@@ -29562,7 +29657,7 @@
       <c r="T57" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U57" s="164" t="s">
+      <c r="U57" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V57" s="105"/>
@@ -29980,7 +30075,7 @@
       <c r="T62" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U62" s="164" t="s">
+      <c r="U62" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V62" s="105"/>
@@ -30391,7 +30486,7 @@
       <c r="T67" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U67" s="164" t="s">
+      <c r="U67" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V67" s="105"/>
@@ -30941,7 +31036,7 @@
       <c r="T74" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U74" s="164" t="s">
+      <c r="U74" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V74" s="105"/>
@@ -31352,7 +31447,7 @@
       <c r="T79" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U79" s="164" t="s">
+      <c r="U79" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V79" s="105"/>
@@ -31915,7 +32010,7 @@
       <c r="T86" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U86" s="164" t="s">
+      <c r="U86" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V86" s="105"/>
@@ -32474,7 +32569,7 @@
       <c r="T93" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U93" s="164" t="s">
+      <c r="U93" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V93" s="105"/>
@@ -32885,7 +32980,7 @@
       <c r="T98" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U98" s="164" t="s">
+      <c r="U98" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V98" s="105"/>
@@ -33456,7 +33551,7 @@
       <c r="T105" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U105" s="164" t="s">
+      <c r="U105" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V105" s="105"/>
@@ -34027,7 +34122,7 @@
       <c r="T112" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U112" s="164" t="s">
+      <c r="U112" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V112" s="105"/>
@@ -34451,7 +34546,7 @@
       <c r="T117" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U117" s="164" t="s">
+      <c r="U117" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V117" s="105"/>
@@ -34890,7 +34985,7 @@
       <c r="T122" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U122" s="164" t="s">
+      <c r="U122" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V122" s="105"/>
@@ -35301,7 +35396,7 @@
       <c r="T127" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="U127" s="164" t="s">
+      <c r="U127" s="165" t="s">
         <v>76</v>
       </c>
       <c r="V127" s="105"/>
@@ -42718,10 +42813,10 @@
       <c r="R225" s="105" t="s">
         <v>86</v>
       </c>
-      <c r="S225" s="166" t="s">
+      <c r="S225" s="164" t="s">
         <v>344</v>
       </c>
-      <c r="T225" s="166" t="s">
+      <c r="T225" s="164" t="s">
         <v>345</v>
       </c>
       <c r="U225" s="105"/>
@@ -45490,21 +45585,45 @@
     </row>
   </sheetData>
   <mergeCells count="70">
-    <mergeCell ref="S23:S25"/>
-    <mergeCell ref="S225:S230"/>
-    <mergeCell ref="S122:S124"/>
-    <mergeCell ref="U57:U59"/>
-    <mergeCell ref="S38:S40"/>
-    <mergeCell ref="U62:U64"/>
-    <mergeCell ref="T117:T119"/>
-    <mergeCell ref="S112:S114"/>
-    <mergeCell ref="S57:S59"/>
-    <mergeCell ref="S28:S30"/>
-    <mergeCell ref="U28:U30"/>
-    <mergeCell ref="U93:U95"/>
-    <mergeCell ref="S127:S129"/>
-    <mergeCell ref="T225:T230"/>
-    <mergeCell ref="S74:S76"/>
+    <mergeCell ref="S242:S245"/>
+    <mergeCell ref="U33:U35"/>
+    <mergeCell ref="U98:U100"/>
+    <mergeCell ref="U67:U69"/>
+    <mergeCell ref="U117:U119"/>
+    <mergeCell ref="U52:U54"/>
+    <mergeCell ref="U79:U81"/>
+    <mergeCell ref="U38:U40"/>
+    <mergeCell ref="U112:U114"/>
+    <mergeCell ref="T122:T124"/>
+    <mergeCell ref="S67:S69"/>
+    <mergeCell ref="T67:T69"/>
+    <mergeCell ref="T127:T129"/>
+    <mergeCell ref="S18:S20"/>
+    <mergeCell ref="U122:U124"/>
+    <mergeCell ref="U18:U20"/>
+    <mergeCell ref="T79:T81"/>
+    <mergeCell ref="U127:U129"/>
+    <mergeCell ref="U23:U25"/>
+    <mergeCell ref="T105:T107"/>
+    <mergeCell ref="T52:T54"/>
+    <mergeCell ref="T86:T88"/>
+    <mergeCell ref="S93:S95"/>
+    <mergeCell ref="S62:S64"/>
+    <mergeCell ref="S33:S35"/>
+    <mergeCell ref="T23:T25"/>
+    <mergeCell ref="T28:T30"/>
+    <mergeCell ref="S45:S47"/>
+    <mergeCell ref="S79:S81"/>
+    <mergeCell ref="U3:U4"/>
+    <mergeCell ref="T57:T59"/>
+    <mergeCell ref="T33:T35"/>
+    <mergeCell ref="T18:T20"/>
+    <mergeCell ref="T98:T100"/>
+    <mergeCell ref="T45:T47"/>
+    <mergeCell ref="U5:U6"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="T5:T6"/>
+    <mergeCell ref="T11:T13"/>
     <mergeCell ref="S11:S13"/>
     <mergeCell ref="T74:T76"/>
     <mergeCell ref="T112:T114"/>
@@ -45521,45 +45640,21 @@
     <mergeCell ref="S52:S54"/>
     <mergeCell ref="S86:S88"/>
     <mergeCell ref="U86:U88"/>
-    <mergeCell ref="U3:U4"/>
-    <mergeCell ref="T57:T59"/>
-    <mergeCell ref="T33:T35"/>
-    <mergeCell ref="T18:T20"/>
-    <mergeCell ref="T98:T100"/>
-    <mergeCell ref="T45:T47"/>
-    <mergeCell ref="U5:U6"/>
-    <mergeCell ref="T3:T4"/>
-    <mergeCell ref="T5:T6"/>
-    <mergeCell ref="T11:T13"/>
-    <mergeCell ref="S18:S20"/>
-    <mergeCell ref="U122:U124"/>
-    <mergeCell ref="U18:U20"/>
-    <mergeCell ref="T79:T81"/>
-    <mergeCell ref="U127:U129"/>
-    <mergeCell ref="U23:U25"/>
-    <mergeCell ref="T105:T107"/>
-    <mergeCell ref="T52:T54"/>
-    <mergeCell ref="T86:T88"/>
-    <mergeCell ref="S93:S95"/>
-    <mergeCell ref="S62:S64"/>
-    <mergeCell ref="S33:S35"/>
-    <mergeCell ref="T23:T25"/>
-    <mergeCell ref="T28:T30"/>
-    <mergeCell ref="S45:S47"/>
-    <mergeCell ref="S79:S81"/>
-    <mergeCell ref="S242:S245"/>
-    <mergeCell ref="U33:U35"/>
-    <mergeCell ref="U98:U100"/>
-    <mergeCell ref="U67:U69"/>
-    <mergeCell ref="U117:U119"/>
-    <mergeCell ref="U52:U54"/>
-    <mergeCell ref="U79:U81"/>
-    <mergeCell ref="U38:U40"/>
-    <mergeCell ref="U112:U114"/>
-    <mergeCell ref="T122:T124"/>
-    <mergeCell ref="S67:S69"/>
-    <mergeCell ref="T67:T69"/>
-    <mergeCell ref="T127:T129"/>
+    <mergeCell ref="S23:S25"/>
+    <mergeCell ref="S225:S230"/>
+    <mergeCell ref="S122:S124"/>
+    <mergeCell ref="U57:U59"/>
+    <mergeCell ref="S38:S40"/>
+    <mergeCell ref="U62:U64"/>
+    <mergeCell ref="T117:T119"/>
+    <mergeCell ref="S112:S114"/>
+    <mergeCell ref="S57:S59"/>
+    <mergeCell ref="S28:S30"/>
+    <mergeCell ref="U28:U30"/>
+    <mergeCell ref="U93:U95"/>
+    <mergeCell ref="S127:S129"/>
+    <mergeCell ref="T225:T230"/>
+    <mergeCell ref="S74:S76"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update used fuel storage cost accounts
</commit_message>
<xml_diff>
--- a/cost/Cost_Database.xlsx
+++ b/cost/Cost_Database.xlsx
@@ -34887,20 +34887,25 @@
       <c r="I28" s="93"/>
       <c r="J28" s="141"/>
       <c r="K28" s="120">
-        <f>493700000/(40000*1000)</f>
-        <v>12.342499999999999</v>
-      </c>
-      <c r="L28" s="100" t="s">
-        <v>186</v>
-      </c>
-      <c r="M28" s="155" t="s">
-        <v>721</v>
+        <v>6171250</v>
+      </c>
+      <c r="L28" s="100" t="inlineStr">
+        <is>
+          <t>$/(reactors/year)</t>
+        </is>
+      </c>
+      <c r="M28" s="155" t="inlineStr">
+        <is>
+          <t>Servicing Rate</t>
+        </is>
       </c>
       <c r="N28" s="121">
         <v>1</v>
       </c>
-      <c r="O28" s="100" t="s">
-        <v>188</v>
+      <c r="O28" s="100" t="inlineStr">
+        <is>
+          <t>reactors/year</t>
+        </is>
       </c>
       <c r="P28" s="123">
         <v>1</v>
@@ -34935,11 +34940,11 @@
       </c>
       <c r="AA28" s="147">
         <f t="shared" si="24"/>
-        <v>11.10825</v>
+        <v>5554125</v>
       </c>
       <c r="AB28" s="147">
         <f t="shared" si="25"/>
-        <v>16.045249999999999</v>
+        <v>8022625</v>
       </c>
       <c r="AC28" s="145" t="s">
         <v>44</v>
@@ -39608,67 +39613,71 @@
         <v>48</v>
       </c>
     </row>
-    <row r="91" spans="1:33" ht="57" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:33" ht="43" x14ac:dyDescent="0.2">
       <c r="A91" s="90">
-        <v>747.3</v>
+        <v>747.24</v>
       </c>
       <c r="B91" s="92">
-        <f t="shared" si="43"/>
-        <v>3</v>
-      </c>
-      <c r="C91" s="109" t="s">
-        <v>694</v>
+        <f>IF(ISNUMBER(A91),IF(AND(A91=INT(A91),MOD(A91,10)=0),0,IF(AND(A91=INT(A91),LEN(A91)=2),1,IF(AND(A91=INT(A91),LEN(A91)=3),2,LEN(A91)-FIND(".",A91)+2))),"")</f>
+        <v>4</v>
+      </c>
+      <c r="C91" s="109" t="inlineStr">
+        <is>
+          <t>Used Fuel Storage Additional Overpacks</t>
+        </is>
       </c>
       <c r="D91" s="93" t="str">
-        <f t="shared" si="44"/>
-        <v xml:space="preserve">                  Annualized Helium Replenishment</v>
+        <f>REPT("   ",B91*2)&amp;C91</f>
+        <v xml:space="preserve">                        Used Fuel Storage Additional Overpacks</v>
       </c>
       <c r="E91" s="93" t="s">
         <v>35</v>
       </c>
-      <c r="F91" s="189" t="s">
-        <v>606</v>
-      </c>
-      <c r="G91" s="94">
-        <v>1</v>
-      </c>
+      <c r="F91" s="93"/>
+      <c r="G91" s="94"/>
       <c r="H91" s="93"/>
       <c r="I91" s="93"/>
       <c r="J91" s="120"/>
       <c r="K91" s="99">
-        <v>170</v>
-      </c>
-      <c r="L91" s="103" t="s">
-        <v>186</v>
-      </c>
-      <c r="M91" s="110" t="s">
-        <v>794</v>
-      </c>
-      <c r="N91" s="103"/>
-      <c r="O91" s="103" t="s">
-        <v>188</v>
-      </c>
-      <c r="P91" s="101"/>
+        <v>200000</v>
+      </c>
+      <c r="L91" s="103" t="inlineStr">
+        <is>
+          <t>$/(reactors/year)</t>
+        </is>
+      </c>
+      <c r="M91" s="110" t="inlineStr">
+        <is>
+          <t>Servicing Rate</t>
+        </is>
+      </c>
+      <c r="N91" s="103">
+        <v>1</v>
+      </c>
+      <c r="O91" s="103" t="inlineStr">
+        <is>
+          <t>reactors/year</t>
+        </is>
+      </c>
+      <c r="P91" s="101">
+        <v>1</v>
+      </c>
       <c r="Q91" s="101">
-        <v>2024</v>
-      </c>
-      <c r="R91" s="103" t="s">
-        <v>153</v>
-      </c>
-      <c r="S91" s="110" t="s">
-        <v>305</v>
-      </c>
-      <c r="T91" s="111" t="s">
-        <v>305</v>
-      </c>
-      <c r="U91" s="182" t="s">
-        <v>306</v>
-      </c>
-      <c r="V91" s="103" t="s">
-        <v>307</v>
-      </c>
-      <c r="W91" s="96" t="s">
-        <v>43</v>
+        <v>2009</v>
+      </c>
+      <c r="R91" s="103" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="S91" s="110"/>
+      <c r="T91" s="111"/>
+      <c r="U91" s="182"/>
+      <c r="V91" s="103"/>
+      <c r="W91" s="96" t="inlineStr">
+        <is>
+          <t>No Learning</t>
+        </is>
       </c>
       <c r="X91" s="104">
         <v>0</v>
@@ -39676,92 +39685,148 @@
       <c r="Y91" s="104">
         <v>0</v>
       </c>
-      <c r="Z91" s="96" t="s">
-        <v>44</v>
+      <c r="Z91" s="96" t="inlineStr">
+        <is>
+          <t>Lognormal</t>
+        </is>
       </c>
       <c r="AA91" s="97">
-        <f>0.9*K91</f>
-        <v>153</v>
+        <f>0.8*K91</f>
+        <v>160000</v>
       </c>
       <c r="AB91" s="97">
-        <f>1.3*K91</f>
-        <v>221</v>
-      </c>
-      <c r="AC91" s="96" t="s">
-        <v>44</v>
-      </c>
-      <c r="AD91" s="97" t="s">
-        <v>45</v>
-      </c>
-      <c r="AE91" s="97" t="s">
-        <v>46</v>
-      </c>
-      <c r="AF91" s="97" t="s">
-        <v>47</v>
-      </c>
-      <c r="AG91" s="96" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="92" spans="1:33" ht="15" x14ac:dyDescent="0.2">
+        <f>2*K91</f>
+        <v>400000</v>
+      </c>
+      <c r="AC91" s="96" t="inlineStr">
+        <is>
+          <t>Lognormal</t>
+        </is>
+      </c>
+      <c r="AD91" s="97">
+        <v>0.1</v>
+      </c>
+      <c r="AE91" s="97">
+        <v>1</v>
+      </c>
+      <c r="AF91" s="97">
+        <v>0</v>
+      </c>
+      <c r="AG91" s="96" t="inlineStr">
+        <is>
+          <t>Truncated Normal</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" spans="1:33" ht="57" x14ac:dyDescent="0.2">
       <c r="A92" s="90">
-        <v>747.4</v>
+        <v>747.3</v>
       </c>
       <c r="B92" s="92">
         <f t="shared" si="43"/>
         <v>3</v>
       </c>
       <c r="C92" s="109" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="D92" s="93" t="str">
         <f t="shared" si="44"/>
-        <v xml:space="preserve">                  Annualized Other Supplies and Utilities</v>
-      </c>
-      <c r="E92" s="93"/>
-      <c r="F92" s="93"/>
-      <c r="G92" s="94"/>
+        <v xml:space="preserve">                  Annualized Helium Replenishment</v>
+      </c>
+      <c r="E92" s="93" t="s">
+        <v>35</v>
+      </c>
+      <c r="F92" s="189" t="s">
+        <v>606</v>
+      </c>
+      <c r="G92" s="94">
+        <v>1</v>
+      </c>
       <c r="H92" s="93"/>
       <c r="I92" s="93"/>
-      <c r="J92" s="181"/>
-      <c r="K92" s="99"/>
-      <c r="L92" s="103"/>
-      <c r="M92" s="110"/>
+      <c r="J92" s="120"/>
+      <c r="K92" s="99">
+        <v>170</v>
+      </c>
+      <c r="L92" s="103" t="s">
+        <v>186</v>
+      </c>
+      <c r="M92" s="110" t="s">
+        <v>794</v>
+      </c>
       <c r="N92" s="103"/>
-      <c r="O92" s="103"/>
+      <c r="O92" s="103" t="s">
+        <v>188</v>
+      </c>
       <c r="P92" s="101"/>
-      <c r="Q92" s="101"/>
-      <c r="R92" s="103"/>
-      <c r="S92" s="110"/>
-      <c r="T92" s="111"/>
-      <c r="U92" s="182"/>
-      <c r="V92" s="103"/>
-      <c r="W92" s="96"/>
-      <c r="X92" s="104"/>
-      <c r="Y92" s="104"/>
-      <c r="Z92" s="96"/>
-      <c r="AA92" s="97"/>
-      <c r="AB92" s="97"/>
-      <c r="AC92" s="96"/>
-      <c r="AD92" s="97"/>
-      <c r="AE92" s="97"/>
-      <c r="AF92" s="97"/>
-      <c r="AG92" s="96"/>
+      <c r="Q92" s="101">
+        <v>2024</v>
+      </c>
+      <c r="R92" s="103" t="s">
+        <v>153</v>
+      </c>
+      <c r="S92" s="110" t="s">
+        <v>305</v>
+      </c>
+      <c r="T92" s="111" t="s">
+        <v>305</v>
+      </c>
+      <c r="U92" s="182" t="s">
+        <v>306</v>
+      </c>
+      <c r="V92" s="103" t="s">
+        <v>307</v>
+      </c>
+      <c r="W92" s="96" t="s">
+        <v>43</v>
+      </c>
+      <c r="X92" s="104">
+        <v>0</v>
+      </c>
+      <c r="Y92" s="104">
+        <v>0</v>
+      </c>
+      <c r="Z92" s="96" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA92" s="97">
+        <f>0.9*K91</f>
+        <v>153</v>
+      </c>
+      <c r="AB92" s="97">
+        <f>1.3*K91</f>
+        <v>221</v>
+      </c>
+      <c r="AC92" s="96" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD92" s="97" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE92" s="97" t="s">
+        <v>46</v>
+      </c>
+      <c r="AF92" s="97" t="s">
+        <v>47</v>
+      </c>
+      <c r="AG92" s="96" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="93" spans="1:33" ht="15" x14ac:dyDescent="0.2">
       <c r="A93" s="90">
-        <v>747.5</v>
+        <v>747.4</v>
       </c>
       <c r="B93" s="92">
         <f t="shared" si="43"/>
         <v>3</v>
       </c>
       <c r="C93" s="109" t="s">
-        <v>795</v>
+        <v>696</v>
       </c>
       <c r="D93" s="93" t="str">
         <f t="shared" si="44"/>
-        <v xml:space="preserve">                  Servicing Vehicle O&amp;M</v>
+        <v xml:space="preserve">                  Annualized Other Supplies and Utilities</v>
       </c>
       <c r="E93" s="93"/>
       <c r="F93" s="93"/>
@@ -39793,110 +39858,71 @@
       <c r="AF93" s="97"/>
       <c r="AG93" s="96"/>
     </row>
-    <row r="94" spans="1:33" ht="29" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:33" ht="15" x14ac:dyDescent="0.2">
       <c r="A94" s="90">
-        <v>747.51</v>
+        <v>747.5</v>
       </c>
       <c r="B94" s="92">
         <f t="shared" si="43"/>
-        <v>4</v>
-      </c>
-      <c r="C94" s="168" t="s">
-        <v>796</v>
+        <v>3</v>
+      </c>
+      <c r="C94" s="109" t="s">
+        <v>795</v>
       </c>
       <c r="D94" s="93" t="str">
         <f t="shared" si="44"/>
-        <v xml:space="preserve">                        Reactor Transport Vehicles O&amp;M</v>
-      </c>
-      <c r="E94" s="93" t="s">
-        <v>35</v>
-      </c>
-      <c r="F94" s="93" t="s">
-        <v>761</v>
-      </c>
-      <c r="G94" s="94">
-        <v>1</v>
-      </c>
+        <v xml:space="preserve">                  Servicing Vehicle O&amp;M</v>
+      </c>
+      <c r="E94" s="93"/>
+      <c r="F94" s="93"/>
+      <c r="G94" s="94"/>
       <c r="H94" s="93"/>
       <c r="I94" s="93"/>
-      <c r="J94" s="181">
-        <f>36*200000+1000000</f>
-        <v>8200000</v>
-      </c>
+      <c r="J94" s="181"/>
       <c r="K94" s="99"/>
       <c r="L94" s="103"/>
       <c r="M94" s="110"/>
       <c r="N94" s="103"/>
       <c r="O94" s="103"/>
       <c r="P94" s="101"/>
-      <c r="Q94" s="101">
-        <v>2024</v>
-      </c>
-      <c r="R94" s="103" t="s">
-        <v>73</v>
-      </c>
+      <c r="Q94" s="101"/>
+      <c r="R94" s="103"/>
       <c r="S94" s="110"/>
       <c r="T94" s="111"/>
       <c r="U94" s="182"/>
       <c r="V94" s="103"/>
-      <c r="W94" s="96" t="s">
-        <v>43</v>
-      </c>
-      <c r="X94" s="104">
-        <f t="shared" ref="X94:X97" si="83">0.9*$J94</f>
-        <v>7380000</v>
-      </c>
-      <c r="Y94" s="104">
-        <f t="shared" ref="Y94:Y97" si="84">1.5*J94</f>
-        <v>12300000</v>
-      </c>
-      <c r="Z94" s="96" t="s">
-        <v>44</v>
-      </c>
-      <c r="AA94" s="97">
-        <f t="shared" ref="AA94:AA97" si="85">0.9*K94</f>
-        <v>0</v>
-      </c>
-      <c r="AB94" s="97">
-        <f t="shared" ref="AB94:AB97" si="86">1.3*K94</f>
-        <v>0</v>
-      </c>
-      <c r="AC94" s="96" t="s">
-        <v>44</v>
-      </c>
-      <c r="AD94" s="97" t="s">
-        <v>45</v>
-      </c>
-      <c r="AE94" s="97" t="s">
-        <v>46</v>
-      </c>
-      <c r="AF94" s="97" t="s">
-        <v>47</v>
-      </c>
-      <c r="AG94" s="96" t="s">
-        <v>48</v>
-      </c>
+      <c r="W94" s="96"/>
+      <c r="X94" s="104"/>
+      <c r="Y94" s="104"/>
+      <c r="Z94" s="96"/>
+      <c r="AA94" s="97"/>
+      <c r="AB94" s="97"/>
+      <c r="AC94" s="96"/>
+      <c r="AD94" s="97"/>
+      <c r="AE94" s="97"/>
+      <c r="AF94" s="97"/>
+      <c r="AG94" s="96"/>
     </row>
     <row r="95" spans="1:33" ht="29" x14ac:dyDescent="0.2">
       <c r="A95" s="90">
-        <v>747.52</v>
+        <v>747.51</v>
       </c>
       <c r="B95" s="92">
         <f t="shared" si="43"/>
         <v>4</v>
       </c>
       <c r="C95" s="168" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="D95" s="93" t="str">
         <f t="shared" si="44"/>
-        <v xml:space="preserve">                        Helium Transport Trucks O&amp;M</v>
+        <v xml:space="preserve">                        Reactor Transport Vehicles O&amp;M</v>
       </c>
       <c r="E95" s="93" t="s">
         <v>35</v>
       </c>
       <c r="F95" s="93" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="G95" s="94">
         <v>1</v>
@@ -39904,8 +39930,8 @@
       <c r="H95" s="93"/>
       <c r="I95" s="93"/>
       <c r="J95" s="181">
-        <f>4*200000+500000</f>
-        <v>1300000</v>
+        <f>36*200000+1000000</f>
+        <v>8200000</v>
       </c>
       <c r="K95" s="99"/>
       <c r="L95" s="103"/>
@@ -39927,22 +39953,22 @@
         <v>43</v>
       </c>
       <c r="X95" s="104">
-        <f t="shared" si="83"/>
-        <v>1170000</v>
+        <f t="shared" ref="X94:X98" si="83">0.9*$J94</f>
+        <v>7380000</v>
       </c>
       <c r="Y95" s="104">
-        <f t="shared" si="84"/>
-        <v>1950000</v>
+        <f t="shared" ref="Y94:Y98" si="84">1.5*J94</f>
+        <v>12300000</v>
       </c>
       <c r="Z95" s="96" t="s">
         <v>44</v>
       </c>
       <c r="AA95" s="97">
-        <f t="shared" si="85"/>
+        <f t="shared" ref="AA94:AA98" si="85">0.9*K94</f>
         <v>0</v>
       </c>
       <c r="AB95" s="97">
-        <f t="shared" si="86"/>
+        <f t="shared" ref="AB94:AB98" si="86">1.3*K94</f>
         <v>0</v>
       </c>
       <c r="AC95" s="96" t="s">
@@ -39963,24 +39989,24 @@
     </row>
     <row r="96" spans="1:33" ht="29" x14ac:dyDescent="0.2">
       <c r="A96" s="90">
-        <v>747.53</v>
+        <v>747.52</v>
       </c>
       <c r="B96" s="92">
         <f t="shared" si="43"/>
         <v>4</v>
       </c>
       <c r="C96" s="168" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="D96" s="93" t="str">
         <f t="shared" si="44"/>
-        <v xml:space="preserve">                        Water Tanker Trucks O&amp;M</v>
+        <v xml:space="preserve">                        Helium Transport Trucks O&amp;M</v>
       </c>
       <c r="E96" s="93" t="s">
         <v>35</v>
       </c>
       <c r="F96" s="93" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="G96" s="94">
         <v>1</v>
@@ -39988,8 +40014,8 @@
       <c r="H96" s="93"/>
       <c r="I96" s="93"/>
       <c r="J96" s="181">
-        <f>4*200000+400000</f>
-        <v>1200000</v>
+        <f>4*200000+500000</f>
+        <v>1300000</v>
       </c>
       <c r="K96" s="99"/>
       <c r="L96" s="103"/>
@@ -40012,11 +40038,11 @@
       </c>
       <c r="X96" s="104">
         <f t="shared" si="83"/>
-        <v>1080000</v>
+        <v>1170000</v>
       </c>
       <c r="Y96" s="104">
         <f t="shared" si="84"/>
-        <v>1800000</v>
+        <v>1950000</v>
       </c>
       <c r="Z96" s="96" t="s">
         <v>44</v>
@@ -40047,24 +40073,24 @@
     </row>
     <row r="97" spans="1:33" ht="29" x14ac:dyDescent="0.2">
       <c r="A97" s="90">
-        <v>747.54</v>
+        <v>747.53</v>
       </c>
       <c r="B97" s="92">
         <f t="shared" si="43"/>
         <v>4</v>
       </c>
       <c r="C97" s="168" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="D97" s="93" t="str">
         <f t="shared" si="44"/>
-        <v xml:space="preserve">                        Maintenance Trucks O&amp;M</v>
+        <v xml:space="preserve">                        Water Tanker Trucks O&amp;M</v>
       </c>
       <c r="E97" s="93" t="s">
         <v>35</v>
       </c>
       <c r="F97" s="93" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="G97" s="94">
         <v>1</v>
@@ -40072,8 +40098,8 @@
       <c r="H97" s="93"/>
       <c r="I97" s="93"/>
       <c r="J97" s="181">
-        <f>10*2*200000+1000000</f>
-        <v>5000000</v>
+        <f>4*200000+400000</f>
+        <v>1200000</v>
       </c>
       <c r="K97" s="99"/>
       <c r="L97" s="103"/>
@@ -40096,11 +40122,11 @@
       </c>
       <c r="X97" s="104">
         <f t="shared" si="83"/>
-        <v>4500000</v>
+        <v>1080000</v>
       </c>
       <c r="Y97" s="104">
         <f t="shared" si="84"/>
-        <v>7500000</v>
+        <v>1800000</v>
       </c>
       <c r="Z97" s="96" t="s">
         <v>44</v>
@@ -40129,65 +40155,104 @@
         <v>48</v>
       </c>
     </row>
-    <row r="98" spans="1:33" ht="15" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:33" ht="29" x14ac:dyDescent="0.2">
       <c r="A98" s="90">
-        <v>75</v>
+        <v>747.54</v>
       </c>
       <c r="B98" s="92">
         <f t="shared" si="43"/>
-        <v>1</v>
-      </c>
-      <c r="C98" s="109" t="s">
-        <v>402</v>
+        <v>4</v>
+      </c>
+      <c r="C98" s="168" t="s">
+        <v>799</v>
       </c>
       <c r="D98" s="93" t="str">
         <f t="shared" si="44"/>
-        <v xml:space="preserve">      Capital Plant Expenditures</v>
-      </c>
-      <c r="E98" s="93"/>
-      <c r="F98" s="93"/>
-      <c r="G98" s="113"/>
-      <c r="H98" s="114"/>
-      <c r="I98" s="114"/>
-      <c r="J98" s="192"/>
-      <c r="K98" s="115"/>
-      <c r="L98" s="116"/>
-      <c r="M98" s="116"/>
-      <c r="N98" s="116"/>
-      <c r="O98" s="116"/>
-      <c r="P98" s="115"/>
-      <c r="Q98" s="116"/>
-      <c r="R98" s="116"/>
-      <c r="S98" s="116"/>
-      <c r="T98" s="116"/>
-      <c r="U98" s="116"/>
-      <c r="V98" s="116"/>
-      <c r="W98" s="116"/>
-      <c r="X98" s="115"/>
-      <c r="Y98" s="115"/>
-      <c r="Z98" s="116"/>
-      <c r="AA98" s="115"/>
-      <c r="AB98" s="115"/>
-      <c r="AC98" s="116"/>
-      <c r="AD98" s="115"/>
-      <c r="AE98" s="115"/>
-      <c r="AF98" s="115"/>
-      <c r="AG98" s="116"/>
+        <v xml:space="preserve">                        Maintenance Trucks O&amp;M</v>
+      </c>
+      <c r="E98" s="93" t="s">
+        <v>35</v>
+      </c>
+      <c r="F98" s="93" t="s">
+        <v>767</v>
+      </c>
+      <c r="G98" s="94">
+        <v>1</v>
+      </c>
+      <c r="H98" s="93"/>
+      <c r="I98" s="93"/>
+      <c r="J98" s="181">
+        <f>10*2*200000+1000000</f>
+        <v>5000000</v>
+      </c>
+      <c r="K98" s="99"/>
+      <c r="L98" s="103"/>
+      <c r="M98" s="110"/>
+      <c r="N98" s="103"/>
+      <c r="O98" s="103"/>
+      <c r="P98" s="101"/>
+      <c r="Q98" s="101">
+        <v>2024</v>
+      </c>
+      <c r="R98" s="103" t="s">
+        <v>73</v>
+      </c>
+      <c r="S98" s="110"/>
+      <c r="T98" s="111"/>
+      <c r="U98" s="182"/>
+      <c r="V98" s="103"/>
+      <c r="W98" s="96" t="s">
+        <v>43</v>
+      </c>
+      <c r="X98" s="104">
+        <f t="shared" si="83"/>
+        <v>4500000</v>
+      </c>
+      <c r="Y98" s="104">
+        <f t="shared" si="84"/>
+        <v>7500000</v>
+      </c>
+      <c r="Z98" s="96" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA98" s="97">
+        <f t="shared" si="85"/>
+        <v>0</v>
+      </c>
+      <c r="AB98" s="97">
+        <f t="shared" si="86"/>
+        <v>0</v>
+      </c>
+      <c r="AC98" s="96" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD98" s="97" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE98" s="97" t="s">
+        <v>46</v>
+      </c>
+      <c r="AF98" s="97" t="s">
+        <v>47</v>
+      </c>
+      <c r="AG98" s="96" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="99" spans="1:33" ht="15" x14ac:dyDescent="0.2">
       <c r="A99" s="90">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B99" s="92">
         <f t="shared" si="43"/>
         <v>1</v>
       </c>
       <c r="C99" s="109" t="s">
-        <v>420</v>
+        <v>402</v>
       </c>
       <c r="D99" s="93" t="str">
         <f t="shared" si="44"/>
-        <v xml:space="preserve">      Annualized Decommissioning Cost</v>
+        <v xml:space="preserve">      Capital Plant Expenditures</v>
       </c>
       <c r="E99" s="93"/>
       <c r="F99" s="93"/>
@@ -40218,6 +40283,51 @@
       <c r="AE99" s="115"/>
       <c r="AF99" s="115"/>
       <c r="AG99" s="116"/>
+    </row>
+    <row r="100" spans="1:33" ht="15" x14ac:dyDescent="0.2">
+      <c r="A100" s="90">
+        <v>78</v>
+      </c>
+      <c r="B100" s="92">
+        <f t="shared" si="43"/>
+        <v>1</v>
+      </c>
+      <c r="C100" s="109" t="s">
+        <v>420</v>
+      </c>
+      <c r="D100" s="93" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">      Annualized Decommissioning Cost</v>
+      </c>
+      <c r="E100" s="93"/>
+      <c r="F100" s="93"/>
+      <c r="G100" s="113"/>
+      <c r="H100" s="114"/>
+      <c r="I100" s="114"/>
+      <c r="J100" s="192"/>
+      <c r="K100" s="115"/>
+      <c r="L100" s="116"/>
+      <c r="M100" s="116"/>
+      <c r="N100" s="116"/>
+      <c r="O100" s="116"/>
+      <c r="P100" s="115"/>
+      <c r="Q100" s="116"/>
+      <c r="R100" s="116"/>
+      <c r="S100" s="116"/>
+      <c r="T100" s="116"/>
+      <c r="U100" s="116"/>
+      <c r="V100" s="116"/>
+      <c r="W100" s="116"/>
+      <c r="X100" s="115"/>
+      <c r="Y100" s="115"/>
+      <c r="Z100" s="116"/>
+      <c r="AA100" s="115"/>
+      <c r="AB100" s="115"/>
+      <c r="AC100" s="116"/>
+      <c r="AD100" s="115"/>
+      <c r="AE100" s="115"/>
+      <c r="AF100" s="115"/>
+      <c r="AG100" s="116"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -40271,17 +40381,17 @@
       <formula>$B2=3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:AG99">
+  <conditionalFormatting sqref="A2:AG100">
     <cfRule type="expression" dxfId="39" priority="12">
       <formula>$B2=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C94:C97">
+  <conditionalFormatting sqref="C94:C98">
     <cfRule type="expression" dxfId="38" priority="7">
       <formula>$B94=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F94:F97">
+  <conditionalFormatting sqref="F94:F98">
     <cfRule type="expression" dxfId="37" priority="6">
       <formula>$B94=0</formula>
     </cfRule>
@@ -40419,31 +40529,31 @@
       <formula>$B82=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W94:AG97">
+  <conditionalFormatting sqref="W94:AG98">
     <cfRule type="expression" dxfId="3" priority="1">
       <formula>$B94=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X2:Z99">
+  <conditionalFormatting sqref="X2:Z100">
     <cfRule type="expression" dxfId="2" priority="51">
       <formula>AND(ISBLANK($X2),ISBLANK($Y2),ISBLANK($Z2),NOT(ISBLANK($E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA2:AC99">
+  <conditionalFormatting sqref="AA2:AC100">
     <cfRule type="expression" dxfId="1" priority="50">
       <formula>AND(ISBLANK($AA2),ISBLANK($AB2),ISBLANK($AC2),NOT(ISBLANK($E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AD2:AG99">
+  <conditionalFormatting sqref="AD2:AG100">
     <cfRule type="expression" dxfId="0" priority="49">
       <formula>AND(ISBLANK($AD2),ISBLANK($AE2),ISBLANK($AF2),NOT(ISBLANK($E2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E99" xr:uid="{00000000-0002-0000-0600-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E100" xr:uid="{00000000-0002-0000-0600-000000000000}">
       <formula1>"standard, nonstandard"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O99" xr:uid="{00000000-0002-0000-0600-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O100" xr:uid="{00000000-0002-0000-0600-000001000000}">
       <formula1>"acres,MWe,m^3,MWt,Kg,Drums,kW,$,m^2,kg/s,Rx/yr"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R90:R97 R2:R88" xr:uid="{00000000-0002-0000-0600-000002000000}">
@@ -40466,13 +40576,13 @@
     <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K9 K11:K31 K33:K97 N1:N1048576" xr:uid="{00000000-0002-0000-0600-000007000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M272:M282" xr:uid="{00000000-0002-0000-0600-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M272:M283" xr:uid="{00000000-0002-0000-0600-000008000000}">
       <formula1>"Land Area, Power MWe, Excavation Volume,  Reactor Building Slab Roof Volume,	Reactor Building  Basement Volume, Reactor Building  Exterior Walls Volume,		Turbine Building Slab Roof Volume,	Turbine Building  Basement Volume,	Turbine Building  Exterior Wall"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1 L100:L1048576" xr:uid="{00000000-0002-0000-0600-000009000000}">
       <formula1>"$/acres, $/MWe, $/m^3, $/MWt"</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P100:P251" xr:uid="{00000000-0002-0000-0600-00000A000000}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P100:P252" xr:uid="{00000000-0002-0000-0600-00000A000000}">
       <formula1>0</formula1>
       <formula2>2</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Update fleet replacement schedules
</commit_message>
<xml_diff>
--- a/cost/Cost_Database.xlsx
+++ b/cost/Cost_Database.xlsx
@@ -8553,9 +8553,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AJ196"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AH197"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14" ns3:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.6640625" style="3" customWidth="1"/>
     <col min="2" max="2" width="9.5" style="3" customWidth="1"/>
@@ -8592,7 +8592,7 @@
     <col min="35" max="16384" width="10.6640625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" s="79" customFormat="1" ht="94.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:33" s="79" customFormat="1" ht="94.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A1" s="50" t="s">
         <v>0</v>
       </c>
@@ -8693,7 +8693,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:33" s="7" customFormat="1" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:33" s="7" customFormat="1" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A2" s="37">
         <v>10</v>
       </c>
@@ -8745,7 +8745,7 @@
       <c r="AF2" s="76"/>
       <c r="AG2" s="74"/>
     </row>
-    <row r="3" spans="1:33" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:33" ht="45" customHeight="1" ns3:dyDescent="0.2">
       <c r="A3" s="37">
         <v>11</v>
       </c>
@@ -8843,7 +8843,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A4" s="37">
         <v>12</v>
       </c>
@@ -8938,7 +8938,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:33" ht="113.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:33" ht="113.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A5" s="37">
         <v>13</v>
       </c>
@@ -9031,7 +9031,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A6" s="37">
         <v>14</v>
       </c>
@@ -9121,7 +9121,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:33" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:33" ht="42.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A7" s="37">
         <v>15</v>
       </c>
@@ -9216,7 +9216,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A8" s="50">
         <v>20</v>
       </c>
@@ -9268,7 +9268,7 @@
       <c r="AF8" s="76"/>
       <c r="AG8" s="74"/>
     </row>
-    <row r="9" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A9" s="37">
         <v>21</v>
       </c>
@@ -9320,7 +9320,7 @@
       <c r="AF9" s="76"/>
       <c r="AG9" s="74"/>
     </row>
-    <row r="10" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A10" s="53">
         <v>211</v>
       </c>
@@ -9372,7 +9372,7 @@
       <c r="AF10" s="76"/>
       <c r="AG10" s="74"/>
     </row>
-    <row r="11" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A11" s="54">
         <v>211.1</v>
       </c>
@@ -9471,7 +9471,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="12" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A12" s="53">
         <v>211.2</v>
       </c>
@@ -9564,7 +9564,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:33" ht="147.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:33" ht="147.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A13" s="53">
         <v>211.3</v>
       </c>
@@ -9657,7 +9657,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:33" s="213" customFormat="1" ht="43" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:33" s="213" customFormat="1" ht="43" ns3:dyDescent="0.2">
       <c r="A14" s="207">
         <v>211.4</v>
       </c>
@@ -9752,7 +9752,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:33" s="213" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:33" s="213" customFormat="1" ht="15" ns3:dyDescent="0.2">
       <c r="A15" s="207">
         <v>211.9</v>
       </c>
@@ -9797,7 +9797,7 @@
       <c r="AF15" s="76"/>
       <c r="AG15" s="74"/>
     </row>
-    <row r="16" spans="1:33" s="213" customFormat="1" ht="43" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:33" s="213" customFormat="1" ht="43" ns3:dyDescent="0.2">
       <c r="A16" s="207">
         <v>211.91</v>
       </c>
@@ -9885,7 +9885,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:33" s="213" customFormat="1" ht="43" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:33" s="213" customFormat="1" ht="43" ns3:dyDescent="0.2">
       <c r="A17" s="207">
         <v>211.92</v>
       </c>
@@ -9973,7 +9973,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="18" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A18" s="53">
         <v>212</v>
       </c>
@@ -10018,7 +10018,7 @@
       <c r="AF18" s="76"/>
       <c r="AG18" s="74"/>
     </row>
-    <row r="19" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A19" s="53">
         <v>212.1</v>
       </c>
@@ -10110,7 +10110,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A20" s="53">
         <v>212.2</v>
       </c>
@@ -10196,7 +10196,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="1:33" ht="76.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:33" ht="76.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A21" s="53">
         <v>212.3</v>
       </c>
@@ -10282,7 +10282,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:33" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:33" ht="101.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A22" s="53">
         <v>212.4</v>
       </c>
@@ -10378,7 +10378,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:33" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:33" ht="101.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A23" s="53">
         <v>212.5</v>
       </c>
@@ -10474,7 +10474,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="24" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A24" s="53">
         <v>213</v>
       </c>
@@ -10519,7 +10519,7 @@
       <c r="AF24" s="76"/>
       <c r="AG24" s="74"/>
     </row>
-    <row r="25" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A25" s="53">
         <v>213.1</v>
       </c>
@@ -10564,7 +10564,7 @@
       <c r="AF25" s="76"/>
       <c r="AG25" s="74"/>
     </row>
-    <row r="26" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A26" s="53">
         <v>213.11</v>
       </c>
@@ -10656,7 +10656,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="27" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A27" s="53">
         <v>213.12</v>
       </c>
@@ -10742,7 +10742,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="28" spans="1:33" ht="76.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:33" ht="76.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A28" s="53">
         <v>213.13</v>
       </c>
@@ -10828,7 +10828,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="29" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A29" s="53">
         <v>213.2</v>
       </c>
@@ -10873,7 +10873,7 @@
       <c r="AF29" s="76"/>
       <c r="AG29" s="74"/>
     </row>
-    <row r="30" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A30" s="53">
         <v>213.21</v>
       </c>
@@ -10965,7 +10965,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="31" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A31" s="53">
         <v>213.22</v>
       </c>
@@ -11051,7 +11051,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="32" spans="1:33" ht="76.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:33" ht="76.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A32" s="53">
         <v>213.23</v>
       </c>
@@ -11137,7 +11137,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="33" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A33" s="53">
         <v>213.3</v>
       </c>
@@ -11186,7 +11186,7 @@
       <c r="AF33" s="76"/>
       <c r="AG33" s="74"/>
     </row>
-    <row r="34" spans="1:33" ht="76.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:33" ht="76.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A34" s="53">
         <v>213.31</v>
       </c>
@@ -11282,7 +11282,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="35" spans="1:33" ht="76.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:33" ht="76.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A35" s="53">
         <v>213.32</v>
       </c>
@@ -11372,7 +11372,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="36" spans="1:33" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:33" ht="101.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A36" s="53">
         <v>213.33</v>
       </c>
@@ -11462,7 +11462,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="37" spans="1:33" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:33" ht="101.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A37" s="53">
         <v>213.34</v>
       </c>
@@ -11562,7 +11562,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="38" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A38" s="53">
         <v>214</v>
       </c>
@@ -11607,7 +11607,7 @@
       <c r="AF38" s="76"/>
       <c r="AG38" s="74"/>
     </row>
-    <row r="39" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A39" s="53">
         <v>214.1</v>
       </c>
@@ -11652,7 +11652,7 @@
       <c r="AF39" s="76"/>
       <c r="AG39" s="74"/>
     </row>
-    <row r="40" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A40" s="53">
         <v>214.11</v>
       </c>
@@ -11697,7 +11697,7 @@
       <c r="AF40" s="76"/>
       <c r="AG40" s="74"/>
     </row>
-    <row r="41" spans="1:33" s="33" customFormat="1" ht="49.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:33" s="33" customFormat="1" ht="49.75" customHeight="1" ns3:dyDescent="0.15">
       <c r="A41" s="53">
         <v>214.11099999999999</v>
       </c>
@@ -11787,7 +11787,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="42" spans="1:33" s="33" customFormat="1" ht="49.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:33" s="33" customFormat="1" ht="49.75" customHeight="1" ns3:dyDescent="0.15">
       <c r="A42" s="53">
         <v>214.11199999999999</v>
       </c>
@@ -11873,7 +11873,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="43" spans="1:33" s="33" customFormat="1" ht="74.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:33" s="33" customFormat="1" ht="74.75" customHeight="1" ns3:dyDescent="0.15">
       <c r="A43" s="53">
         <v>214.113</v>
       </c>
@@ -11959,7 +11959,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A44" s="53">
         <v>214.12</v>
       </c>
@@ -12004,7 +12004,7 @@
       <c r="AF44" s="76"/>
       <c r="AG44" s="74"/>
     </row>
-    <row r="45" spans="1:33" s="33" customFormat="1" ht="49.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:33" s="33" customFormat="1" ht="49.75" customHeight="1" ns3:dyDescent="0.15">
       <c r="A45" s="53">
         <v>214.12100000000001</v>
       </c>
@@ -12096,7 +12096,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="46" spans="1:33" s="33" customFormat="1" ht="49.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:33" s="33" customFormat="1" ht="49.75" customHeight="1" ns3:dyDescent="0.15">
       <c r="A46" s="53">
         <v>214.12200000000001</v>
       </c>
@@ -12182,7 +12182,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="47" spans="1:33" s="33" customFormat="1" ht="74.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:33" s="33" customFormat="1" ht="74.75" customHeight="1" ns3:dyDescent="0.15">
       <c r="A47" s="53">
         <v>214.12299999999999</v>
       </c>
@@ -12268,7 +12268,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="48" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A48" s="53">
         <v>214.7</v>
       </c>
@@ -12313,7 +12313,7 @@
       <c r="AF48" s="76"/>
       <c r="AG48" s="74"/>
     </row>
-    <row r="49" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A49" s="53">
         <v>214.71</v>
       </c>
@@ -12365,7 +12365,7 @@
       <c r="AF49" s="76"/>
       <c r="AG49" s="74"/>
     </row>
-    <row r="50" spans="1:33" s="33" customFormat="1" ht="49.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:33" s="33" customFormat="1" ht="49.75" customHeight="1" ns3:dyDescent="0.15">
       <c r="A50" s="53">
         <v>214.71100000000001</v>
       </c>
@@ -12457,7 +12457,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="1:33" s="33" customFormat="1" ht="49.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:33" s="33" customFormat="1" ht="49.75" customHeight="1" ns3:dyDescent="0.15">
       <c r="A51" s="53">
         <v>214.71199999999999</v>
       </c>
@@ -12543,7 +12543,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="52" spans="1:33" s="33" customFormat="1" ht="74.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:33" s="33" customFormat="1" ht="74.75" customHeight="1" ns3:dyDescent="0.15">
       <c r="A52" s="53">
         <v>214.71299999999999</v>
       </c>
@@ -12629,7 +12629,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="53" spans="1:33" ht="185" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:33" ht="185" customHeight="1" ns3:dyDescent="0.2">
       <c r="A53" s="53">
         <v>214.72</v>
       </c>
@@ -12726,7 +12726,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="54" spans="1:33" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:33" ht="22.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A54" s="53">
         <v>214.8</v>
       </c>
@@ -12771,7 +12771,7 @@
       <c r="AF54" s="76"/>
       <c r="AG54" s="74"/>
     </row>
-    <row r="55" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A55" s="53">
         <v>214.81</v>
       </c>
@@ -12816,7 +12816,7 @@
       <c r="AF55" s="76"/>
       <c r="AG55" s="74"/>
     </row>
-    <row r="56" spans="1:33" ht="76.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:33" ht="76.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A56" s="53">
         <v>214.81100000000001</v>
       </c>
@@ -12910,7 +12910,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="57" spans="1:33" ht="76.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:33" ht="76.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A57" s="53">
         <v>214.81200000000001</v>
       </c>
@@ -12996,7 +12996,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="58" spans="1:33" ht="76.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:33" ht="76.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A58" s="53">
         <v>214.81299999999999</v>
       </c>
@@ -13082,7 +13082,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="59" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A59" s="53">
         <v>215</v>
       </c>
@@ -13127,7 +13127,7 @@
       <c r="AF59" s="76"/>
       <c r="AG59" s="74"/>
     </row>
-    <row r="60" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A60" s="53">
         <v>215.1</v>
       </c>
@@ -13172,7 +13172,7 @@
       <c r="AF60" s="76"/>
       <c r="AG60" s="74"/>
     </row>
-    <row r="61" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A61" s="53">
         <v>215.11</v>
       </c>
@@ -13264,7 +13264,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="62" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A62" s="53">
         <v>215.12</v>
       </c>
@@ -13350,7 +13350,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="63" spans="1:33" ht="76.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:33" ht="76.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A63" s="53">
         <v>215.13</v>
       </c>
@@ -13436,7 +13436,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="64" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A64" s="53">
         <v>215.4</v>
       </c>
@@ -13481,7 +13481,7 @@
       <c r="AF64" s="76"/>
       <c r="AG64" s="74"/>
     </row>
-    <row r="65" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A65" s="53">
         <v>215.41</v>
       </c>
@@ -13573,7 +13573,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="66" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A66" s="53">
         <v>215.42</v>
       </c>
@@ -13659,7 +13659,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="67" spans="1:33" ht="76.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:33" ht="76.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A67" s="53">
         <v>215.43</v>
       </c>
@@ -13745,7 +13745,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="68" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A68" s="37">
         <v>22</v>
       </c>
@@ -13790,7 +13790,7 @@
       <c r="AF68" s="76"/>
       <c r="AG68" s="74"/>
     </row>
-    <row r="69" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A69" s="53">
         <v>221</v>
       </c>
@@ -13835,7 +13835,7 @@
       <c r="AF69" s="76"/>
       <c r="AG69" s="74"/>
     </row>
-    <row r="70" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A70" s="53">
         <v>221.1</v>
       </c>
@@ -13880,7 +13880,7 @@
       <c r="AF70" s="76"/>
       <c r="AG70" s="74"/>
     </row>
-    <row r="71" spans="1:33" ht="112" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:33" ht="112" customHeight="1" ns3:dyDescent="0.2">
       <c r="A71" s="53">
         <v>221.11</v>
       </c>
@@ -13975,7 +13975,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="72" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A72" s="53">
         <v>221.12</v>
       </c>
@@ -14072,7 +14072,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="73" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A73" s="53">
         <v>221.12</v>
       </c>
@@ -14161,7 +14161,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="74" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A74" s="53">
         <v>221.12</v>
       </c>
@@ -14257,7 +14257,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="75" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A75" s="53">
         <v>221.13</v>
       </c>
@@ -14362,7 +14362,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="76" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A76" s="53">
         <v>221.13</v>
       </c>
@@ -14458,7 +14458,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="77" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A77" s="53">
         <v>221.13</v>
       </c>
@@ -14554,7 +14554,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="78" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A78" s="53">
         <v>221.2</v>
       </c>
@@ -14606,7 +14606,7 @@
       <c r="AF78" s="76"/>
       <c r="AG78" s="74"/>
     </row>
-    <row r="79" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A79" s="53">
         <v>221.21</v>
       </c>
@@ -14658,7 +14658,7 @@
       <c r="AF79" s="76"/>
       <c r="AG79" s="74"/>
     </row>
-    <row r="80" spans="1:33" s="33" customFormat="1" ht="74.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="80" spans="1:33" s="33" customFormat="1" ht="74.75" customHeight="1" ns3:dyDescent="0.15">
       <c r="A80" s="53">
         <v>221.21100000000001</v>
       </c>
@@ -14757,7 +14757,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="81" spans="1:36" s="33" customFormat="1" x14ac:dyDescent="0.15">
+    <row r="81" spans="1:36" s="33" customFormat="1" ns3:dyDescent="0.15">
       <c r="A81" s="53">
         <v>221.21199999999999</v>
       </c>
@@ -14850,7 +14850,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="82" spans="1:36" s="33" customFormat="1" ht="53.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="82" spans="1:36" s="33" customFormat="1" ht="53.25" customHeight="1" ns3:dyDescent="0.15">
       <c r="A82" s="53">
         <v>221.21299999999999</v>
       </c>
@@ -14954,7 +14954,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="83" spans="1:36" s="33" customFormat="1" ht="53.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="83" spans="1:36" s="33" customFormat="1" ht="53.25" customHeight="1" ns3:dyDescent="0.15">
       <c r="A83" s="53">
         <v>221.21299999999999</v>
       </c>
@@ -15050,7 +15050,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="84" spans="1:36" s="33" customFormat="1" ht="53.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="84" spans="1:36" s="33" customFormat="1" ht="53.25" customHeight="1" ns3:dyDescent="0.15">
       <c r="A84" s="53">
         <v>221.214</v>
       </c>
@@ -15154,7 +15154,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="85" spans="1:36" s="33" customFormat="1" ht="53.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="85" spans="1:36" s="33" customFormat="1" ht="53.25" customHeight="1" ns3:dyDescent="0.15">
       <c r="A85" s="53">
         <v>221.214</v>
       </c>
@@ -15259,7 +15259,7 @@
       </c>
       <c r="AJ85" s="36"/>
     </row>
-    <row r="86" spans="1:36" s="33" customFormat="1" ht="53.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="86" spans="1:36" s="33" customFormat="1" ht="53.25" customHeight="1" ns3:dyDescent="0.15">
       <c r="A86" s="53">
         <v>221.214</v>
       </c>
@@ -15357,7 +15357,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="87" spans="1:36" s="33" customFormat="1" ht="53.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="87" spans="1:36" s="33" customFormat="1" ht="53.25" customHeight="1" ns3:dyDescent="0.15">
       <c r="A87" s="53">
         <v>221.215</v>
       </c>
@@ -15453,7 +15453,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="88" spans="1:36" s="33" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:36" s="33" customFormat="1" ht="40" customHeight="1" ns3:dyDescent="0.2">
       <c r="A88" s="53">
         <v>221.21600000000001</v>
       </c>
@@ -15540,7 +15540,7 @@
       <c r="AF88" s="76"/>
       <c r="AG88" s="74"/>
     </row>
-    <row r="89" spans="1:36" s="33" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:36" s="33" customFormat="1" ht="40" customHeight="1" ns3:dyDescent="0.2">
       <c r="A89" s="53">
         <v>221.21600000000001</v>
       </c>
@@ -15627,7 +15627,7 @@
       <c r="AF89" s="76"/>
       <c r="AG89" s="74"/>
     </row>
-    <row r="90" spans="1:36" s="33" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:36" s="33" customFormat="1" ht="40" customHeight="1" ns3:dyDescent="0.2">
       <c r="A90" s="53">
         <v>221.21700000000001</v>
       </c>
@@ -15716,7 +15716,7 @@
       <c r="AF90" s="76"/>
       <c r="AG90" s="74"/>
     </row>
-    <row r="91" spans="1:36" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:36" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A91" s="53">
         <v>221.3</v>
       </c>
@@ -15770,7 +15770,7 @@
       <c r="AF91" s="76"/>
       <c r="AG91" s="74"/>
     </row>
-    <row r="92" spans="1:36" ht="25.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:36" ht="25.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A92" s="53">
         <v>221.31</v>
       </c>
@@ -15822,7 +15822,7 @@
       <c r="AF92" s="76"/>
       <c r="AG92" s="74"/>
     </row>
-    <row r="93" spans="1:36" ht="25.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:36" ht="25.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A93" s="53">
         <v>221.31100000000001</v>
       </c>
@@ -15933,7 +15933,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="94" spans="1:36" ht="25.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:36" ht="25.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A94" s="53">
         <v>221.31200000000001</v>
       </c>
@@ -16039,7 +16039,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="95" spans="1:36" ht="25.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:36" ht="25.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A95" s="53">
         <v>221.31100000000001</v>
       </c>
@@ -16138,7 +16138,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="96" spans="1:36" ht="25.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:36" ht="25.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A96" s="53">
         <v>221.31200000000001</v>
       </c>
@@ -16235,7 +16235,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="97" spans="1:33" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:33" ht="101.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A97" s="53">
         <v>221.31100000000001</v>
       </c>
@@ -16326,7 +16326,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="98" spans="1:33" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:33" ht="101.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A98" s="53">
         <v>221.31200000000001</v>
       </c>
@@ -16417,7 +16417,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="99" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A99" s="53">
         <v>221.31100000000001</v>
       </c>
@@ -16506,7 +16506,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="100" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A100" s="53">
         <v>221.31200000000001</v>
       </c>
@@ -16595,7 +16595,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="101" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A101" s="53">
         <v>221.32</v>
       </c>
@@ -16647,7 +16647,7 @@
       <c r="AF101" s="76"/>
       <c r="AG101" s="74"/>
     </row>
-    <row r="102" spans="1:33" s="33" customFormat="1" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:33" s="33" customFormat="1" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A102" s="53">
         <v>221.321</v>
       </c>
@@ -16754,7 +16754,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="103" spans="1:33" s="33" customFormat="1" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:33" s="33" customFormat="1" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A103" s="53">
         <v>221.322</v>
       </c>
@@ -16857,7 +16857,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="104" spans="1:33" ht="122.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:33" ht="122.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A104" s="85">
         <v>221.33</v>
       </c>
@@ -16944,7 +16944,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="105" spans="1:33" ht="122.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:33" ht="122.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A105" s="85">
         <v>221.33</v>
       </c>
@@ -17030,7 +17030,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="106" spans="1:33" ht="122.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:33" ht="122.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A106" s="85">
         <v>221.33</v>
       </c>
@@ -17117,7 +17117,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="107" spans="1:33" ht="122.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:33" ht="122.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A107" s="85">
         <v>221.33</v>
       </c>
@@ -17202,7 +17202,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="108" spans="1:33" ht="122.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:33" ht="122.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A108" s="85">
         <v>221.34</v>
       </c>
@@ -17289,7 +17289,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="109" spans="1:33" ht="122.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:33" ht="122.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A109" s="85">
         <v>221.34</v>
       </c>
@@ -17374,7 +17374,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="110" spans="1:33" ht="122.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:33" ht="122.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A110" s="85">
         <v>221.34</v>
       </c>
@@ -17463,7 +17463,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="111" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A111" s="53">
         <v>222</v>
       </c>
@@ -17515,7 +17515,7 @@
       <c r="AF111" s="76"/>
       <c r="AG111" s="74"/>
     </row>
-    <row r="112" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A112" s="53">
         <v>222.1</v>
       </c>
@@ -17567,7 +17567,7 @@
       <c r="AF112" s="76"/>
       <c r="AG112" s="74"/>
     </row>
-    <row r="113" spans="1:33" ht="109" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:33" ht="109" customHeight="1" ns3:dyDescent="0.2">
       <c r="A113" s="42">
         <v>222.11</v>
       </c>
@@ -17670,7 +17670,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="114" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A114" s="42">
         <v>222.12</v>
       </c>
@@ -17768,7 +17768,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="115" spans="1:33" ht="176" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:33" ht="176" customHeight="1" ns3:dyDescent="0.2">
       <c r="A115" s="42">
         <v>222.13</v>
       </c>
@@ -17866,7 +17866,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="116" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A116" s="53">
         <v>222.2</v>
       </c>
@@ -17964,7 +17964,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="117" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A117" s="53">
         <v>222.2</v>
       </c>
@@ -18062,7 +18062,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="118" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A118" s="53">
         <v>222.2</v>
       </c>
@@ -18162,7 +18162,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="119" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A119" s="53">
         <v>222.3</v>
       </c>
@@ -18214,7 +18214,7 @@
       <c r="AF119" s="76"/>
       <c r="AG119" s="74"/>
     </row>
-    <row r="120" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A120" s="53">
         <v>222.31</v>
       </c>
@@ -18314,7 +18314,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="121" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A121" s="53">
         <v>222.31</v>
       </c>
@@ -18414,7 +18414,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="122" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A122" s="53">
         <v>222.32</v>
       </c>
@@ -18514,7 +18514,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="123" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A123" s="53">
         <v>222.32</v>
       </c>
@@ -18614,7 +18614,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="124" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A124" s="53">
         <v>222.5</v>
       </c>
@@ -18718,7 +18718,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="125" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A125" s="53">
         <v>222.5</v>
       </c>
@@ -18806,7 +18806,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="126" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A126" s="53">
         <v>222.6</v>
       </c>
@@ -18862,7 +18862,7 @@
       <c r="AF126" s="76"/>
       <c r="AG126" s="74"/>
     </row>
-    <row r="127" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A127" s="53">
         <v>222.61</v>
       </c>
@@ -18957,7 +18957,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="128" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A128" s="53">
         <v>222.62</v>
       </c>
@@ -19055,7 +19055,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="129" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A129" s="53">
         <v>223</v>
       </c>
@@ -19100,7 +19100,7 @@
       <c r="AF129" s="76"/>
       <c r="AG129" s="74"/>
     </row>
-    <row r="130" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A130" s="53">
         <v>223.2</v>
       </c>
@@ -19145,7 +19145,7 @@
       <c r="AF130" s="76"/>
       <c r="AG130" s="74"/>
     </row>
-    <row r="131" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A131" s="53">
         <v>223.21</v>
       </c>
@@ -19233,7 +19233,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="132" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A132" s="53">
         <v>223.22</v>
       </c>
@@ -19321,7 +19321,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="133" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A133" s="53">
         <v>226</v>
       </c>
@@ -19407,7 +19407,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="134" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A134" s="53">
         <v>226</v>
       </c>
@@ -19508,7 +19508,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="135" spans="1:33" ht="76.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:33" ht="76.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A135" s="53">
         <v>227</v>
       </c>
@@ -19602,7 +19602,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="136" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A136" s="53">
         <v>228</v>
       </c>
@@ -19691,7 +19691,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="137" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A137" s="37">
         <v>23</v>
       </c>
@@ -19736,7 +19736,7 @@
       <c r="AF137" s="76"/>
       <c r="AG137" s="74"/>
     </row>
-    <row r="138" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A138" s="53">
         <v>232</v>
       </c>
@@ -19781,7 +19781,7 @@
       <c r="AF138" s="76"/>
       <c r="AG138" s="74"/>
     </row>
-    <row r="139" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A139" s="53">
         <v>232.1</v>
       </c>
@@ -19874,7 +19874,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="140" spans="1:33" ht="76.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:33" ht="76.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A140" s="53">
         <v>236</v>
       </c>
@@ -19943,7 +19943,7 @@
       <c r="AF140" s="76"/>
       <c r="AG140" s="74"/>
     </row>
-    <row r="141" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A141" s="37">
         <v>24</v>
       </c>
@@ -19988,7 +19988,7 @@
       <c r="AF141" s="76"/>
       <c r="AG141" s="74"/>
     </row>
-    <row r="142" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A142" s="37">
         <v>241</v>
       </c>
@@ -20080,7 +20080,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="143" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A143" s="37">
         <v>242</v>
       </c>
@@ -20168,7 +20168,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="144" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A144" s="37">
         <v>243</v>
       </c>
@@ -20256,7 +20256,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="145" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A145" s="37">
         <v>244</v>
       </c>
@@ -20344,7 +20344,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="146" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A146" s="37">
         <v>245</v>
       </c>
@@ -20432,7 +20432,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="147" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A147" s="37">
         <v>246</v>
       </c>
@@ -20520,7 +20520,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="148" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A148" s="37">
         <v>25</v>
       </c>
@@ -20565,7 +20565,7 @@
       <c r="AF148" s="76"/>
       <c r="AG148" s="74"/>
     </row>
-    <row r="149" spans="1:33" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:33" ht="29" customHeight="1" ns3:dyDescent="0.2">
       <c r="A149" s="53">
         <v>251</v>
       </c>
@@ -20652,7 +20652,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="150" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A150" s="53">
         <v>252</v>
       </c>
@@ -20735,7 +20735,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="151" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A151" s="53">
         <v>253</v>
       </c>
@@ -20820,7 +20820,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="152" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A152" s="53">
         <v>254</v>
       </c>
@@ -20911,7 +20911,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="153" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A153" s="53">
         <v>254</v>
       </c>
@@ -21009,7 +21009,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="154" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A154" s="53">
         <v>254</v>
       </c>
@@ -21103,7 +21103,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="155" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A155" s="37">
         <v>26</v>
       </c>
@@ -21193,7 +21193,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="156" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A156" s="50">
         <v>30</v>
       </c>
@@ -21245,7 +21245,7 @@
       <c r="AF156" s="76"/>
       <c r="AG156" s="74"/>
     </row>
-    <row r="157" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A157" s="50">
         <v>31</v>
       </c>
@@ -21289,7 +21289,7 @@
       <c r="AF157" s="76"/>
       <c r="AG157" s="74"/>
     </row>
-    <row r="158" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A158" s="50">
         <v>32</v>
       </c>
@@ -21333,7 +21333,7 @@
       <c r="AF158" s="76"/>
       <c r="AG158" s="74"/>
     </row>
-    <row r="159" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A159" s="37">
         <v>33</v>
       </c>
@@ -21422,7 +21422,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="160" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A160" s="37">
         <v>34</v>
       </c>
@@ -21502,7 +21502,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="161" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A161" s="37">
         <v>35</v>
       </c>
@@ -21582,7 +21582,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="162" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A162" s="37">
         <v>36</v>
       </c>
@@ -21662,7 +21662,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="163" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A163" s="37">
         <v>40</v>
       </c>
@@ -21707,7 +21707,7 @@
       <c r="AF163" s="76"/>
       <c r="AG163" s="74"/>
     </row>
-    <row r="164" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A164" s="37">
         <v>41</v>
       </c>
@@ -21790,7 +21790,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="165" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A165" s="50">
         <v>60</v>
       </c>
@@ -21835,7 +21835,7 @@
       <c r="AF165" s="76"/>
       <c r="AG165" s="74"/>
     </row>
-    <row r="166" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A166" s="37">
         <v>62</v>
       </c>
@@ -21880,7 +21880,7 @@
       <c r="AF166" s="76"/>
       <c r="AG166" s="74"/>
     </row>
-    <row r="167" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A167" s="37">
         <v>70</v>
       </c>
@@ -21925,7 +21925,7 @@
       <c r="AF167" s="76"/>
       <c r="AG167" s="74"/>
     </row>
-    <row r="168" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A168" s="37">
         <v>71</v>
       </c>
@@ -21970,7 +21970,7 @@
       <c r="AF168" s="76"/>
       <c r="AG168" s="74"/>
     </row>
-    <row r="169" spans="1:33" ht="126.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:33" ht="126.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A169" s="53">
         <v>711</v>
       </c>
@@ -22057,7 +22057,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="170" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A170" s="53">
         <v>712</v>
       </c>
@@ -22148,7 +22148,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="171" spans="1:33" ht="151" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:33" ht="151" customHeight="1" ns3:dyDescent="0.2">
       <c r="A171" s="53">
         <v>713</v>
       </c>
@@ -22235,7 +22235,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="172" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A172" s="37">
         <v>72</v>
       </c>
@@ -22280,7 +22280,7 @@
       <c r="AF172" s="76"/>
       <c r="AG172" s="74"/>
     </row>
-    <row r="173" spans="1:33" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:33" ht="101.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A173" s="37">
         <v>721</v>
       </c>
@@ -22377,7 +22377,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="174" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A174" s="37">
         <v>721</v>
       </c>
@@ -22477,7 +22477,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="175" spans="1:33" ht="275.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:33" ht="275.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A175" s="37">
         <v>73</v>
       </c>
@@ -22554,7 +22554,7 @@
       <c r="AF175" s="76"/>
       <c r="AG175" s="74"/>
     </row>
-    <row r="176" spans="1:33" ht="225.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:33" ht="225.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A176" s="37">
         <v>75</v>
       </c>
@@ -22605,7 +22605,7 @@
       <c r="AF176" s="76"/>
       <c r="AG176" s="74"/>
     </row>
-    <row r="177" spans="1:33" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:33" ht="22.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A177" s="37">
         <v>751</v>
       </c>
@@ -22656,7 +22656,7 @@
       <c r="AF177" s="76"/>
       <c r="AG177" s="74"/>
     </row>
-    <row r="178" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A178" s="37">
         <v>752</v>
       </c>
@@ -22701,7 +22701,7 @@
       <c r="AF178" s="76"/>
       <c r="AG178" s="74"/>
     </row>
-    <row r="179" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A179" s="37">
         <v>753</v>
       </c>
@@ -22746,7 +22746,7 @@
       <c r="AF179" s="76"/>
       <c r="AG179" s="74"/>
     </row>
-    <row r="180" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A180" s="37">
         <v>754</v>
       </c>
@@ -22791,7 +22791,7 @@
       <c r="AF180" s="76"/>
       <c r="AG180" s="74"/>
     </row>
-    <row r="181" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A181" s="37">
         <v>755</v>
       </c>
@@ -22836,20 +22836,22 @@
       <c r="AF181" s="76"/>
       <c r="AG181" s="74"/>
     </row>
-    <row r="182" spans="1:33" ht="45.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:33" ht="45.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A182" s="37">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="B182" s="38">
-        <f t="shared" si="52"/>
         <v>2</v>
       </c>
-      <c r="C182" s="55" t="s">
-        <v>410</v>
-      </c>
-      <c r="D182" s="39" t="str">
-        <f t="shared" si="51"/>
-        <v xml:space="preserve">            Annualized Moderator Booster Replacements</v>
+      <c r="C182" s="55" t="inlineStr">
+        <is>
+          <t>Annualized Integrated Heat Transfer Vessel Replacements</t>
+        </is>
+      </c>
+      <c r="D182" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            Annualized Integrated Heat Transfer Vessel Replacements</t>
+        </is>
       </c>
       <c r="E182" s="39"/>
       <c r="F182" s="39"/>
@@ -22881,20 +22883,20 @@
       <c r="AF182" s="76"/>
       <c r="AG182" s="74"/>
     </row>
-    <row r="183" spans="1:33" ht="45.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:33" ht="45.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A183" s="37">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="B183" s="38">
         <f t="shared" si="52"/>
         <v>2</v>
       </c>
       <c r="C183" s="55" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="D183" s="39" t="str">
         <f t="shared" si="51"/>
-        <v xml:space="preserve">            Annualized Plant Maintenance (Misc.)</v>
+        <v xml:space="preserve">            Annualized Moderator Booster Replacements</v>
       </c>
       <c r="E183" s="39"/>
       <c r="F183" s="39"/>
@@ -22910,10 +22912,10 @@
       <c r="P183" s="49"/>
       <c r="Q183" s="65"/>
       <c r="R183" s="49"/>
-      <c r="S183" s="205"/>
-      <c r="T183" s="205"/>
+      <c r="S183" s="204"/>
+      <c r="T183" s="204"/>
       <c r="U183" s="49"/>
-      <c r="V183" s="205"/>
+      <c r="V183" s="204"/>
       <c r="W183" s="74"/>
       <c r="X183" s="77"/>
       <c r="Y183" s="77"/>
@@ -22926,20 +22928,20 @@
       <c r="AF183" s="76"/>
       <c r="AG183" s="74"/>
     </row>
-    <row r="184" spans="1:33" ht="56" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:33" ht="45.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A184" s="37">
-        <v>759.1</v>
+        <v>759</v>
       </c>
       <c r="B184" s="38">
-        <f t="shared" ref="B184:B191" si="53">IF(ISNUMBER(A184),IF(AND(A184=INT(A184),MOD(A184,10)=0),0,IF(AND(A184=INT(A184),LEN(A184)=2),1,IF(AND(A184=INT(A184),LEN(A184)=3),2,LEN(A184)-FIND(".",A184)+2))),"")</f>
-        <v>3</v>
+        <f t="shared" si="52"/>
+        <v>2</v>
       </c>
       <c r="C184" s="55" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="D184" s="39" t="str">
-        <f t="shared" ref="D184:D191" si="54">REPT("   ",B184*2)&amp;C184</f>
-        <v xml:space="preserve">                  Annualized Building and Structural Maintenance (Accounts 212–215)</v>
+        <f t="shared" si="51"/>
+        <v xml:space="preserve">            Annualized Plant Maintenance (Misc.)</v>
       </c>
       <c r="E184" s="39"/>
       <c r="F184" s="39"/>
@@ -22971,20 +22973,20 @@
       <c r="AF184" s="76"/>
       <c r="AG184" s="74"/>
     </row>
-    <row r="185" spans="1:33" ht="56" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:33" ht="56" customHeight="1" ns3:dyDescent="0.2">
       <c r="A185" s="37">
-        <v>759.2</v>
+        <v>759.1</v>
       </c>
       <c r="B185" s="38">
-        <f t="shared" si="53"/>
+        <f t="shared" ref="B184:B191" si="53">IF(ISNUMBER(A185),IF(AND(A185=INT(A185),MOD(A185,10)=0),0,IF(AND(A185=INT(A185),LEN(A185)=2),1,IF(AND(A185=INT(A185),LEN(A185)=3),2,LEN(A185)-FIND(".",A185)+2))),"")</f>
         <v>3</v>
       </c>
       <c r="C185" s="55" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="D185" s="39" t="str">
-        <f t="shared" si="54"/>
-        <v xml:space="preserve">                  Annualized Main Heat Transport System Maintenance (Accounts 222.1–222.3 and 222.6)</v>
+        <f t="shared" ref="D184:D191" si="54">REPT("   ",B185*2)&amp;C185</f>
+        <v xml:space="preserve">                  Annualized Building and Structural Maintenance (Accounts 212–215)</v>
       </c>
       <c r="E185" s="39"/>
       <c r="F185" s="39"/>
@@ -23016,20 +23018,20 @@
       <c r="AF185" s="76"/>
       <c r="AG185" s="74"/>
     </row>
-    <row r="186" spans="1:33" ht="56" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:33" ht="56" customHeight="1" ns3:dyDescent="0.2">
       <c r="A186" s="37">
-        <v>759.3</v>
+        <v>759.2</v>
       </c>
       <c r="B186" s="38">
         <f t="shared" si="53"/>
         <v>3</v>
       </c>
       <c r="C186" s="55" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D186" s="39" t="str">
         <f t="shared" si="54"/>
-        <v xml:space="preserve">                  Annualized Safety System Maintenance (Account 223)</v>
+        <v xml:space="preserve">                  Annualized Main Heat Transport System Maintenance (Accounts 222.1–222.3 and 222.6)</v>
       </c>
       <c r="E186" s="39"/>
       <c r="F186" s="39"/>
@@ -23061,20 +23063,20 @@
       <c r="AF186" s="76"/>
       <c r="AG186" s="74"/>
     </row>
-    <row r="187" spans="1:33" ht="56" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:33" ht="56" customHeight="1" ns3:dyDescent="0.2">
       <c r="A187" s="37">
-        <v>759.4</v>
+        <v>759.3</v>
       </c>
       <c r="B187" s="38">
         <f t="shared" si="53"/>
         <v>3</v>
       </c>
       <c r="C187" s="55" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D187" s="39" t="str">
         <f t="shared" si="54"/>
-        <v xml:space="preserve">                  Annualized Reactor Plant Equipment Maintenance (Accounts 221.11, 226, and 228)</v>
+        <v xml:space="preserve">                  Annualized Safety System Maintenance (Account 223)</v>
       </c>
       <c r="E187" s="39"/>
       <c r="F187" s="39"/>
@@ -23106,20 +23108,20 @@
       <c r="AF187" s="76"/>
       <c r="AG187" s="74"/>
     </row>
-    <row r="188" spans="1:33" ht="56" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:33" ht="56" customHeight="1" ns3:dyDescent="0.2">
       <c r="A188" s="37">
-        <v>759.5</v>
+        <v>759.4</v>
       </c>
       <c r="B188" s="38">
         <f t="shared" si="53"/>
         <v>3</v>
       </c>
       <c r="C188" s="55" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D188" s="39" t="str">
         <f t="shared" si="54"/>
-        <v xml:space="preserve">                  Annualized Reactor I&amp;C Maintenance (Account 227)</v>
+        <v xml:space="preserve">                  Annualized Reactor Plant Equipment Maintenance (Accounts 221.11, 226, and 228)</v>
       </c>
       <c r="E188" s="39"/>
       <c r="F188" s="39"/>
@@ -23151,20 +23153,20 @@
       <c r="AF188" s="76"/>
       <c r="AG188" s="74"/>
     </row>
-    <row r="189" spans="1:33" ht="56" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:33" ht="56" customHeight="1" ns3:dyDescent="0.2">
       <c r="A189" s="37">
-        <v>759.6</v>
+        <v>759.5</v>
       </c>
       <c r="B189" s="38">
         <f t="shared" si="53"/>
         <v>3</v>
       </c>
       <c r="C189" s="55" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D189" s="39" t="str">
         <f t="shared" si="54"/>
-        <v xml:space="preserve">                  Annualized Energy Conversion System Maintenance (Account 23)</v>
+        <v xml:space="preserve">                  Annualized Reactor I&amp;C Maintenance (Account 227)</v>
       </c>
       <c r="E189" s="39"/>
       <c r="F189" s="39"/>
@@ -23196,20 +23198,20 @@
       <c r="AF189" s="76"/>
       <c r="AG189" s="74"/>
     </row>
-    <row r="190" spans="1:33" ht="56" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:33" ht="56" customHeight="1" ns3:dyDescent="0.2">
       <c r="A190" s="37">
-        <v>759.7</v>
+        <v>759.6</v>
       </c>
       <c r="B190" s="38">
         <f t="shared" si="53"/>
         <v>3</v>
       </c>
       <c r="C190" s="55" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D190" s="39" t="str">
         <f t="shared" si="54"/>
-        <v xml:space="preserve">                  Annualized Electrical Equipment Maintenance (Account 24)</v>
+        <v xml:space="preserve">                  Annualized Energy Conversion System Maintenance (Account 23)</v>
       </c>
       <c r="E190" s="39"/>
       <c r="F190" s="39"/>
@@ -23241,20 +23243,20 @@
       <c r="AF190" s="76"/>
       <c r="AG190" s="74"/>
     </row>
-    <row r="191" spans="1:33" ht="56" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:33" ht="56" customHeight="1" ns3:dyDescent="0.2">
       <c r="A191" s="37">
-        <v>759.8</v>
+        <v>759.7</v>
       </c>
       <c r="B191" s="38">
         <f t="shared" si="53"/>
         <v>3</v>
       </c>
       <c r="C191" s="55" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="D191" s="39" t="str">
         <f t="shared" si="54"/>
-        <v xml:space="preserve">                  Annualized Miscellaneous Equipment Maintenance (Account 26)</v>
+        <v xml:space="preserve">                  Annualized Electrical Equipment Maintenance (Account 24)</v>
       </c>
       <c r="E191" s="39"/>
       <c r="F191" s="39"/>
@@ -23286,27 +23288,20 @@
       <c r="AF191" s="76"/>
       <c r="AG191" s="74"/>
     </row>
-    <row r="192" spans="1:33" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:33" ht="56" customHeight="1" ns3:dyDescent="0.2">
       <c r="A192" s="37">
-        <v>78</v>
+        <v>759.8</v>
       </c>
       <c r="B192" s="38">
-        <f>IF(ISNUMBER(A192),
-    IF(AND(A192=INT(A192), MOD(A192, 10) = 0), 0,
-        IF(AND(A192=INT(A192), LEN(A192)=2), 1,
-            IF(AND(A192=INT(A192), LEN(A192)=3), 2,
-                LEN(A192) - FIND(".", A192) + 2)
-        )
-    ),
-"")</f>
-        <v>1</v>
+        <f t="shared" si="53"/>
+        <v>3</v>
       </c>
       <c r="C192" s="55" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D192" s="39" t="str">
-        <f t="shared" si="51"/>
-        <v xml:space="preserve">      Annualized Decommissioning Cost</v>
+        <f t="shared" si="54"/>
+        <v xml:space="preserve">                  Annualized Miscellaneous Equipment Maintenance (Account 26)</v>
       </c>
       <c r="E192" s="39"/>
       <c r="F192" s="39"/>
@@ -23314,20 +23309,18 @@
       <c r="H192" s="39"/>
       <c r="I192" s="39"/>
       <c r="J192" s="43"/>
-      <c r="K192" s="70"/>
+      <c r="K192" s="60"/>
       <c r="L192" s="49"/>
-      <c r="M192" s="45"/>
+      <c r="M192" s="58"/>
       <c r="N192" s="49"/>
       <c r="O192" s="49"/>
       <c r="P192" s="49"/>
       <c r="Q192" s="65"/>
       <c r="R192" s="49"/>
-      <c r="S192" s="58"/>
-      <c r="T192" s="58"/>
+      <c r="S192" s="205"/>
+      <c r="T192" s="205"/>
       <c r="U192" s="49"/>
-      <c r="V192" s="58" t="s">
-        <v>421</v>
-      </c>
+      <c r="V192" s="205"/>
       <c r="W192" s="74"/>
       <c r="X192" s="77"/>
       <c r="Y192" s="77"/>
@@ -23340,46 +23333,48 @@
       <c r="AF192" s="76"/>
       <c r="AG192" s="74"/>
     </row>
-    <row r="193" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:33" ht="53.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A193" s="37">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B193" s="38">
         <f>IF(ISNUMBER(A193),
-IF(AND(A193=INT(A193), MOD(A193, 10) = 0), 0,
-IF(AND(A193=INT(A193), LEN(A193)=2), 1,
-IF(AND(A193=INT(A193), LEN(A193)=3), 2,
-LEN(A193) - FIND(".", A193) + 2)
-)
-),
+    IF(AND(A193=INT(A193), MOD(A193, 10) = 0), 0,
+        IF(AND(A193=INT(A193), LEN(A193)=2), 1,
+            IF(AND(A193=INT(A193), LEN(A193)=3), 2,
+                LEN(A193) - FIND(".", A193) + 2)
+        )
+    ),
 "")</f>
-        <v>0</v>
-      </c>
-      <c r="C193" s="69" t="s">
-        <v>422</v>
+        <v>1</v>
+      </c>
+      <c r="C193" s="55" t="s">
+        <v>420</v>
       </c>
       <c r="D193" s="39" t="str">
         <f t="shared" si="51"/>
-        <v>Annualized Fuel Cost</v>
+        <v xml:space="preserve">      Annualized Decommissioning Cost</v>
       </c>
       <c r="E193" s="39"/>
       <c r="F193" s="39"/>
       <c r="G193" s="39"/>
       <c r="H193" s="39"/>
       <c r="I193" s="39"/>
-      <c r="J193" s="40"/>
-      <c r="K193" s="40"/>
-      <c r="L193" s="38"/>
-      <c r="M193" s="41"/>
-      <c r="N193" s="38"/>
-      <c r="O193" s="38"/>
-      <c r="P193" s="38"/>
-      <c r="Q193" s="40"/>
-      <c r="R193" s="38"/>
-      <c r="S193" s="41"/>
-      <c r="T193" s="38"/>
-      <c r="U193" s="38"/>
-      <c r="V193" s="38"/>
+      <c r="J193" s="43"/>
+      <c r="K193" s="70"/>
+      <c r="L193" s="49"/>
+      <c r="M193" s="45"/>
+      <c r="N193" s="49"/>
+      <c r="O193" s="49"/>
+      <c r="P193" s="49"/>
+      <c r="Q193" s="65"/>
+      <c r="R193" s="49"/>
+      <c r="S193" s="58"/>
+      <c r="T193" s="58"/>
+      <c r="U193" s="49"/>
+      <c r="V193" s="58" t="s">
+        <v>421</v>
+      </c>
       <c r="W193" s="74"/>
       <c r="X193" s="77"/>
       <c r="Y193" s="77"/>
@@ -23392,9 +23387,9 @@
       <c r="AF193" s="76"/>
       <c r="AG193" s="74"/>
     </row>
-    <row r="194" spans="1:33" ht="151" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A194" s="37">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B194" s="38">
         <f>IF(ISNUMBER(A194),
@@ -23405,90 +23400,48 @@
 )
 ),
 "")</f>
-        <v>1</v>
-      </c>
-      <c r="C194" s="55" t="s">
-        <v>423</v>
+        <v>0</v>
+      </c>
+      <c r="C194" s="69" t="s">
+        <v>422</v>
       </c>
       <c r="D194" s="39" t="str">
         <f t="shared" si="51"/>
-        <v xml:space="preserve">      Refueling Operations</v>
-      </c>
-      <c r="E194" s="39" t="s">
-        <v>268</v>
-      </c>
+        <v>Annualized Fuel Cost</v>
+      </c>
+      <c r="E194" s="39"/>
       <c r="F194" s="39"/>
       <c r="G194" s="39"/>
       <c r="H194" s="39"/>
       <c r="I194" s="39"/>
-      <c r="J194" s="43"/>
-      <c r="K194" s="60">
-        <v>178500</v>
-      </c>
-      <c r="L194" s="49" t="s">
-        <v>386</v>
-      </c>
-      <c r="M194" s="58" t="s">
-        <v>387</v>
-      </c>
-      <c r="N194" s="49"/>
-      <c r="O194" s="49"/>
-      <c r="P194" s="49">
-        <v>1</v>
-      </c>
-      <c r="Q194" s="65">
-        <v>2024</v>
-      </c>
-      <c r="R194" s="49" t="s">
-        <v>53</v>
-      </c>
-      <c r="S194" s="58"/>
-      <c r="T194" s="58" t="s">
-        <v>388</v>
-      </c>
-      <c r="U194" s="49"/>
-      <c r="V194" s="49"/>
-      <c r="W194" s="74" t="s">
-        <v>43</v>
-      </c>
-      <c r="X194" s="77">
-        <f>0.9*$J194</f>
-        <v>0</v>
-      </c>
-      <c r="Y194" s="77">
-        <f>1.5*J194</f>
-        <v>0</v>
-      </c>
-      <c r="Z194" s="74" t="s">
-        <v>44</v>
-      </c>
-      <c r="AA194" s="76">
-        <f>0.9*K194</f>
-        <v>160650</v>
-      </c>
-      <c r="AB194" s="76">
-        <f>1.3*K194</f>
-        <v>232050</v>
-      </c>
-      <c r="AC194" s="74" t="s">
-        <v>44</v>
-      </c>
-      <c r="AD194" s="76" t="s">
-        <v>45</v>
-      </c>
-      <c r="AE194" s="76" t="s">
-        <v>46</v>
-      </c>
-      <c r="AF194" s="76" t="s">
-        <v>47</v>
-      </c>
-      <c r="AG194" s="74" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="195" spans="1:33" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J194" s="40"/>
+      <c r="K194" s="40"/>
+      <c r="L194" s="38"/>
+      <c r="M194" s="41"/>
+      <c r="N194" s="38"/>
+      <c r="O194" s="38"/>
+      <c r="P194" s="38"/>
+      <c r="Q194" s="40"/>
+      <c r="R194" s="38"/>
+      <c r="S194" s="41"/>
+      <c r="T194" s="38"/>
+      <c r="U194" s="38"/>
+      <c r="V194" s="38"/>
+      <c r="W194" s="74"/>
+      <c r="X194" s="77"/>
+      <c r="Y194" s="77"/>
+      <c r="Z194" s="74"/>
+      <c r="AA194" s="76"/>
+      <c r="AB194" s="76"/>
+      <c r="AC194" s="74"/>
+      <c r="AD194" s="76"/>
+      <c r="AE194" s="76"/>
+      <c r="AF194" s="76"/>
+      <c r="AG194" s="74"/>
+    </row>
+    <row r="195" spans="1:33" ht="151" customHeight="1" ns3:dyDescent="0.2">
       <c r="A195" s="37">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B195" s="38">
         <f>IF(ISNUMBER(A195),
@@ -23502,45 +23455,87 @@
         <v>1</v>
       </c>
       <c r="C195" s="55" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D195" s="39" t="str">
         <f t="shared" si="51"/>
-        <v xml:space="preserve">      Additional Nuclear Fuel</v>
-      </c>
-      <c r="E195" s="39"/>
+        <v xml:space="preserve">      Refueling Operations</v>
+      </c>
+      <c r="E195" s="39" t="s">
+        <v>268</v>
+      </c>
       <c r="F195" s="39"/>
       <c r="G195" s="39"/>
       <c r="H195" s="39"/>
       <c r="I195" s="39"/>
       <c r="J195" s="43"/>
-      <c r="K195" s="60"/>
-      <c r="L195" s="49"/>
-      <c r="M195" s="58"/>
+      <c r="K195" s="60">
+        <v>178500</v>
+      </c>
+      <c r="L195" s="49" t="s">
+        <v>386</v>
+      </c>
+      <c r="M195" s="58" t="s">
+        <v>387</v>
+      </c>
       <c r="N195" s="49"/>
       <c r="O195" s="49"/>
-      <c r="P195" s="49"/>
-      <c r="Q195" s="65"/>
-      <c r="R195" s="49"/>
+      <c r="P195" s="49">
+        <v>1</v>
+      </c>
+      <c r="Q195" s="65">
+        <v>2024</v>
+      </c>
+      <c r="R195" s="49" t="s">
+        <v>53</v>
+      </c>
       <c r="S195" s="58"/>
-      <c r="T195" s="49"/>
+      <c r="T195" s="58" t="s">
+        <v>388</v>
+      </c>
       <c r="U195" s="49"/>
       <c r="V195" s="49"/>
-      <c r="W195" s="74"/>
-      <c r="X195" s="77"/>
-      <c r="Y195" s="77"/>
-      <c r="Z195" s="74"/>
-      <c r="AA195" s="76"/>
-      <c r="AB195" s="76"/>
-      <c r="AC195" s="74"/>
-      <c r="AD195" s="76"/>
-      <c r="AE195" s="76"/>
-      <c r="AF195" s="76"/>
-      <c r="AG195" s="74"/>
-    </row>
-    <row r="196" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W195" s="74" t="s">
+        <v>43</v>
+      </c>
+      <c r="X195" s="77">
+        <f>0.9*$J195</f>
+        <v>0</v>
+      </c>
+      <c r="Y195" s="77">
+        <f>1.5*J195</f>
+        <v>0</v>
+      </c>
+      <c r="Z195" s="74" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA195" s="76">
+        <f>0.9*K195</f>
+        <v>160650</v>
+      </c>
+      <c r="AB195" s="76">
+        <f>1.3*K195</f>
+        <v>232050</v>
+      </c>
+      <c r="AC195" s="74" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD195" s="76" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE195" s="76" t="s">
+        <v>46</v>
+      </c>
+      <c r="AF195" s="76" t="s">
+        <v>47</v>
+      </c>
+      <c r="AG195" s="74" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="196" spans="1:33" ht="26.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A196" s="37">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B196" s="38">
         <f>IF(ISNUMBER(A196),
@@ -23554,79 +23549,131 @@
         <v>1</v>
       </c>
       <c r="C196" s="55" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D196" s="39" t="str">
         <f t="shared" si="51"/>
-        <v xml:space="preserve">      Spent Fuel Management</v>
-      </c>
-      <c r="E196" s="39" t="s">
-        <v>35</v>
-      </c>
+        <v xml:space="preserve">      Additional Nuclear Fuel</v>
+      </c>
+      <c r="E196" s="39"/>
       <c r="F196" s="39"/>
       <c r="G196" s="39"/>
       <c r="H196" s="39"/>
       <c r="I196" s="39"/>
       <c r="J196" s="43"/>
-      <c r="K196" s="60">
-        <v>1</v>
-      </c>
-      <c r="L196" s="49" t="s">
-        <v>426</v>
-      </c>
-      <c r="M196" s="58" t="s">
-        <v>427</v>
-      </c>
+      <c r="K196" s="60"/>
+      <c r="L196" s="49"/>
+      <c r="M196" s="58"/>
       <c r="N196" s="49"/>
       <c r="O196" s="49"/>
-      <c r="P196" s="49">
-        <v>1</v>
-      </c>
-      <c r="Q196" s="65">
-        <v>2024</v>
-      </c>
-      <c r="R196" s="49" t="s">
-        <v>86</v>
-      </c>
+      <c r="P196" s="49"/>
+      <c r="Q196" s="65"/>
+      <c r="R196" s="49"/>
       <c r="S196" s="58"/>
       <c r="T196" s="49"/>
       <c r="U196" s="49"/>
       <c r="V196" s="49"/>
-      <c r="W196" s="74" t="s">
+      <c r="W196" s="74"/>
+      <c r="X196" s="77"/>
+      <c r="Y196" s="77"/>
+      <c r="Z196" s="74"/>
+      <c r="AA196" s="76"/>
+      <c r="AB196" s="76"/>
+      <c r="AC196" s="74"/>
+      <c r="AD196" s="76"/>
+      <c r="AE196" s="76"/>
+      <c r="AF196" s="76"/>
+      <c r="AG196" s="74"/>
+    </row>
+    <row r="197" spans="1:33" ht="51.75" customHeight="1" ns3:dyDescent="0.2">
+      <c r="A197" s="37">
+        <v>83</v>
+      </c>
+      <c r="B197" s="38">
+        <f>IF(ISNUMBER(A197),
+IF(AND(A197=INT(A197), MOD(A197, 10) = 0), 0,
+IF(AND(A197=INT(A197), LEN(A197)=2), 1,
+IF(AND(A197=INT(A197), LEN(A197)=3), 2,
+LEN(A197) - FIND(".", A197) + 2)
+)
+),
+"")</f>
+        <v>1</v>
+      </c>
+      <c r="C197" s="55" t="s">
+        <v>425</v>
+      </c>
+      <c r="D197" s="39" t="str">
+        <f t="shared" si="51"/>
+        <v xml:space="preserve">      Spent Fuel Management</v>
+      </c>
+      <c r="E197" s="39" t="s">
+        <v>35</v>
+      </c>
+      <c r="F197" s="39"/>
+      <c r="G197" s="39"/>
+      <c r="H197" s="39"/>
+      <c r="I197" s="39"/>
+      <c r="J197" s="43"/>
+      <c r="K197" s="60">
+        <v>1</v>
+      </c>
+      <c r="L197" s="49" t="s">
+        <v>426</v>
+      </c>
+      <c r="M197" s="58" t="s">
+        <v>427</v>
+      </c>
+      <c r="N197" s="49"/>
+      <c r="O197" s="49"/>
+      <c r="P197" s="49">
+        <v>1</v>
+      </c>
+      <c r="Q197" s="65">
+        <v>2024</v>
+      </c>
+      <c r="R197" s="49" t="s">
+        <v>86</v>
+      </c>
+      <c r="S197" s="58"/>
+      <c r="T197" s="49"/>
+      <c r="U197" s="49"/>
+      <c r="V197" s="49"/>
+      <c r="W197" s="74" t="s">
         <v>43</v>
       </c>
-      <c r="X196" s="77">
-        <f>0.9*$J196</f>
-        <v>0</v>
-      </c>
-      <c r="Y196" s="77">
-        <f>1.5*J196</f>
-        <v>0</v>
-      </c>
-      <c r="Z196" s="74" t="s">
-        <v>44</v>
-      </c>
-      <c r="AA196" s="76">
-        <f>0.9*K196</f>
+      <c r="X197" s="77">
+        <f>0.9*$J197</f>
+        <v>0</v>
+      </c>
+      <c r="Y197" s="77">
+        <f>1.5*J197</f>
+        <v>0</v>
+      </c>
+      <c r="Z197" s="74" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA197" s="76">
+        <f>0.9*K197</f>
         <v>0.9</v>
       </c>
-      <c r="AB196" s="76">
-        <f>1.3*K196</f>
+      <c r="AB197" s="76">
+        <f>1.3*K197</f>
         <v>1.3</v>
       </c>
-      <c r="AC196" s="74" t="s">
-        <v>44</v>
-      </c>
-      <c r="AD196" s="76" t="s">
+      <c r="AC197" s="74" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD197" s="76" t="s">
         <v>45</v>
       </c>
-      <c r="AE196" s="76" t="s">
+      <c r="AE197" s="76" t="s">
         <v>46</v>
       </c>
-      <c r="AF196" s="76" t="s">
+      <c r="AF197" s="76" t="s">
         <v>47</v>
       </c>
-      <c r="AG196" s="74" t="s">
+      <c r="AG197" s="74" t="s">
         <v>48</v>
       </c>
     </row>
@@ -24950,76 +24997,76 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="17">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q194:R201 Q155:Q201 Q2:Q153" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q194:R201 Q155:Q201 Q2:Q153" ns2:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>1950</formula1>
       <formula2>2025</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J134:J135 J138:J145 J149:J193 K2:K9 K56:K58 K61:K63 K65:K67 K71:K83 K88 K98:K108 K110:K151 K153:K193 N109:N1048576 N75:N87 N89:N107 N1:N71 J2:J131 K11:K52" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J134:J135 J138:J145 J149:J193 K2:K9 K56:K58 K61:K63 K65:K67 K71:K83 K88 K98:K108 K110:K151 K153:K193 N109:N1048576 N75:N87 N89:N107 N1:N71 J2:J131 K11:K52" ns2:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M360:M370" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M360:M370" ns2:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Land Area, Power MWe, Excavation Volume,  Reactor Building Slab Roof Volume,	Reactor Building  Basement Volume, Reactor Building  Exterior Walls Volume,		Turbine Building Slab Roof Volume,	Turbine Building  Basement Volume,	Turbine Building  Exterior Wall"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1 L194:L1048576" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1 L194:L1048576" ns2:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"$/acres, $/MWe, $/m^3, $/MWt"</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P194:P339" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P194:P339" ns2:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>0</formula1>
       <formula2>2</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P145:P201 P86:P138 P2:P84" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P145:P201 P86:P138 P2:P84" ns2:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>0</formula1>
       <formula2>2</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O145:O201 O86:O135 O138 O2:O13 O18:O84 O15" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O145:O201 O86:O135 O138 O2:O13 O18:O84 O15" ns2:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"acres, MWe, m^3, MWt, Kg, Drums, kW, $, m^2, kg/s"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L145:L201 L86:L114 L116:L138 L2:L13 L18:L84 L15" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L145:L201 L86:L114 L116:L138 L2:L13 L18:L84 L15" ns2:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"$/m^2,$/MWeHour,$/FTE, $/acres, $/MWe, $/m^3, $/MWt, $/Kg, $/Drum, $/(kg.sec), $/SWU, unitless, $/kWe"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O136:O137" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O136:O137" ns2:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"acres, MWe, m^3, MWt, Kg, Drums, kW, $, m^2, kg/s, kWe"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L85 L139:L144" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L85 L139:L144" ns2:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"$/MWeHour,$/FTE, $/acres, $/MWe, $/m^3, $/MWt, $/Kg, $/Drum, $/(kg.sec), $/SWU, unitless"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O85 O139:O144" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O85 O139:O144" ns2:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"acres, MWe, m^3, MWt, Kg, Drums, kW, $"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P85 P139:P144" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P85 P139:P144" ns2:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E201" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E201" ns2:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"standard, nonstandard"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R2:R201" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R2:R201" ns2:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"NA, General, Labor, Material, Equipment,Lab and Mat and Equip, 'Lab and Equip"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L115" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L115" ns2:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"$/heatpipe,$/m^2,$/MWeHour,$/FTE, $/acres, $/MWe, $/m^3, $/MWt, $/Kg, $/Drum, $/(kg.sec), $/SWU, unitless, $/kWe"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O16:O17 O14" xr:uid="{404860D7-E1E0-6A4B-A6BA-FCD332FF61FE}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O16:O17 O14" ns2:uid="{404860D7-E1E0-6A4B-A6BA-FCD332FF61FE}">
       <formula1>"m,acres, MWe, m^3, MWt, Kg, Drums, kW, $, m^2, kg/s"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L16:L17 L14" xr:uid="{F79DC16A-CFBC-5E4B-AA4C-06A7E72D0753}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L16:L17 L14" ns2:uid="{F79DC16A-CFBC-5E4B-AA4C-06A7E72D0753}">
       <formula1>"$/m,$/m^2,$/MWeHour,$/FTE, $/acres, $/MWe, $/m^3, $/MWt, $/Kg, $/Drum, $/(kg.sec), $/SWU, unitless, $/kWe"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="U3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="U5" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="U22" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="U23" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="U37" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="U53" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="U113" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="U124" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="U134" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="U135" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="U139" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="U140" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="U173" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="U3" ns4:id="rId1" ns2:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="U5" ns4:id="rId2" ns2:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="U22" ns4:id="rId3" ns2:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="U23" ns4:id="rId4" ns2:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="U37" ns4:id="rId5" ns2:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="U53" ns4:id="rId6" ns2:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="U113" ns4:id="rId7" ns2:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="U124" ns4:id="rId8" ns2:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="U134" ns4:id="rId9" ns2:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="U135" ns4:id="rId10" ns2:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="U139" ns4:id="rId11" ns2:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="U140" ns4:id="rId12" ns2:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="U173" ns4:id="rId13" ns2:uid="{00000000-0004-0000-0000-00000C000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Set licensing learning rate in cost database
</commit_message>
<xml_diff>
--- a/cost/Cost_Database.xlsx
+++ b/cost/Cost_Database.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Database" sheetId="1" r:id="Ra6ad543c9d44473d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MARVEL_Cost" sheetId="2" r:id="R6ed59536b00e4688"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Variables" sheetId="3" r:id="R28656b16e27a4f7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inflation Adjustment" sheetId="4" r:id="Rc2102c44b4df4727"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economics Parameters" sheetId="5" r:id="Re9d62dbb14f04944"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Central Facility Database" sheetId="6" r:id="R7ba09e4ef963496c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Database" sheetId="1" r:id="R8cc44493ef054a9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MARVEL_Cost" sheetId="2" r:id="Re4aa994d4c6e4113"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Variables" sheetId="3" r:id="R35fa29f8c23f47a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inflation Adjustment" sheetId="4" r:id="R2599c6bc273d4be8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economics Parameters" sheetId="5" r:id="Rd77e61a29aa64e13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Central Facility Database" sheetId="6" r:id="Rbc74ca9b80be4fad"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="CRF">#REF!</x:definedName>
@@ -23987,18 +23987,18 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R0281d7ce810e4451"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="R82b232edbd624732"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="Reb6f65dd0e1a47d8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U33" r:id="Ra4002a568e124ac2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U49" r:id="R7524d5683ae44095"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U109" r:id="R78622f477640423d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U120" r:id="R1ad73cd1835e4784"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U130" r:id="R15f7cc3e99024840"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U131" r:id="R453a2e4fd8a54c20"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U135" r:id="R69e2a49543e5492c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U136" r:id="R91a2632a9a404bdd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U169" r:id="Re400fd8edc2e403f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R64a7bc95d2b244be"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="Rbea2ed0682ad42c8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="R8bd514e035814680"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U33" r:id="R73f75fcec6b64441"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U49" r:id="R4d545bf921944e39"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U109" r:id="Recffc00ba694489e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U120" r:id="R5fd6063ac96a46ef"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U130" r:id="R6efd8303c6174cea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U131" r:id="Rc54f9c7a66614c55"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U135" r:id="R59f7d1cdc1e04726"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U136" r:id="R24533926a3b443e3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U169" r:id="Racff3a829c8a4959"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -27301,7 +27301,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a13f44cb7ee40fe"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R610ab24701144f01"/>
 </x:worksheet>
 </file>
 
@@ -27454,7 +27454,7 @@
         </x:is>
       </x:c>
       <x:c r="B11" t="n">
-        <x:v>0</x:v>
+        <x:v>0.2</x:v>
       </x:c>
     </x:row>
     <x:row r="12">

</xml_diff>